<commit_message>
Docs: reconcile L3 with 675 budget and 1325 cash; sample floor warning
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UFhYQrmawc4QNd7RjXn8ny
</commit_message>
<xml_diff>
--- a/docs/operacao/modelo-caixa-anuncios.xlsx
+++ b/docs/operacao/modelo-caixa-anuncios.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="411">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="415">
   <si>
     <t xml:space="preserve">Resumo — caixa necessário para o teste de anúncios</t>
   </si>
@@ -122,6 +122,18 @@
   </si>
   <si>
     <t xml:space="preserve">o que o cartão realmente cobra pela verba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leads no teste</t>
+  </si>
+  <si>
+    <t xml:space="preserve">verba ÷ CPL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Piso de amostra (mais de 500 leads e 50 pedidos)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L3 item 4, assinado em 02/10</t>
   </si>
   <si>
     <t xml:space="preserve">Gasto antecipado e tempo até virar caixa — por caminho</t>
@@ -1802,7 +1814,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="62"/>
@@ -1999,243 +2011,267 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="11" t="s">
+      <c r="A19" s="2" t="s">
         <v>32</v>
       </c>
+      <c r="B19" s="5" t="n">
+        <f aca="false">B5/Premissas!$B$18</f>
+        <v>450</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B20" s="3" t="s">
+      <c r="A20" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="B20" s="6" t="str">
+        <f aca="false">IF(AND(B19&gt;500,B6&gt;50),"passa","abaixo do piso")</f>
+        <v>abaixo do piso</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D20" s="3" t="s">
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="11" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D23" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B21" s="12" t="n">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B24" s="12" t="n">
         <f aca="false">(Premissas!$B$18*(1+Premissas!$B$17)+Premissas!$B$20)/Premissas!$B$19+Premissas!$B$21</f>
         <v>19.8145</v>
       </c>
-      <c r="C21" s="12" t="n">
+      <c r="C24" s="12" t="n">
         <f aca="false">(Premissas!$B$18*(1+Premissas!$B$17)+Premissas!$B$20)/Premissas!$B$19+Premissas!$B$21</f>
         <v>19.8145</v>
       </c>
-      <c r="D21" s="2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B22" s="12" t="n">
+      <c r="D24" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B25" s="12" t="n">
         <f aca="false">Premissas!$B$59*Unitário!$B$22</f>
         <v>30</v>
       </c>
-      <c r="C22" s="12" t="n">
+      <c r="C25" s="12" t="n">
         <f aca="false">Premissas!$B$59*Unitário!$B$22</f>
         <v>30</v>
       </c>
-      <c r="D22" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="B23" s="12" t="n">
+      <c r="D25" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B26" s="12" t="n">
         <f aca="false">Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25</f>
         <v>36.56001</v>
       </c>
-      <c r="C23" s="12" t="n">
+      <c r="C26" s="12" t="n">
         <f aca="false">Premissas!$B$31</f>
         <v>5</v>
       </c>
-      <c r="D23" s="2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="B24" s="12" t="n">
+      <c r="D26" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B27" s="12" t="n">
         <f aca="false">-Premissas!$B$26*(Premissas!$B$59*Unitário!$B$22+Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25)-Premissas!$B$27*(Premissas!$B$59*Unitário!$B$22+(1-Premissas!$B$62)*(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25))+Premissas!$B$26*Premissas!$B$39+Premissas!$B$27*Premissas!$B$41</f>
         <v>-7.6169017</v>
       </c>
-      <c r="C24" s="12" t="n">
+      <c r="C27" s="12" t="n">
         <f aca="false">-Premissas!$B$27*(Premissas!$B$59*Unitário!$B$22+(1-Premissas!$B$62)*Premissas!$B$31)+Premissas!$B$27*Premissas!$B$41</f>
         <v>2</v>
       </c>
-      <c r="D24" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="13" t="s">
-        <v>44</v>
-      </c>
-      <c r="B25" s="14" t="n">
-        <f aca="false">SUM(B22:B24)</f>
+      <c r="D27" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="B28" s="14" t="n">
+        <f aca="false">SUM(B25:B27)</f>
         <v>58.9431083</v>
       </c>
-      <c r="C25" s="14" t="n">
-        <f aca="false">SUM(C22:C24)</f>
+      <c r="C28" s="14" t="n">
+        <f aca="false">SUM(C25:C27)</f>
         <v>37</v>
       </c>
-      <c r="D25" s="2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="B26" s="15" t="n">
+      <c r="D28" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29" s="15" t="n">
         <f aca="false">Premissas!$B$54+Premissas!$B$55</f>
         <v>16</v>
       </c>
-      <c r="C26" s="15" t="n">
+      <c r="C29" s="15" t="n">
         <f aca="false">Premissas!$B$56</f>
         <v>0</v>
       </c>
-      <c r="D26" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B27" s="12" t="n">
+      <c r="D29" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30" s="12" t="n">
         <f aca="false">Unitário!$B$21*Premissas!$B$51</f>
         <v>94.827</v>
       </c>
-      <c r="C27" s="12" t="n">
+      <c r="C30" s="12" t="n">
         <f aca="false">(1-Premissas!$B$27)*Premissas!$B$52</f>
         <v>105.219</v>
       </c>
-      <c r="D27" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="11" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C31" s="3" t="s">
+      <c r="D30" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="D31" s="3" t="s">
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="11" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="B32" s="17" t="n">
-        <f aca="false">A32*B5</f>
-        <v>675</v>
-      </c>
-      <c r="C32" s="17" t="n">
-        <f aca="false">A32*B9</f>
-        <v>879.4672187</v>
-      </c>
-      <c r="D32" s="17" t="n">
-        <f aca="false">$B$13-C32</f>
-        <v>195.5327813</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="16" t="n">
-        <v>2</v>
-      </c>
-      <c r="B33" s="17" t="n">
-        <f aca="false">A33*B5</f>
-        <v>1350</v>
-      </c>
-      <c r="C33" s="17" t="n">
-        <f aca="false">A33*B9</f>
-        <v>1758.9344374</v>
-      </c>
-      <c r="D33" s="17" t="n">
-        <f aca="false">$B$13-C33</f>
-        <v>-683.9344374</v>
-      </c>
-    </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="16" t="n">
-        <v>3</v>
-      </c>
-      <c r="B34" s="17" t="n">
-        <f aca="false">A34*B5</f>
-        <v>2025</v>
-      </c>
-      <c r="C34" s="17" t="n">
-        <f aca="false">A34*B9</f>
-        <v>2638.4016561</v>
-      </c>
-      <c r="D34" s="17" t="n">
-        <f aca="false">$B$13-C34</f>
-        <v>-1563.4016561</v>
+      <c r="A34" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="B35" s="17" t="n">
         <f aca="false">A35*B5</f>
-        <v>3375</v>
+        <v>675</v>
       </c>
       <c r="C35" s="17" t="n">
         <f aca="false">A35*B9</f>
-        <v>4397.3360935</v>
+        <v>879.4672187</v>
       </c>
       <c r="D35" s="17" t="n">
         <f aca="false">$B$13-C35</f>
-        <v>-3322.3360935</v>
+        <v>195.5327813</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="16" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="B36" s="17" t="n">
         <f aca="false">A36*B5</f>
-        <v>6750</v>
+        <v>1350</v>
       </c>
       <c r="C36" s="17" t="n">
         <f aca="false">A36*B9</f>
-        <v>8794.672187</v>
+        <v>1758.9344374</v>
       </c>
       <c r="D36" s="17" t="n">
         <f aca="false">$B$13-C36</f>
+        <v>-683.9344374</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="B37" s="17" t="n">
+        <f aca="false">A37*B5</f>
+        <v>2025</v>
+      </c>
+      <c r="C37" s="17" t="n">
+        <f aca="false">A37*B9</f>
+        <v>2638.4016561</v>
+      </c>
+      <c r="D37" s="17" t="n">
+        <f aca="false">$B$13-C37</f>
+        <v>-1563.4016561</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="B38" s="17" t="n">
+        <f aca="false">A38*B5</f>
+        <v>3375</v>
+      </c>
+      <c r="C38" s="17" t="n">
+        <f aca="false">A38*B9</f>
+        <v>4397.3360935</v>
+      </c>
+      <c r="D38" s="17" t="n">
+        <f aca="false">$B$13-C38</f>
+        <v>-3322.3360935</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="B39" s="17" t="n">
+        <f aca="false">A39*B5</f>
+        <v>6750</v>
+      </c>
+      <c r="C39" s="17" t="n">
+        <f aca="false">A39*B9</f>
+        <v>8794.672187</v>
+      </c>
+      <c r="D39" s="17" t="n">
+        <f aca="false">$B$13-C39</f>
         <v>-7719.672187</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="2" t="s">
-        <v>55</v>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="2" t="s">
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -2264,31 +2300,31 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>3</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B5" s="19"/>
       <c r="C5" s="19"/>
@@ -2296,231 +2332,231 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="B6" s="20" t="n">
         <v>375</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B7" s="21" t="n">
         <v>5</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B8" s="21" t="n">
         <v>2</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B9" s="20" t="n">
         <v>300</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="B10" s="21" t="n">
         <v>5</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B11" s="22" t="n">
         <v>46318</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B12" s="23" t="n">
         <v>22</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B13" s="24" t="n">
         <v>100</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B14" s="24" t="n">
         <v>20</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="B15" s="21" t="n">
         <v>2</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="B16" s="21" t="n">
         <v>29</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B17" s="25" t="n">
         <v>0.1383</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B18" s="24" t="n">
         <v>1.5</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B19" s="26" t="n">
         <v>0.1</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="B20" s="24" t="n">
         <v>0.27</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B21" s="24" t="n">
         <v>0.04</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="18" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="B22" s="19"/>
       <c r="C22" s="19"/>
@@ -2528,34 +2564,34 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B23" s="26" t="n">
         <v>0.7</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B24" s="27" t="n">
         <f aca="false">1-Premissas!$B$23</f>
         <v>0.3</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="D24" s="2"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="18" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B25" s="19"/>
       <c r="C25" s="19"/>
@@ -2563,35 +2599,35 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B26" s="26" t="n">
         <v>0.17</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B27" s="26" t="n">
         <v>0.1</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="18" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="B28" s="19"/>
       <c r="C28" s="19"/>
@@ -2599,219 +2635,219 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B29" s="24" t="n">
         <v>30</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="B30" s="24" t="n">
         <v>19.99</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="B31" s="24" t="n">
         <v>5</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B32" s="28" t="n">
         <v>0.0699</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="B33" s="24" t="n">
         <v>2.49</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B34" s="28" t="n">
         <v>0.0099</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="B35" s="24" t="n">
         <v>1</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B36" s="28" t="n">
         <v>0.0498</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="B37" s="26" t="n">
         <v>0.5</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B38" s="24" t="n">
         <v>4.99</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B39" s="12" t="n">
         <f aca="false">Premissas!$B$38+Premissas!$B$31</f>
         <v>9.99</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="B40" s="20" t="n">
         <v>45</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="B41" s="12" t="n">
         <f aca="false">Premissas!$B$40+Premissas!$B$31</f>
         <v>50</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="B42" s="26" t="n">
         <v>0</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B43" s="24" t="n">
         <v>53.5</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="18" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B44" s="19"/>
       <c r="C44" s="19"/>
@@ -2819,21 +2855,21 @@
     </row>
     <row r="45" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="3" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="B46" s="24" t="n">
         <v>129.9</v>
@@ -2847,7 +2883,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="B47" s="24" t="n">
         <v>233.82</v>
@@ -2861,7 +2897,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B48" s="24" t="n">
         <v>311.76</v>
@@ -2875,7 +2911,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="2" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="D49" s="27" t="n">
         <f aca="false">SUM(D46:D48)</f>
@@ -2884,46 +2920,46 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="2" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="B50" s="29" t="n">
         <f aca="false">1*D46+2*D47+3*D48</f>
         <v>1</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="D50" s="2"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="2" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="B51" s="12" t="n">
         <f aca="false">SUMPRODUCT(B46:B48,D46:D48)</f>
         <v>129.9</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D51" s="2"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="2" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="B52" s="12" t="n">
         <f aca="false">SUMPRODUCT(C46:C48,D46:D48)</f>
         <v>116.91</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D52" s="2"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="18" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="B53" s="19"/>
       <c r="C53" s="19"/>
@@ -2931,63 +2967,63 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="2" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="B54" s="23" t="n">
         <v>2</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="2" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="B55" s="21" t="n">
         <v>14</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="B56" s="21" t="n">
         <v>0</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="2" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="B57" s="23" t="n">
         <v>7</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="18" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="B58" s="19"/>
       <c r="C58" s="19"/>
@@ -2995,77 +3031,77 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="2" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="B59" s="21" t="n">
         <v>1</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="2" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="B60" s="23" t="n">
         <v>1</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="2" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="B61" s="21" t="n">
         <v>1</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="2" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="B62" s="21" t="n">
         <v>1</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="2" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="B63" s="21" t="n">
         <v>1</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="18" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="B64" s="19"/>
       <c r="C64" s="19"/>
@@ -3073,58 +3109,58 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="2" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="B65" s="24" t="n">
         <v>1325</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="2" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="B66" s="24" t="n">
         <v>250</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="2" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="B67" s="24" t="n">
         <v>3.99</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="2" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="B68" s="21" t="n">
         <v>1</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
     </row>
   </sheetData>
@@ -3153,26 +3189,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="B4" s="12" t="n">
         <f aca="false">Premissas!$B$51</f>
@@ -3186,7 +3222,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="B5" s="12" t="n">
         <f aca="false">-Premissas!$B$29*Premissas!$B$50</f>
@@ -3197,12 +3233,12 @@
         <v>-30</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="B6" s="12" t="n">
         <f aca="false">-(Premissas!$B$32*Premissas!$B$51+Premissas!$B$33)</f>
@@ -3216,7 +3252,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="B7" s="12" t="n">
         <f aca="false">-Premissas!$B$30</f>
@@ -3227,12 +3263,12 @@
         <v>0</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="B8" s="12" t="n">
         <f aca="false">-Premissas!$B$31</f>
@@ -3246,7 +3282,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="B9" s="14" t="n">
         <f aca="false">SUM(B4:B8)</f>
@@ -3260,7 +3296,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="B10" s="12" t="n">
         <f aca="false">-Premissas!$B$26*(B9+Premissas!$B$39)</f>
@@ -3271,12 +3307,12 @@
         <v>0</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="B11" s="12" t="n">
         <f aca="false">-Premissas!$B$27*(B9+Premissas!$B$41+Premissas!$B$62*(Premissas!$B$30+Premissas!$B$31+Premissas!$B$32*Premissas!$B$51+Premissas!$B$33))</f>
@@ -3287,12 +3323,12 @@
         <v>-13.691</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="B12" s="14" t="n">
         <f aca="false">SUM(B9:B11)</f>
@@ -3306,7 +3342,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="B13" s="12" t="n">
         <f aca="false">-Premissas!$B$18*(1+Premissas!$B$17)/Premissas!$B$19</f>
@@ -3317,12 +3353,12 @@
         <v>-17.0745</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="B14" s="12" t="n">
         <f aca="false">-Premissas!$B$20/Premissas!$B$19</f>
@@ -3336,7 +3372,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="B15" s="12" t="n">
         <f aca="false">-Premissas!$B$21</f>
@@ -3350,7 +3386,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="B16" s="12" t="n">
         <f aca="false">-Premissas!$B$42*Premissas!$B$51*(1-Premissas!$B$26-Premissas!$B$27)</f>
@@ -3364,7 +3400,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="B17" s="14" t="n">
         <f aca="false">SUM(B12:B16)</f>
@@ -3378,7 +3414,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="B18" s="14" t="n">
         <f aca="false">Premissas!$B$23*B17+Premissas!$B$24*C17</f>
@@ -3387,12 +3423,12 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="B21" s="27" t="n">
         <f aca="false">1-Premissas!$B$26-Premissas!$B$27</f>
@@ -3401,7 +3437,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="B22" s="12" t="n">
         <f aca="false">Premissas!$B$29*Premissas!$B$50</f>
@@ -3410,7 +3446,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="B23" s="12" t="n">
         <f aca="false">-(B6+B7+B8)</f>
@@ -3419,7 +3455,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="B24" s="12" t="n">
         <f aca="false">-(B7+B8)</f>
@@ -3428,7 +3464,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="B25" s="12" t="n">
         <f aca="false">-B6</f>
@@ -3437,7 +3473,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="B26" s="12" t="n">
         <f aca="false">Unitário!$B$21*Unitário!$B$23+Premissas!$B$26*Premissas!$B$39+Premissas!$B$27*Premissas!$B$41</f>
@@ -3446,7 +3482,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="B27" s="12" t="n">
         <f aca="false">-C6</f>
@@ -3478,98 +3514,98 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="P4" s="3" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="Q4" s="3" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="R4" s="3" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="S4" s="3" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="T4" s="3" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="U4" s="3" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="V4" s="3" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="W4" s="3" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="X4" s="3" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="Y4" s="3" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="Z4" s="3" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="AA4" s="3" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="AB4" s="3" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13744,7 +13780,7 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="13" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="C95" s="14" t="n">
         <f aca="false">SUM(C5:C94)</f>
@@ -13809,7 +13845,7 @@
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="13" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="B99" s="14" t="n">
         <f aca="false">MIN(S5:S94)</f>
@@ -13818,7 +13854,7 @@
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="13" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="B100" s="32" t="n">
         <f aca="false">INDEX(A5:A94,MATCH(B99,S5:S94,0))</f>
@@ -13827,7 +13863,7 @@
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="13" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="B101" s="32" t="n">
         <f aca="false">IFERROR(INDEX(A5:A94,MATCH(1,T5:T94,0)),"não volta em 90 dias")</f>
@@ -13871,24 +13907,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13896,13 +13932,13 @@
         <v>1</v>
       </c>
       <c r="B4" s="33" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="C4" s="33" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="D4" s="33" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="E4" s="34"/>
     </row>
@@ -13911,13 +13947,13 @@
         <v>2</v>
       </c>
       <c r="B5" s="33" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="C5" s="33" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="D5" s="33" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="E5" s="34"/>
     </row>
@@ -13926,13 +13962,13 @@
         <v>3</v>
       </c>
       <c r="B6" s="33" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="C6" s="33" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="D6" s="33" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="E6" s="34"/>
     </row>
@@ -13941,13 +13977,13 @@
         <v>4</v>
       </c>
       <c r="B7" s="33" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="D7" s="33" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="E7" s="34"/>
     </row>
@@ -13979,296 +14015,296 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="33" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="B4" s="33" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="C4" s="33" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="D4" s="33" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="E4" s="33" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="33" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="B5" s="33" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="C5" s="33" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="D5" s="33" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="E5" s="33" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="33" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="B6" s="33" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="C6" s="33" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="D6" s="33" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="33" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="B7" s="33" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="D7" s="33" t="s">
+        <v>291</v>
+      </c>
+      <c r="E7" s="33" t="s">
         <v>287</v>
-      </c>
-      <c r="E7" s="33" t="s">
-        <v>283</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="33" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="B8" s="33" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="C8" s="33" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="D8" s="33" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="E8" s="33" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="33" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="B9" s="33" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="C9" s="33" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="D9" s="33" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="E9" s="33" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="33" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="B10" s="33" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="C10" s="33" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="D10" s="33" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="E10" s="33" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="33" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="B11" s="33" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="C11" s="33" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="D11" s="33" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="E11" s="33" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="33" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
       <c r="B12" s="33" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="C12" s="33" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="D12" s="33" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="E12" s="33" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="33" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="B13" s="33" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="D13" s="33" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="E13" s="33" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="33" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="B14" s="33" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="C14" s="33" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
       <c r="D14" s="33" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
       <c r="E14" s="33" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="33" t="s">
-        <v>320</v>
+        <v>324</v>
       </c>
       <c r="B15" s="33" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="C15" s="33" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
       <c r="D15" s="33" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="E15" s="33" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="33" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="B16" s="33" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="C16" s="33" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="D16" s="33" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="E16" s="33" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="33" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="B17" s="33" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="C17" s="33" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
       <c r="D17" s="33" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="E17" s="33" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="33" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="B18" s="33" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="C18" s="33" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
       <c r="D18" s="33" t="s">
-        <v>334</v>
+        <v>338</v>
       </c>
       <c r="E18" s="33" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="33" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="B19" s="33" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="D19" s="33" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="E19" s="33" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
     </row>
   </sheetData>
@@ -14301,469 +14337,469 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="33" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="B5" s="33" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="C5" s="35" t="n">
         <f aca="false">Premissas!$B$29*Premissas!$B$50</f>
         <v>30</v>
       </c>
       <c r="D5" s="33" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="E5" s="33" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
       <c r="F5" s="33" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
       <c r="G5" s="33" t="s">
-        <v>351</v>
+        <v>355</v>
       </c>
       <c r="H5" s="33" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="33" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="B6" s="33" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="C6" s="35" t="n">
         <f aca="false">Premissas!$B$30</f>
         <v>19.99</v>
       </c>
       <c r="D6" s="33" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
       <c r="F6" s="33" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="G6" s="33" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="H6" s="33" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="33" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="B7" s="33" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C7" s="35" t="n">
         <f aca="false">Premissas!$B$31</f>
         <v>5</v>
       </c>
       <c r="D7" s="33" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
       <c r="F7" s="33" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="G7" s="33" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="H7" s="33" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="33" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="B8" s="33" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
       <c r="C8" s="35" t="n">
         <f aca="false">Unitário!$B$25</f>
         <v>11.57001</v>
       </c>
       <c r="D8" s="33" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="E8" s="33" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="F8" s="33" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="G8" s="33" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="H8" s="33" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="33" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="B9" s="33" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="C9" s="35" t="n">
         <f aca="false">Premissas!$B$38</f>
         <v>4.99</v>
       </c>
       <c r="D9" s="33" t="s">
-        <v>366</v>
+        <v>370</v>
       </c>
       <c r="E9" s="33" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="F9" s="33" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="G9" s="33" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="H9" s="33" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="33" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="B10" s="33" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="C10" s="35" t="n">
         <f aca="false">Premissas!$B$39</f>
         <v>9.99</v>
       </c>
       <c r="D10" s="33" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="E10" s="33" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="F10" s="33" t="s">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="G10" s="33" t="s">
-        <v>371</v>
+        <v>375</v>
       </c>
       <c r="H10" s="33" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="33" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="B11" s="33" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="C11" s="35" t="n">
         <f aca="false">Premissas!$B$41+Premissas!$B$62*(Unitário!$B$24+Unitário!$B$25)</f>
         <v>86.56001</v>
       </c>
       <c r="D11" s="33" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
       <c r="E11" s="33" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="F11" s="33" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
       <c r="G11" s="33" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
       <c r="H11" s="33" t="s">
-        <v>377</v>
+        <v>381</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="33" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="B12" s="33" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="C12" s="35" t="n">
         <f aca="false">Premissas!$B$29*Premissas!$B$50</f>
         <v>30</v>
       </c>
       <c r="D12" s="33" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="E12" s="33" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
       <c r="F12" s="33" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
       <c r="G12" s="33" t="s">
-        <v>378</v>
+        <v>382</v>
       </c>
       <c r="H12" s="33" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="33" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="B13" s="33" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="C13" s="35" t="n">
         <f aca="false">Premissas!$B$41+Premissas!$B$62*Premissas!$B$31+Unitário!$B$27</f>
         <v>58.9897635</v>
       </c>
       <c r="D13" s="33" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
       <c r="E13" s="33" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="F13" s="33" t="s">
-        <v>379</v>
+        <v>383</v>
       </c>
       <c r="G13" s="33" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
       <c r="H13" s="33" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="33" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="B14" s="33" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C14" s="35" t="n">
         <f aca="false">Premissas!$B$31</f>
         <v>5</v>
       </c>
       <c r="D14" s="33" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="E14" s="33" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
       <c r="F14" s="33" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="G14" s="33" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="H14" s="33" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="33" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="B15" s="33" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
       <c r="C15" s="35" t="n">
         <f aca="false">Unitário!$B$27</f>
         <v>3.9897635</v>
       </c>
       <c r="D15" s="33" t="s">
-        <v>382</v>
+        <v>386</v>
       </c>
       <c r="E15" s="33" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="F15" s="33" t="s">
-        <v>384</v>
+        <v>388</v>
       </c>
       <c r="G15" s="33" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="H15" s="33" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="33" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="B16" s="33" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="C16" s="35" t="n">
         <v>0</v>
       </c>
       <c r="D16" s="33" t="s">
-        <v>387</v>
+        <v>391</v>
       </c>
       <c r="E16" s="33" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="F16" s="33" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="G16" s="33" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="H16" s="33" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="33" t="s">
-        <v>390</v>
+        <v>394</v>
       </c>
       <c r="B17" s="33" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
       <c r="C17" s="35" t="n">
         <f aca="false">Premissas!$B$18/Premissas!$B$19*(1+Premissas!$B$17)</f>
         <v>17.0745</v>
       </c>
       <c r="D17" s="33" t="s">
-        <v>392</v>
+        <v>396</v>
       </c>
       <c r="E17" s="33" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="F17" s="33" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="G17" s="33" t="s">
-        <v>395</v>
+        <v>399</v>
       </c>
       <c r="H17" s="33" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="33" t="s">
-        <v>390</v>
+        <v>394</v>
       </c>
       <c r="B18" s="33" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="C18" s="35" t="n">
         <f aca="false">Premissas!$B$20/Premissas!$B$19+Premissas!$B$21</f>
         <v>2.74</v>
       </c>
       <c r="D18" s="33" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="E18" s="33" t="s">
-        <v>398</v>
+        <v>402</v>
       </c>
       <c r="F18" s="33" t="s">
+        <v>403</v>
+      </c>
+      <c r="G18" s="33" t="s">
         <v>399</v>
       </c>
-      <c r="G18" s="33" t="s">
-        <v>395</v>
-      </c>
       <c r="H18" s="33" t="s">
-        <v>400</v>
+        <v>404</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="33" t="s">
-        <v>401</v>
+        <v>405</v>
       </c>
       <c r="B19" s="33" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
       <c r="C19" s="35" t="n">
         <f aca="false">Premissas!$B$43</f>
         <v>53.5</v>
       </c>
       <c r="D19" s="33" t="s">
-        <v>403</v>
+        <v>407</v>
       </c>
       <c r="E19" s="33" t="s">
-        <v>398</v>
+        <v>402</v>
       </c>
       <c r="F19" s="33" t="s">
-        <v>404</v>
+        <v>408</v>
       </c>
       <c r="G19" s="33" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="H19" s="33" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="33" t="s">
-        <v>405</v>
+        <v>409</v>
       </c>
       <c r="B20" s="33" t="s">
-        <v>406</v>
+        <v>410</v>
       </c>
       <c r="C20" s="35" t="n">
         <f aca="false">Premissas!$B$67*Premissas!$B$68</f>
         <v>3.99</v>
       </c>
       <c r="D20" s="33" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
       <c r="E20" s="33" t="s">
-        <v>408</v>
+        <v>412</v>
       </c>
       <c r="F20" s="33" t="s">
-        <v>409</v>
+        <v>413</v>
       </c>
       <c r="G20" s="33" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="H20" s="33" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cash model and docs: 7-day tests at R$ 50/day per phase (R$ 700), peak R$ 752, below sample floor at CPL 1.50
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UFhYQrmawc4QNd7RjXn8ny
</commit_message>
<xml_diff>
--- a/docs/operacao/modelo-caixa-anuncios.xlsx
+++ b/docs/operacao/modelo-caixa-anuncios.xlsx
@@ -232,7 +232,7 @@
     <t xml:space="preserve">R$</t>
   </si>
   <si>
-    <t xml:space="preserve">Operador, 09/10: 7 dias a R$ 55/dia (plano escolhido; antes R$ 375 em 5 dias)</t>
+    <t xml:space="preserve">Operador, 09/10: 7 dias a R$ 50/dia (antes R$ 55/dia; antes ainda R$ 375 em 5 dias)</t>
   </si>
   <si>
     <t xml:space="preserve">Fase 1 — dias</t>
@@ -253,7 +253,7 @@
     <t xml:space="preserve">Fase 2 — verba total</t>
   </si>
   <si>
-    <t xml:space="preserve">Operador, 09/10: 7 dias a R$ 55/dia (plano escolhido; antes R$ 300 em 5 dias)</t>
+    <t xml:space="preserve">Operador, 09/10: 7 dias a R$ 50/dia (antes R$ 55/dia; antes ainda R$ 300 em 5 dias)</t>
   </si>
   <si>
     <t xml:space="preserve">Fase 2 — dias</t>
@@ -565,7 +565,7 @@
     <t xml:space="preserve">Caixa disponível</t>
   </si>
   <si>
-    <t xml:space="preserve">Operador, 09/10 (dos R$ 2.000 investidos; a verba de R$ 770 vai no cartão e é paga com o repasse do COD, não com este caixa)</t>
+    <t xml:space="preserve">Operador, 09/10 (dos R$ 2.000 investidos; a verba de R$ 700 vai no cartão e é paga com o repasse do COD, não com este caixa)</t>
   </si>
   <si>
     <t xml:space="preserve">Margem de segurança</t>
@@ -1853,7 +1853,7 @@
       </c>
       <c r="B5" s="4" t="n">
         <f aca="false">'Fluxo diário'!C95</f>
-        <v>770</v>
+        <v>700</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>6</v>
@@ -1865,7 +1865,7 @@
       </c>
       <c r="B6" s="5" t="n">
         <f aca="false">'Fluxo diário'!G95+'Fluxo diário'!H95</f>
-        <v>51.3333333333333</v>
+        <v>46.6666666666667</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>8</v>
@@ -1877,7 +1877,7 @@
       </c>
       <c r="B7" s="6" t="str">
         <f aca="false">TEXT('Fluxo diário'!G95,"0.0")&amp;" / "&amp;TEXT('Fluxo diário'!H95,"0.0")</f>
-        <v>35.9 / 15.4</v>
+        <v>32.7 / 14.0</v>
       </c>
       <c r="C7" s="2"/>
     </row>
@@ -1887,7 +1887,7 @@
       </c>
       <c r="B8" s="4" t="n">
         <f aca="false">'Fluxo diário'!G95*Premissas!$B$51+'Fluxo diário'!H95*Premissas!$B$52</f>
-        <v>6468.154</v>
+        <v>5880.14</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>11</v>
@@ -1899,7 +1899,7 @@
       </c>
       <c r="B9" s="8" t="n">
         <f aca="false">-'Fluxo diário'!B99</f>
-        <v>827.567485873333</v>
+        <v>752.334078066667</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>13</v>
@@ -1935,7 +1935,7 @@
       </c>
       <c r="B12" s="4" t="n">
         <f aca="false">-'Fluxo diário'!B102</f>
-        <v>1704.05848587333</v>
+        <v>1549.14407806667</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>19</v>
@@ -1959,7 +1959,7 @@
       </c>
       <c r="B14" s="8" t="n">
         <f aca="false">B13-B9</f>
-        <v>247.432514126667</v>
+        <v>322.665921933333</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>23</v>
@@ -1971,7 +1971,7 @@
       </c>
       <c r="B15" s="4" t="n">
         <f aca="false">'Fluxo diário'!S94</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>25</v>
@@ -1995,7 +1995,7 @@
       </c>
       <c r="B17" s="10" t="n">
         <f aca="false">IFERROR(B13/B9,0)</f>
-        <v>1.29898771804157</v>
+        <v>1.42888648984573</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>29</v>
@@ -2007,7 +2007,7 @@
       </c>
       <c r="B18" s="4" t="n">
         <f aca="false">B5*(1+Premissas!$B$17)</f>
-        <v>876.491</v>
+        <v>796.81</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>31</v>
@@ -2019,7 +2019,7 @@
       </c>
       <c r="B19" s="5" t="n">
         <f aca="false">B5/Premissas!$B$18</f>
-        <v>513.333333333333</v>
+        <v>466.666666666667</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>33</v>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="B20" s="6" t="str">
         <f aca="false">IF(AND(B19&gt;500,B6&gt;50),"passa","abaixo do piso")</f>
-        <v>passa</v>
+        <v>abaixo do piso</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>35</v>
@@ -2193,15 +2193,15 @@
       </c>
       <c r="B35" s="17" t="n">
         <f aca="false">A35*B5</f>
-        <v>770</v>
+        <v>700</v>
       </c>
       <c r="C35" s="17" t="n">
         <f aca="false">A35*B9</f>
-        <v>827.567485873333</v>
+        <v>752.334078066667</v>
       </c>
       <c r="D35" s="17" t="n">
         <f aca="false">$B$13-C35</f>
-        <v>247.432514126667</v>
+        <v>322.665921933333</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2210,15 +2210,15 @@
       </c>
       <c r="B36" s="17" t="n">
         <f aca="false">A36*B5</f>
-        <v>1540</v>
+        <v>1400</v>
       </c>
       <c r="C36" s="17" t="n">
         <f aca="false">A36*B9</f>
-        <v>1655.13497174667</v>
+        <v>1504.66815613333</v>
       </c>
       <c r="D36" s="17" t="n">
         <f aca="false">$B$13-C36</f>
-        <v>-580.134971746667</v>
+        <v>-429.668156133333</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2227,15 +2227,15 @@
       </c>
       <c r="B37" s="17" t="n">
         <f aca="false">A37*B5</f>
-        <v>2310</v>
+        <v>2100</v>
       </c>
       <c r="C37" s="17" t="n">
         <f aca="false">A37*B9</f>
-        <v>2482.70245762</v>
+        <v>2257.0022342</v>
       </c>
       <c r="D37" s="17" t="n">
         <f aca="false">$B$13-C37</f>
-        <v>-1407.70245762</v>
+        <v>-1182.0022342</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2244,15 +2244,15 @@
       </c>
       <c r="B38" s="17" t="n">
         <f aca="false">A38*B5</f>
-        <v>3850</v>
+        <v>3500</v>
       </c>
       <c r="C38" s="17" t="n">
         <f aca="false">A38*B9</f>
-        <v>4137.83742936667</v>
+        <v>3761.67039033333</v>
       </c>
       <c r="D38" s="17" t="n">
         <f aca="false">$B$13-C38</f>
-        <v>-3062.83742936667</v>
+        <v>-2686.67039033333</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2261,15 +2261,15 @@
       </c>
       <c r="B39" s="17" t="n">
         <f aca="false">A39*B5</f>
-        <v>7700</v>
+        <v>7000</v>
       </c>
       <c r="C39" s="17" t="n">
         <f aca="false">A39*B9</f>
-        <v>8275.67485873333</v>
+        <v>7523.34078066667</v>
       </c>
       <c r="D39" s="17" t="n">
         <f aca="false">$B$13-C39</f>
-        <v>-7200.67485873333</v>
+        <v>-6448.34078066667</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2338,7 +2338,7 @@
         <v>66</v>
       </c>
       <c r="B6" s="20" t="n">
-        <v>385</v>
+        <v>350</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>67</v>
@@ -2380,7 +2380,7 @@
         <v>74</v>
       </c>
       <c r="B9" s="20" t="n">
-        <v>385</v>
+        <v>350</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>67</v>
@@ -3621,7 +3621,7 @@
       </c>
       <c r="C5" s="12" t="n">
         <f aca="false">IF(A5&lt;=Premissas!$B$7,Premissas!$B$6/Premissas!$B$7,IF(A5&lt;=Premissas!$B$7+Premissas!$B$8,0,IF(A5&lt;=Premissas!$B$7+Premissas!$B$8+Premissas!$B$10,Premissas!$B$9/Premissas!$B$10,0)))</f>
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="D5" s="15" t="n">
         <f aca="false">IF(Y5&gt;0,IF(DAY(B5)&lt;=Premissas!$B$12,DATE(YEAR(B5),MONTH(B5),Premissas!$B$16),DATE(YEAR(B5),MONTH(B5)+1,Premissas!$B$16))-Premissas!$B$11+1-Premissas!$B$15,0)</f>
@@ -3637,11 +3637,11 @@
       </c>
       <c r="G5" s="29" t="n">
         <f aca="false">C5/Premissas!$B$18*Premissas!$B$19*Premissas!$B$23</f>
-        <v>2.56666666666667</v>
+        <v>2.33333333333333</v>
       </c>
       <c r="H5" s="29" t="n">
         <f aca="false">C5/Premissas!$B$18*Premissas!$B$19*Premissas!$B$24</f>
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="I5" s="12" t="n">
         <f aca="false">-IF($A5-(Premissas!$B$60)&gt;=1,INDEX($G$5:$G$94,$A5-(Premissas!$B$60)),0)*(Premissas!$B$59*Unitário!$B$22+(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25))</f>
@@ -3661,7 +3661,7 @@
       </c>
       <c r="M5" s="12" t="n">
         <f aca="false">IF($A5-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A5-(Premissas!$B$56)),0)*(Premissas!$B$52-Unitário!$B$27)</f>
-        <v>124.21226015</v>
+        <v>112.9202365</v>
       </c>
       <c r="N5" s="12" t="n">
         <f aca="false">-IF($A5-(Premissas!$B$60)&gt;=1,INDEX($H$5:$H$94,$A5-(Premissas!$B$60)),0)*(Premissas!$B$59*Unitário!$B$22+Premissas!$B$31)</f>
@@ -3681,11 +3681,11 @@
       </c>
       <c r="R5" s="12" t="n">
         <f aca="false">E5+F5+SUM(I5:Q5)</f>
-        <v>124.21226015</v>
+        <v>112.9202365</v>
       </c>
       <c r="S5" s="12" t="n">
         <f aca="false">R5</f>
-        <v>124.21226015</v>
+        <v>112.9202365</v>
       </c>
       <c r="T5" s="15" t="n">
         <f aca="false">IF(AND($A5&gt;$B$100,S5&gt;=0),1,0)</f>
@@ -3693,11 +3693,11 @@
       </c>
       <c r="U5" s="12" t="n">
         <f aca="false">S5-SUM($E$5:E5)-(1+Premissas!$B$17)*SUM($C$5:C5)</f>
-        <v>61.60576015</v>
+        <v>56.0052365</v>
       </c>
       <c r="V5" s="12" t="n">
         <f aca="false">(G5+H5)*Premissas!$B$21</f>
-        <v>0.146666666666667</v>
+        <v>0.133333333333333</v>
       </c>
       <c r="W5" s="15" t="n">
         <f aca="false">IF(V5&gt;0,DATE(YEAR(B5),MONTH(B5)+1,Premissas!$B$16)-Premissas!$B$11+1-Premissas!$B$15,0)</f>
@@ -3705,7 +3705,7 @@
       </c>
       <c r="X5" s="12" t="n">
         <f aca="false">C5*(1+Premissas!$B$17)</f>
-        <v>62.6065</v>
+        <v>56.915</v>
       </c>
       <c r="Y5" s="12" t="n">
         <f aca="false">IF(OR(X5&gt;=Premissas!$B$13,B5=DATE(YEAR(B5),MONTH(B5)+1,0)),X5,0)</f>
@@ -3713,7 +3713,7 @@
       </c>
       <c r="Z5" s="12" t="n">
         <f aca="false">C5/Premissas!$B$18*Premissas!$B$20</f>
-        <v>9.9</v>
+        <v>9</v>
       </c>
       <c r="AA5" s="12" t="n">
         <f aca="false">IF(OR(Z5&gt;=Premissas!$B$14,B5=DATE(YEAR(B5),MONTH(B5)+1,0)),Z5,0)</f>
@@ -3734,7 +3734,7 @@
       </c>
       <c r="C6" s="12" t="n">
         <f aca="false">IF(A6&lt;=Premissas!$B$7,Premissas!$B$6/Premissas!$B$7,IF(A6&lt;=Premissas!$B$7+Premissas!$B$8,0,IF(A6&lt;=Premissas!$B$7+Premissas!$B$8+Premissas!$B$10,Premissas!$B$9/Premissas!$B$10,0)))</f>
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="D6" s="15" t="n">
         <f aca="false">IF(Y6&gt;0,IF(DAY(B6)&lt;=Premissas!$B$12,DATE(YEAR(B6),MONTH(B6),Premissas!$B$16),DATE(YEAR(B6),MONTH(B6)+1,Premissas!$B$16))-Premissas!$B$11+1-Premissas!$B$15,0)</f>
@@ -3750,15 +3750,15 @@
       </c>
       <c r="G6" s="29" t="n">
         <f aca="false">C6/Premissas!$B$18*Premissas!$B$19*Premissas!$B$23</f>
-        <v>2.56666666666667</v>
+        <v>2.33333333333333</v>
       </c>
       <c r="H6" s="29" t="n">
         <f aca="false">C6/Premissas!$B$18*Premissas!$B$19*Premissas!$B$24</f>
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="I6" s="12" t="n">
         <f aca="false">-IF($A6-(Premissas!$B$60)&gt;=1,INDEX($G$5:$G$94,$A6-(Premissas!$B$60)),0)*(Premissas!$B$59*Unitário!$B$22+(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25))</f>
-        <v>-170.837359</v>
+        <v>-155.30669</v>
       </c>
       <c r="J6" s="12" t="n">
         <f aca="false">IF($A6-(Premissas!$B$54)&gt;=1,INDEX($G$5:$G$94,$A6-(Premissas!$B$54)),0)*Premissas!$B$26*((Premissas!$B$59*Unitário!$B$22+(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25))-Premissas!$B$39)</f>
@@ -3774,11 +3774,11 @@
       </c>
       <c r="M6" s="12" t="n">
         <f aca="false">IF($A6-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A6-(Premissas!$B$56)),0)*(Premissas!$B$52-Unitário!$B$27)</f>
-        <v>124.21226015</v>
+        <v>112.9202365</v>
       </c>
       <c r="N6" s="12" t="n">
         <f aca="false">-IF($A6-(Premissas!$B$60)&gt;=1,INDEX($H$5:$H$94,$A6-(Premissas!$B$60)),0)*(Premissas!$B$59*Unitário!$B$22+Premissas!$B$31)</f>
-        <v>-38.5</v>
+        <v>-35</v>
       </c>
       <c r="O6" s="12" t="n">
         <f aca="false">IF($A6-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($H$5:$H$94,$A6-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(-Premissas!$B$52-Premissas!$B$41+(1-Premissas!$B$62)*Premissas!$B$31+Premissas!$B$59*Unitário!$B$22)</f>
@@ -3794,11 +3794,11 @@
       </c>
       <c r="R6" s="12" t="n">
         <f aca="false">E6+F6+SUM(I6:Q6)</f>
-        <v>-85.12509885</v>
+        <v>-77.3864535</v>
       </c>
       <c r="S6" s="12" t="n">
         <f aca="false">S5+R6</f>
-        <v>39.0871613</v>
+        <v>35.533783</v>
       </c>
       <c r="T6" s="15" t="n">
         <f aca="false">IF(AND($A6&gt;$B$100,S6&gt;=0),1,0)</f>
@@ -3806,11 +3806,11 @@
       </c>
       <c r="U6" s="12" t="n">
         <f aca="false">S6-SUM($E$5:E6)-(1+Premissas!$B$17)*SUM($C$5:C6)</f>
-        <v>-86.1258387</v>
+        <v>-78.296217</v>
       </c>
       <c r="V6" s="12" t="n">
         <f aca="false">(G6+H6)*Premissas!$B$21</f>
-        <v>0.146666666666667</v>
+        <v>0.133333333333333</v>
       </c>
       <c r="W6" s="15" t="n">
         <f aca="false">IF(V6&gt;0,DATE(YEAR(B6),MONTH(B6)+1,Premissas!$B$16)-Premissas!$B$11+1-Premissas!$B$15,0)</f>
@@ -3818,15 +3818,15 @@
       </c>
       <c r="X6" s="12" t="n">
         <f aca="false">X5-Y5+C6*(1+Premissas!$B$17)</f>
-        <v>125.213</v>
+        <v>113.83</v>
       </c>
       <c r="Y6" s="12" t="n">
         <f aca="false">IF(OR(X6&gt;=Premissas!$B$13,B6=DATE(YEAR(B6),MONTH(B6)+1,0)),X6,0)</f>
-        <v>125.213</v>
+        <v>113.83</v>
       </c>
       <c r="Z6" s="12" t="n">
         <f aca="false">Z5-AA5+C6/Premissas!$B$18*Premissas!$B$20</f>
-        <v>19.8</v>
+        <v>18</v>
       </c>
       <c r="AA6" s="12" t="n">
         <f aca="false">IF(OR(Z6&gt;=Premissas!$B$14,B6=DATE(YEAR(B6),MONTH(B6)+1,0)),Z6,0)</f>
@@ -3847,7 +3847,7 @@
       </c>
       <c r="C7" s="12" t="n">
         <f aca="false">IF(A7&lt;=Premissas!$B$7,Premissas!$B$6/Premissas!$B$7,IF(A7&lt;=Premissas!$B$7+Premissas!$B$8,0,IF(A7&lt;=Premissas!$B$7+Premissas!$B$8+Premissas!$B$10,Premissas!$B$9/Premissas!$B$10,0)))</f>
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="D7" s="15" t="n">
         <f aca="false">IF(Y7&gt;0,IF(DAY(B7)&lt;=Premissas!$B$12,DATE(YEAR(B7),MONTH(B7),Premissas!$B$16),DATE(YEAR(B7),MONTH(B7)+1,Premissas!$B$16))-Premissas!$B$11+1-Premissas!$B$15,0)</f>
@@ -3863,19 +3863,19 @@
       </c>
       <c r="G7" s="29" t="n">
         <f aca="false">C7/Premissas!$B$18*Premissas!$B$19*Premissas!$B$23</f>
-        <v>2.56666666666667</v>
+        <v>2.33333333333333</v>
       </c>
       <c r="H7" s="29" t="n">
         <f aca="false">C7/Premissas!$B$18*Premissas!$B$19*Premissas!$B$24</f>
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="I7" s="12" t="n">
         <f aca="false">-IF($A7-(Premissas!$B$60)&gt;=1,INDEX($G$5:$G$94,$A7-(Premissas!$B$60)),0)*(Premissas!$B$59*Unitário!$B$22+(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25))</f>
-        <v>-170.837359</v>
+        <v>-155.30669</v>
       </c>
       <c r="J7" s="12" t="n">
         <f aca="false">IF($A7-(Premissas!$B$54)&gt;=1,INDEX($G$5:$G$94,$A7-(Premissas!$B$54)),0)*Premissas!$B$26*((Premissas!$B$59*Unitário!$B$22+(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25))-Premissas!$B$39)</f>
-        <v>24.68338103</v>
+        <v>22.4394373</v>
       </c>
       <c r="K7" s="12" t="n">
         <f aca="false">IF($A7-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($G$5:$G$94,$A7-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(Premissas!$B$59*Unitário!$B$22+(1-Premissas!$B$62)*(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25)-Premissas!$B$62*((1-Premissas!$B$61)*Unitário!$B$24+(1-Premissas!$B$63)*Unitário!$B$25)-Premissas!$B$41)</f>
@@ -3887,11 +3887,11 @@
       </c>
       <c r="M7" s="12" t="n">
         <f aca="false">IF($A7-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A7-(Premissas!$B$56)),0)*(Premissas!$B$52-Unitário!$B$27)</f>
-        <v>124.21226015</v>
+        <v>112.9202365</v>
       </c>
       <c r="N7" s="12" t="n">
         <f aca="false">-IF($A7-(Premissas!$B$60)&gt;=1,INDEX($H$5:$H$94,$A7-(Premissas!$B$60)),0)*(Premissas!$B$59*Unitário!$B$22+Premissas!$B$31)</f>
-        <v>-38.5</v>
+        <v>-35</v>
       </c>
       <c r="O7" s="12" t="n">
         <f aca="false">IF($A7-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($H$5:$H$94,$A7-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(-Premissas!$B$52-Premissas!$B$41+(1-Premissas!$B$62)*Premissas!$B$31+Premissas!$B$59*Unitário!$B$22)</f>
@@ -3907,11 +3907,11 @@
       </c>
       <c r="R7" s="12" t="n">
         <f aca="false">E7+F7+SUM(I7:Q7)</f>
-        <v>-60.44171782</v>
+        <v>-54.9470162</v>
       </c>
       <c r="S7" s="12" t="n">
         <f aca="false">S6+R7</f>
-        <v>-21.35455652</v>
+        <v>-19.4132332</v>
       </c>
       <c r="T7" s="15" t="n">
         <f aca="false">IF(AND($A7&gt;$B$100,S7&gt;=0),1,0)</f>
@@ -3919,11 +3919,11 @@
       </c>
       <c r="U7" s="12" t="n">
         <f aca="false">S7-SUM($E$5:E7)-(1+Premissas!$B$17)*SUM($C$5:C7)</f>
-        <v>-209.17405652</v>
+        <v>-190.1582332</v>
       </c>
       <c r="V7" s="12" t="n">
         <f aca="false">(G7+H7)*Premissas!$B$21</f>
-        <v>0.146666666666667</v>
+        <v>0.133333333333333</v>
       </c>
       <c r="W7" s="15" t="n">
         <f aca="false">IF(V7&gt;0,DATE(YEAR(B7),MONTH(B7)+1,Premissas!$B$16)-Premissas!$B$11+1-Premissas!$B$15,0)</f>
@@ -3931,7 +3931,7 @@
       </c>
       <c r="X7" s="12" t="n">
         <f aca="false">X6-Y6+C7*(1+Premissas!$B$17)</f>
-        <v>62.6065</v>
+        <v>56.915</v>
       </c>
       <c r="Y7" s="12" t="n">
         <f aca="false">IF(OR(X7&gt;=Premissas!$B$13,B7=DATE(YEAR(B7),MONTH(B7)+1,0)),X7,0)</f>
@@ -3939,11 +3939,11 @@
       </c>
       <c r="Z7" s="12" t="n">
         <f aca="false">Z6-AA6+C7/Premissas!$B$18*Premissas!$B$20</f>
-        <v>29.7</v>
+        <v>27</v>
       </c>
       <c r="AA7" s="12" t="n">
         <f aca="false">IF(OR(Z7&gt;=Premissas!$B$14,B7=DATE(YEAR(B7),MONTH(B7)+1,0)),Z7,0)</f>
-        <v>29.7</v>
+        <v>27</v>
       </c>
       <c r="AB7" s="15" t="n">
         <f aca="false">IF(AA7&gt;0,IF(DAY(B7)&lt;=Premissas!$B$12,DATE(YEAR(B7),MONTH(B7),Premissas!$B$16),DATE(YEAR(B7),MONTH(B7)+1,Premissas!$B$16))-Premissas!$B$11+1-Premissas!$B$15,0)</f>
@@ -3960,7 +3960,7 @@
       </c>
       <c r="C8" s="12" t="n">
         <f aca="false">IF(A8&lt;=Premissas!$B$7,Premissas!$B$6/Premissas!$B$7,IF(A8&lt;=Premissas!$B$7+Premissas!$B$8,0,IF(A8&lt;=Premissas!$B$7+Premissas!$B$8+Premissas!$B$10,Premissas!$B$9/Premissas!$B$10,0)))</f>
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="D8" s="15" t="n">
         <f aca="false">IF(Y8&gt;0,IF(DAY(B8)&lt;=Premissas!$B$12,DATE(YEAR(B8),MONTH(B8),Premissas!$B$16),DATE(YEAR(B8),MONTH(B8)+1,Premissas!$B$16))-Premissas!$B$11+1-Premissas!$B$15,0)</f>
@@ -3976,19 +3976,19 @@
       </c>
       <c r="G8" s="29" t="n">
         <f aca="false">C8/Premissas!$B$18*Premissas!$B$19*Premissas!$B$23</f>
-        <v>2.56666666666667</v>
+        <v>2.33333333333333</v>
       </c>
       <c r="H8" s="29" t="n">
         <f aca="false">C8/Premissas!$B$18*Premissas!$B$19*Premissas!$B$24</f>
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="I8" s="12" t="n">
         <f aca="false">-IF($A8-(Premissas!$B$60)&gt;=1,INDEX($G$5:$G$94,$A8-(Premissas!$B$60)),0)*(Premissas!$B$59*Unitário!$B$22+(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25))</f>
-        <v>-170.837359</v>
+        <v>-155.30669</v>
       </c>
       <c r="J8" s="12" t="n">
         <f aca="false">IF($A8-(Premissas!$B$54)&gt;=1,INDEX($G$5:$G$94,$A8-(Premissas!$B$54)),0)*Premissas!$B$26*((Premissas!$B$59*Unitário!$B$22+(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25))-Premissas!$B$39)</f>
-        <v>24.68338103</v>
+        <v>22.4394373</v>
       </c>
       <c r="K8" s="12" t="n">
         <f aca="false">IF($A8-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($G$5:$G$94,$A8-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(Premissas!$B$59*Unitário!$B$22+(1-Premissas!$B$62)*(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25)-Premissas!$B$62*((1-Premissas!$B$61)*Unitário!$B$24+(1-Premissas!$B$63)*Unitário!$B$25)-Premissas!$B$41)</f>
@@ -4000,11 +4000,11 @@
       </c>
       <c r="M8" s="12" t="n">
         <f aca="false">IF($A8-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A8-(Premissas!$B$56)),0)*(Premissas!$B$52-Unitário!$B$27)</f>
-        <v>124.21226015</v>
+        <v>112.9202365</v>
       </c>
       <c r="N8" s="12" t="n">
         <f aca="false">-IF($A8-(Premissas!$B$60)&gt;=1,INDEX($H$5:$H$94,$A8-(Premissas!$B$60)),0)*(Premissas!$B$59*Unitário!$B$22+Premissas!$B$31)</f>
-        <v>-38.5</v>
+        <v>-35</v>
       </c>
       <c r="O8" s="12" t="n">
         <f aca="false">IF($A8-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($H$5:$H$94,$A8-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(-Premissas!$B$52-Premissas!$B$41+(1-Premissas!$B$62)*Premissas!$B$31+Premissas!$B$59*Unitário!$B$22)</f>
@@ -4020,11 +4020,11 @@
       </c>
       <c r="R8" s="12" t="n">
         <f aca="false">E8+F8+SUM(I8:Q8)</f>
-        <v>-60.44171782</v>
+        <v>-54.9470162</v>
       </c>
       <c r="S8" s="12" t="n">
         <f aca="false">S7+R8</f>
-        <v>-81.7962743399999</v>
+        <v>-74.3602494</v>
       </c>
       <c r="T8" s="15" t="n">
         <f aca="false">IF(AND($A8&gt;$B$100,S8&gt;=0),1,0)</f>
@@ -4032,11 +4032,11 @@
       </c>
       <c r="U8" s="12" t="n">
         <f aca="false">S8-SUM($E$5:E8)-(1+Premissas!$B$17)*SUM($C$5:C8)</f>
-        <v>-332.22227434</v>
+        <v>-302.0202494</v>
       </c>
       <c r="V8" s="12" t="n">
         <f aca="false">(G8+H8)*Premissas!$B$21</f>
-        <v>0.146666666666667</v>
+        <v>0.133333333333333</v>
       </c>
       <c r="W8" s="15" t="n">
         <f aca="false">IF(V8&gt;0,DATE(YEAR(B8),MONTH(B8)+1,Premissas!$B$16)-Premissas!$B$11+1-Premissas!$B$15,0)</f>
@@ -4044,15 +4044,15 @@
       </c>
       <c r="X8" s="12" t="n">
         <f aca="false">X7-Y7+C8*(1+Premissas!$B$17)</f>
-        <v>125.213</v>
+        <v>113.83</v>
       </c>
       <c r="Y8" s="12" t="n">
         <f aca="false">IF(OR(X8&gt;=Premissas!$B$13,B8=DATE(YEAR(B8),MONTH(B8)+1,0)),X8,0)</f>
-        <v>125.213</v>
+        <v>113.83</v>
       </c>
       <c r="Z8" s="12" t="n">
         <f aca="false">Z7-AA7+C8/Premissas!$B$18*Premissas!$B$20</f>
-        <v>9.9</v>
+        <v>9</v>
       </c>
       <c r="AA8" s="12" t="n">
         <f aca="false">IF(OR(Z8&gt;=Premissas!$B$14,B8=DATE(YEAR(B8),MONTH(B8)+1,0)),Z8,0)</f>
@@ -4073,7 +4073,7 @@
       </c>
       <c r="C9" s="12" t="n">
         <f aca="false">IF(A9&lt;=Premissas!$B$7,Premissas!$B$6/Premissas!$B$7,IF(A9&lt;=Premissas!$B$7+Premissas!$B$8,0,IF(A9&lt;=Premissas!$B$7+Premissas!$B$8+Premissas!$B$10,Premissas!$B$9/Premissas!$B$10,0)))</f>
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="D9" s="15" t="n">
         <f aca="false">IF(Y9&gt;0,IF(DAY(B9)&lt;=Premissas!$B$12,DATE(YEAR(B9),MONTH(B9),Premissas!$B$16),DATE(YEAR(B9),MONTH(B9)+1,Premissas!$B$16))-Premissas!$B$11+1-Premissas!$B$15,0)</f>
@@ -4089,19 +4089,19 @@
       </c>
       <c r="G9" s="29" t="n">
         <f aca="false">C9/Premissas!$B$18*Premissas!$B$19*Premissas!$B$23</f>
-        <v>2.56666666666667</v>
+        <v>2.33333333333333</v>
       </c>
       <c r="H9" s="29" t="n">
         <f aca="false">C9/Premissas!$B$18*Premissas!$B$19*Premissas!$B$24</f>
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="I9" s="12" t="n">
         <f aca="false">-IF($A9-(Premissas!$B$60)&gt;=1,INDEX($G$5:$G$94,$A9-(Premissas!$B$60)),0)*(Premissas!$B$59*Unitário!$B$22+(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25))</f>
-        <v>-170.837359</v>
+        <v>-155.30669</v>
       </c>
       <c r="J9" s="12" t="n">
         <f aca="false">IF($A9-(Premissas!$B$54)&gt;=1,INDEX($G$5:$G$94,$A9-(Premissas!$B$54)),0)*Premissas!$B$26*((Premissas!$B$59*Unitário!$B$22+(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25))-Premissas!$B$39)</f>
-        <v>24.68338103</v>
+        <v>22.4394373</v>
       </c>
       <c r="K9" s="12" t="n">
         <f aca="false">IF($A9-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($G$5:$G$94,$A9-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(Premissas!$B$59*Unitário!$B$22+(1-Premissas!$B$62)*(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25)-Premissas!$B$62*((1-Premissas!$B$61)*Unitário!$B$24+(1-Premissas!$B$63)*Unitário!$B$25)-Premissas!$B$41)</f>
@@ -4113,11 +4113,11 @@
       </c>
       <c r="M9" s="12" t="n">
         <f aca="false">IF($A9-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A9-(Premissas!$B$56)),0)*(Premissas!$B$52-Unitário!$B$27)</f>
-        <v>124.21226015</v>
+        <v>112.9202365</v>
       </c>
       <c r="N9" s="12" t="n">
         <f aca="false">-IF($A9-(Premissas!$B$60)&gt;=1,INDEX($H$5:$H$94,$A9-(Premissas!$B$60)),0)*(Premissas!$B$59*Unitário!$B$22+Premissas!$B$31)</f>
-        <v>-38.5</v>
+        <v>-35</v>
       </c>
       <c r="O9" s="12" t="n">
         <f aca="false">IF($A9-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($H$5:$H$94,$A9-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(-Premissas!$B$52-Premissas!$B$41+(1-Premissas!$B$62)*Premissas!$B$31+Premissas!$B$59*Unitário!$B$22)</f>
@@ -4133,11 +4133,11 @@
       </c>
       <c r="R9" s="12" t="n">
         <f aca="false">E9+F9+SUM(I9:Q9)</f>
-        <v>-60.44171782</v>
+        <v>-54.9470162</v>
       </c>
       <c r="S9" s="12" t="n">
         <f aca="false">S8+R9</f>
-        <v>-142.23799216</v>
+        <v>-129.3072656</v>
       </c>
       <c r="T9" s="15" t="n">
         <f aca="false">IF(AND($A9&gt;$B$100,S9&gt;=0),1,0)</f>
@@ -4145,11 +4145,11 @@
       </c>
       <c r="U9" s="12" t="n">
         <f aca="false">S9-SUM($E$5:E9)-(1+Premissas!$B$17)*SUM($C$5:C9)</f>
-        <v>-455.27049216</v>
+        <v>-413.8822656</v>
       </c>
       <c r="V9" s="12" t="n">
         <f aca="false">(G9+H9)*Premissas!$B$21</f>
-        <v>0.146666666666667</v>
+        <v>0.133333333333333</v>
       </c>
       <c r="W9" s="15" t="n">
         <f aca="false">IF(V9&gt;0,DATE(YEAR(B9),MONTH(B9)+1,Premissas!$B$16)-Premissas!$B$11+1-Premissas!$B$15,0)</f>
@@ -4157,7 +4157,7 @@
       </c>
       <c r="X9" s="12" t="n">
         <f aca="false">X8-Y8+C9*(1+Premissas!$B$17)</f>
-        <v>62.6065</v>
+        <v>56.915</v>
       </c>
       <c r="Y9" s="12" t="n">
         <f aca="false">IF(OR(X9&gt;=Premissas!$B$13,B9=DATE(YEAR(B9),MONTH(B9)+1,0)),X9,0)</f>
@@ -4165,7 +4165,7 @@
       </c>
       <c r="Z9" s="12" t="n">
         <f aca="false">Z8-AA8+C9/Premissas!$B$18*Premissas!$B$20</f>
-        <v>19.8</v>
+        <v>18</v>
       </c>
       <c r="AA9" s="12" t="n">
         <f aca="false">IF(OR(Z9&gt;=Premissas!$B$14,B9=DATE(YEAR(B9),MONTH(B9)+1,0)),Z9,0)</f>
@@ -4186,7 +4186,7 @@
       </c>
       <c r="C10" s="12" t="n">
         <f aca="false">IF(A10&lt;=Premissas!$B$7,Premissas!$B$6/Premissas!$B$7,IF(A10&lt;=Premissas!$B$7+Premissas!$B$8,0,IF(A10&lt;=Premissas!$B$7+Premissas!$B$8+Premissas!$B$10,Premissas!$B$9/Premissas!$B$10,0)))</f>
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="D10" s="15" t="n">
         <f aca="false">IF(Y10&gt;0,IF(DAY(B10)&lt;=Premissas!$B$12,DATE(YEAR(B10),MONTH(B10),Premissas!$B$16),DATE(YEAR(B10),MONTH(B10)+1,Premissas!$B$16))-Premissas!$B$11+1-Premissas!$B$15,0)</f>
@@ -4202,19 +4202,19 @@
       </c>
       <c r="G10" s="29" t="n">
         <f aca="false">C10/Premissas!$B$18*Premissas!$B$19*Premissas!$B$23</f>
-        <v>2.56666666666667</v>
+        <v>2.33333333333333</v>
       </c>
       <c r="H10" s="29" t="n">
         <f aca="false">C10/Premissas!$B$18*Premissas!$B$19*Premissas!$B$24</f>
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="I10" s="12" t="n">
         <f aca="false">-IF($A10-(Premissas!$B$60)&gt;=1,INDEX($G$5:$G$94,$A10-(Premissas!$B$60)),0)*(Premissas!$B$59*Unitário!$B$22+(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25))</f>
-        <v>-170.837359</v>
+        <v>-155.30669</v>
       </c>
       <c r="J10" s="12" t="n">
         <f aca="false">IF($A10-(Premissas!$B$54)&gt;=1,INDEX($G$5:$G$94,$A10-(Premissas!$B$54)),0)*Premissas!$B$26*((Premissas!$B$59*Unitário!$B$22+(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25))-Premissas!$B$39)</f>
-        <v>24.68338103</v>
+        <v>22.4394373</v>
       </c>
       <c r="K10" s="12" t="n">
         <f aca="false">IF($A10-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($G$5:$G$94,$A10-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(Premissas!$B$59*Unitário!$B$22+(1-Premissas!$B$62)*(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25)-Premissas!$B$62*((1-Premissas!$B$61)*Unitário!$B$24+(1-Premissas!$B$63)*Unitário!$B$25)-Premissas!$B$41)</f>
@@ -4226,11 +4226,11 @@
       </c>
       <c r="M10" s="12" t="n">
         <f aca="false">IF($A10-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A10-(Premissas!$B$56)),0)*(Premissas!$B$52-Unitário!$B$27)</f>
-        <v>124.21226015</v>
+        <v>112.9202365</v>
       </c>
       <c r="N10" s="12" t="n">
         <f aca="false">-IF($A10-(Premissas!$B$60)&gt;=1,INDEX($H$5:$H$94,$A10-(Premissas!$B$60)),0)*(Premissas!$B$59*Unitário!$B$22+Premissas!$B$31)</f>
-        <v>-38.5</v>
+        <v>-35</v>
       </c>
       <c r="O10" s="12" t="n">
         <f aca="false">IF($A10-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($H$5:$H$94,$A10-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(-Premissas!$B$52-Premissas!$B$41+(1-Premissas!$B$62)*Premissas!$B$31+Premissas!$B$59*Unitário!$B$22)</f>
@@ -4246,11 +4246,11 @@
       </c>
       <c r="R10" s="12" t="n">
         <f aca="false">E10+F10+SUM(I10:Q10)</f>
-        <v>-60.44171782</v>
+        <v>-54.9470162</v>
       </c>
       <c r="S10" s="12" t="n">
         <f aca="false">S9+R10</f>
-        <v>-202.67970998</v>
+        <v>-184.2542818</v>
       </c>
       <c r="T10" s="15" t="n">
         <f aca="false">IF(AND($A10&gt;$B$100,S10&gt;=0),1,0)</f>
@@ -4258,11 +4258,11 @@
       </c>
       <c r="U10" s="12" t="n">
         <f aca="false">S10-SUM($E$5:E10)-(1+Premissas!$B$17)*SUM($C$5:C10)</f>
-        <v>-578.31870998</v>
+        <v>-525.7442818</v>
       </c>
       <c r="V10" s="12" t="n">
         <f aca="false">(G10+H10)*Premissas!$B$21</f>
-        <v>0.146666666666667</v>
+        <v>0.133333333333333</v>
       </c>
       <c r="W10" s="15" t="n">
         <f aca="false">IF(V10&gt;0,DATE(YEAR(B10),MONTH(B10)+1,Premissas!$B$16)-Premissas!$B$11+1-Premissas!$B$15,0)</f>
@@ -4270,19 +4270,19 @@
       </c>
       <c r="X10" s="12" t="n">
         <f aca="false">X9-Y9+C10*(1+Premissas!$B$17)</f>
-        <v>125.213</v>
+        <v>113.83</v>
       </c>
       <c r="Y10" s="12" t="n">
         <f aca="false">IF(OR(X10&gt;=Premissas!$B$13,B10=DATE(YEAR(B10),MONTH(B10)+1,0)),X10,0)</f>
-        <v>125.213</v>
+        <v>113.83</v>
       </c>
       <c r="Z10" s="12" t="n">
         <f aca="false">Z9-AA9+C10/Premissas!$B$18*Premissas!$B$20</f>
-        <v>29.7</v>
+        <v>27</v>
       </c>
       <c r="AA10" s="12" t="n">
         <f aca="false">IF(OR(Z10&gt;=Premissas!$B$14,B10=DATE(YEAR(B10),MONTH(B10)+1,0)),Z10,0)</f>
-        <v>29.7</v>
+        <v>27</v>
       </c>
       <c r="AB10" s="15" t="n">
         <f aca="false">IF(AA10&gt;0,IF(DAY(B10)&lt;=Premissas!$B$12,DATE(YEAR(B10),MONTH(B10),Premissas!$B$16),DATE(YEAR(B10),MONTH(B10)+1,Premissas!$B$16))-Premissas!$B$11+1-Premissas!$B$15,0)</f>
@@ -4299,7 +4299,7 @@
       </c>
       <c r="C11" s="12" t="n">
         <f aca="false">IF(A11&lt;=Premissas!$B$7,Premissas!$B$6/Premissas!$B$7,IF(A11&lt;=Premissas!$B$7+Premissas!$B$8,0,IF(A11&lt;=Premissas!$B$7+Premissas!$B$8+Premissas!$B$10,Premissas!$B$9/Premissas!$B$10,0)))</f>
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="D11" s="15" t="n">
         <f aca="false">IF(Y11&gt;0,IF(DAY(B11)&lt;=Premissas!$B$12,DATE(YEAR(B11),MONTH(B11),Premissas!$B$16),DATE(YEAR(B11),MONTH(B11)+1,Premissas!$B$16))-Premissas!$B$11+1-Premissas!$B$15,0)</f>
@@ -4315,19 +4315,19 @@
       </c>
       <c r="G11" s="29" t="n">
         <f aca="false">C11/Premissas!$B$18*Premissas!$B$19*Premissas!$B$23</f>
-        <v>2.56666666666667</v>
+        <v>2.33333333333333</v>
       </c>
       <c r="H11" s="29" t="n">
         <f aca="false">C11/Premissas!$B$18*Premissas!$B$19*Premissas!$B$24</f>
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="I11" s="12" t="n">
         <f aca="false">-IF($A11-(Premissas!$B$60)&gt;=1,INDEX($G$5:$G$94,$A11-(Premissas!$B$60)),0)*(Premissas!$B$59*Unitário!$B$22+(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25))</f>
-        <v>-170.837359</v>
+        <v>-155.30669</v>
       </c>
       <c r="J11" s="12" t="n">
         <f aca="false">IF($A11-(Premissas!$B$54)&gt;=1,INDEX($G$5:$G$94,$A11-(Premissas!$B$54)),0)*Premissas!$B$26*((Premissas!$B$59*Unitário!$B$22+(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25))-Premissas!$B$39)</f>
-        <v>24.68338103</v>
+        <v>22.4394373</v>
       </c>
       <c r="K11" s="12" t="n">
         <f aca="false">IF($A11-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($G$5:$G$94,$A11-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(Premissas!$B$59*Unitário!$B$22+(1-Premissas!$B$62)*(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25)-Premissas!$B$62*((1-Premissas!$B$61)*Unitário!$B$24+(1-Premissas!$B$63)*Unitário!$B$25)-Premissas!$B$41)</f>
@@ -4339,11 +4339,11 @@
       </c>
       <c r="M11" s="12" t="n">
         <f aca="false">IF($A11-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A11-(Premissas!$B$56)),0)*(Premissas!$B$52-Unitário!$B$27)</f>
-        <v>124.21226015</v>
+        <v>112.9202365</v>
       </c>
       <c r="N11" s="12" t="n">
         <f aca="false">-IF($A11-(Premissas!$B$60)&gt;=1,INDEX($H$5:$H$94,$A11-(Premissas!$B$60)),0)*(Premissas!$B$59*Unitário!$B$22+Premissas!$B$31)</f>
-        <v>-38.5</v>
+        <v>-35</v>
       </c>
       <c r="O11" s="12" t="n">
         <f aca="false">IF($A11-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($H$5:$H$94,$A11-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(-Premissas!$B$52-Premissas!$B$41+(1-Premissas!$B$62)*Premissas!$B$31+Premissas!$B$59*Unitário!$B$22)</f>
@@ -4359,11 +4359,11 @@
       </c>
       <c r="R11" s="12" t="n">
         <f aca="false">E11+F11+SUM(I11:Q11)</f>
-        <v>-60.44171782</v>
+        <v>-54.9470162</v>
       </c>
       <c r="S11" s="12" t="n">
         <f aca="false">S10+R11</f>
-        <v>-263.1214278</v>
+        <v>-239.201298</v>
       </c>
       <c r="T11" s="15" t="n">
         <f aca="false">IF(AND($A11&gt;$B$100,S11&gt;=0),1,0)</f>
@@ -4371,11 +4371,11 @@
       </c>
       <c r="U11" s="12" t="n">
         <f aca="false">S11-SUM($E$5:E11)-(1+Premissas!$B$17)*SUM($C$5:C11)</f>
-        <v>-701.3669278</v>
+        <v>-637.606298</v>
       </c>
       <c r="V11" s="12" t="n">
         <f aca="false">(G11+H11)*Premissas!$B$21</f>
-        <v>0.146666666666667</v>
+        <v>0.133333333333333</v>
       </c>
       <c r="W11" s="15" t="n">
         <f aca="false">IF(V11&gt;0,DATE(YEAR(B11),MONTH(B11)+1,Premissas!$B$16)-Premissas!$B$11+1-Premissas!$B$15,0)</f>
@@ -4383,7 +4383,7 @@
       </c>
       <c r="X11" s="12" t="n">
         <f aca="false">X10-Y10+C11*(1+Premissas!$B$17)</f>
-        <v>62.6065</v>
+        <v>56.915</v>
       </c>
       <c r="Y11" s="12" t="n">
         <f aca="false">IF(OR(X11&gt;=Premissas!$B$13,B11=DATE(YEAR(B11),MONTH(B11)+1,0)),X11,0)</f>
@@ -4391,7 +4391,7 @@
       </c>
       <c r="Z11" s="12" t="n">
         <f aca="false">Z10-AA10+C11/Premissas!$B$18*Premissas!$B$20</f>
-        <v>9.9</v>
+        <v>9</v>
       </c>
       <c r="AA11" s="12" t="n">
         <f aca="false">IF(OR(Z11&gt;=Premissas!$B$14,B11=DATE(YEAR(B11),MONTH(B11)+1,0)),Z11,0)</f>
@@ -4436,11 +4436,11 @@
       </c>
       <c r="I12" s="12" t="n">
         <f aca="false">-IF($A12-(Premissas!$B$60)&gt;=1,INDEX($G$5:$G$94,$A12-(Premissas!$B$60)),0)*(Premissas!$B$59*Unitário!$B$22+(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25))</f>
-        <v>-170.837359</v>
+        <v>-155.30669</v>
       </c>
       <c r="J12" s="12" t="n">
         <f aca="false">IF($A12-(Premissas!$B$54)&gt;=1,INDEX($G$5:$G$94,$A12-(Premissas!$B$54)),0)*Premissas!$B$26*((Premissas!$B$59*Unitário!$B$22+(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25))-Premissas!$B$39)</f>
-        <v>24.68338103</v>
+        <v>22.4394373</v>
       </c>
       <c r="K12" s="12" t="n">
         <f aca="false">IF($A12-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($G$5:$G$94,$A12-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(Premissas!$B$59*Unitário!$B$22+(1-Premissas!$B$62)*(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25)-Premissas!$B$62*((1-Premissas!$B$61)*Unitário!$B$24+(1-Premissas!$B$63)*Unitário!$B$25)-Premissas!$B$41)</f>
@@ -4456,7 +4456,7 @@
       </c>
       <c r="N12" s="12" t="n">
         <f aca="false">-IF($A12-(Premissas!$B$60)&gt;=1,INDEX($H$5:$H$94,$A12-(Premissas!$B$60)),0)*(Premissas!$B$59*Unitário!$B$22+Premissas!$B$31)</f>
-        <v>-38.5</v>
+        <v>-35</v>
       </c>
       <c r="O12" s="12" t="n">
         <f aca="false">IF($A12-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($H$5:$H$94,$A12-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(-Premissas!$B$52-Premissas!$B$41+(1-Premissas!$B$62)*Premissas!$B$31+Premissas!$B$59*Unitário!$B$22)</f>
@@ -4472,11 +4472,11 @@
       </c>
       <c r="R12" s="12" t="n">
         <f aca="false">E12+F12+SUM(I12:Q12)</f>
-        <v>-184.65397797</v>
+        <v>-167.8672527</v>
       </c>
       <c r="S12" s="12" t="n">
         <f aca="false">S11+R12</f>
-        <v>-447.77540577</v>
+        <v>-407.0685507</v>
       </c>
       <c r="T12" s="15" t="n">
         <f aca="false">IF(AND($A12&gt;$B$100,S12&gt;=0),1,0)</f>
@@ -4484,7 +4484,7 @@
       </c>
       <c r="U12" s="12" t="n">
         <f aca="false">S12-SUM($E$5:E12)-(1+Premissas!$B$17)*SUM($C$5:C12)</f>
-        <v>-886.02090577</v>
+        <v>-805.4735507</v>
       </c>
       <c r="V12" s="12" t="n">
         <f aca="false">(G12+H12)*Premissas!$B$21</f>
@@ -4496,7 +4496,7 @@
       </c>
       <c r="X12" s="12" t="n">
         <f aca="false">X11-Y11+C12*(1+Premissas!$B$17)</f>
-        <v>62.6065</v>
+        <v>56.915</v>
       </c>
       <c r="Y12" s="12" t="n">
         <f aca="false">IF(OR(X12&gt;=Premissas!$B$13,B12=DATE(YEAR(B12),MONTH(B12)+1,0)),X12,0)</f>
@@ -4504,7 +4504,7 @@
       </c>
       <c r="Z12" s="12" t="n">
         <f aca="false">Z11-AA11+C12/Premissas!$B$18*Premissas!$B$20</f>
-        <v>9.9</v>
+        <v>9</v>
       </c>
       <c r="AA12" s="12" t="n">
         <f aca="false">IF(OR(Z12&gt;=Premissas!$B$14,B12=DATE(YEAR(B12),MONTH(B12)+1,0)),Z12,0)</f>
@@ -4553,7 +4553,7 @@
       </c>
       <c r="J13" s="12" t="n">
         <f aca="false">IF($A13-(Premissas!$B$54)&gt;=1,INDEX($G$5:$G$94,$A13-(Premissas!$B$54)),0)*Premissas!$B$26*((Premissas!$B$59*Unitário!$B$22+(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25))-Premissas!$B$39)</f>
-        <v>24.68338103</v>
+        <v>22.4394373</v>
       </c>
       <c r="K13" s="12" t="n">
         <f aca="false">IF($A13-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($G$5:$G$94,$A13-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(Premissas!$B$59*Unitário!$B$22+(1-Premissas!$B$62)*(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25)-Premissas!$B$62*((1-Premissas!$B$61)*Unitário!$B$24+(1-Premissas!$B$63)*Unitário!$B$25)-Premissas!$B$41)</f>
@@ -4585,11 +4585,11 @@
       </c>
       <c r="R13" s="12" t="n">
         <f aca="false">E13+F13+SUM(I13:Q13)</f>
-        <v>24.68338103</v>
+        <v>22.4394373</v>
       </c>
       <c r="S13" s="12" t="n">
         <f aca="false">S12+R13</f>
-        <v>-423.09202474</v>
+        <v>-384.6291134</v>
       </c>
       <c r="T13" s="15" t="n">
         <f aca="false">IF(AND($A13&gt;$B$100,S13&gt;=0),1,0)</f>
@@ -4597,7 +4597,7 @@
       </c>
       <c r="U13" s="12" t="n">
         <f aca="false">S13-SUM($E$5:E13)-(1+Premissas!$B$17)*SUM($C$5:C13)</f>
-        <v>-861.33752474</v>
+        <v>-783.0341134</v>
       </c>
       <c r="V13" s="12" t="n">
         <f aca="false">(G13+H13)*Premissas!$B$21</f>
@@ -4609,19 +4609,19 @@
       </c>
       <c r="X13" s="12" t="n">
         <f aca="false">X12-Y12+C13*(1+Premissas!$B$17)</f>
-        <v>62.6065</v>
+        <v>56.915</v>
       </c>
       <c r="Y13" s="12" t="n">
         <f aca="false">IF(OR(X13&gt;=Premissas!$B$13,B13=DATE(YEAR(B13),MONTH(B13)+1,0)),X13,0)</f>
-        <v>62.6065</v>
+        <v>56.915</v>
       </c>
       <c r="Z13" s="12" t="n">
         <f aca="false">Z12-AA12+C13/Premissas!$B$18*Premissas!$B$20</f>
-        <v>9.9</v>
+        <v>9</v>
       </c>
       <c r="AA13" s="12" t="n">
         <f aca="false">IF(OR(Z13&gt;=Premissas!$B$14,B13=DATE(YEAR(B13),MONTH(B13)+1,0)),Z13,0)</f>
-        <v>9.9</v>
+        <v>9</v>
       </c>
       <c r="AB13" s="15" t="n">
         <f aca="false">IF(AA13&gt;0,IF(DAY(B13)&lt;=Premissas!$B$12,DATE(YEAR(B13),MONTH(B13),Premissas!$B$16),DATE(YEAR(B13),MONTH(B13)+1,Premissas!$B$16))-Premissas!$B$11+1-Premissas!$B$15,0)</f>
@@ -4638,7 +4638,7 @@
       </c>
       <c r="C14" s="12" t="n">
         <f aca="false">IF(A14&lt;=Premissas!$B$7,Premissas!$B$6/Premissas!$B$7,IF(A14&lt;=Premissas!$B$7+Premissas!$B$8,0,IF(A14&lt;=Premissas!$B$7+Premissas!$B$8+Premissas!$B$10,Premissas!$B$9/Premissas!$B$10,0)))</f>
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="D14" s="15" t="n">
         <f aca="false">IF(Y14&gt;0,IF(DAY(B14)&lt;=Premissas!$B$12,DATE(YEAR(B14),MONTH(B14),Premissas!$B$16),DATE(YEAR(B14),MONTH(B14)+1,Premissas!$B$16))-Premissas!$B$11+1-Premissas!$B$15,0)</f>
@@ -4654,11 +4654,11 @@
       </c>
       <c r="G14" s="29" t="n">
         <f aca="false">C14/Premissas!$B$18*Premissas!$B$19*Premissas!$B$23</f>
-        <v>2.56666666666667</v>
+        <v>2.33333333333333</v>
       </c>
       <c r="H14" s="29" t="n">
         <f aca="false">C14/Premissas!$B$18*Premissas!$B$19*Premissas!$B$24</f>
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="I14" s="12" t="n">
         <f aca="false">-IF($A14-(Premissas!$B$60)&gt;=1,INDEX($G$5:$G$94,$A14-(Premissas!$B$60)),0)*(Premissas!$B$59*Unitário!$B$22+(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25))</f>
@@ -4670,7 +4670,7 @@
       </c>
       <c r="K14" s="12" t="n">
         <f aca="false">IF($A14-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($G$5:$G$94,$A14-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(Premissas!$B$59*Unitário!$B$22+(1-Premissas!$B$62)*(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25)-Premissas!$B$62*((1-Premissas!$B$61)*Unitário!$B$24+(1-Premissas!$B$63)*Unitário!$B$25)-Premissas!$B$41)</f>
-        <v>-5.13333333333333</v>
+        <v>-4.66666666666667</v>
       </c>
       <c r="L14" s="12" t="n">
         <f aca="false">IF($A14-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A14-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*(Premissas!$B$51-(1-Premissas!$B$61)*Unitário!$B$24-(1-Premissas!$B$63)*Unitário!$B$25-(1-Premissas!$B$59)*Unitário!$B$22)</f>
@@ -4678,7 +4678,7 @@
       </c>
       <c r="M14" s="12" t="n">
         <f aca="false">IF($A14-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A14-(Premissas!$B$56)),0)*(Premissas!$B$52-Unitário!$B$27)</f>
-        <v>124.21226015</v>
+        <v>112.9202365</v>
       </c>
       <c r="N14" s="12" t="n">
         <f aca="false">-IF($A14-(Premissas!$B$60)&gt;=1,INDEX($H$5:$H$94,$A14-(Premissas!$B$60)),0)*(Premissas!$B$59*Unitário!$B$22+Premissas!$B$31)</f>
@@ -4686,7 +4686,7 @@
       </c>
       <c r="O14" s="12" t="n">
         <f aca="false">IF($A14-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($H$5:$H$94,$A14-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(-Premissas!$B$52-Premissas!$B$41+(1-Premissas!$B$62)*Premissas!$B$31+Premissas!$B$59*Unitário!$B$22)</f>
-        <v>-15.0601</v>
+        <v>-13.691</v>
       </c>
       <c r="P14" s="12" t="n">
         <f aca="false">-Premissas!$B$42*(IF($A14-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A14-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*Premissas!$B$51+IF($A14-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A14-(Premissas!$B$56)),0)*(1-Premissas!$B$27)*Premissas!$B$52)</f>
@@ -4698,11 +4698,11 @@
       </c>
       <c r="R14" s="12" t="n">
         <f aca="false">E14+F14+SUM(I14:Q14)</f>
-        <v>104.018826816667</v>
+        <v>94.5625698333334</v>
       </c>
       <c r="S14" s="12" t="n">
         <f aca="false">S13+R14</f>
-        <v>-319.073197923333</v>
+        <v>-290.066543566667</v>
       </c>
       <c r="T14" s="15" t="n">
         <f aca="false">IF(AND($A14&gt;$B$100,S14&gt;=0),1,0)</f>
@@ -4710,11 +4710,11 @@
       </c>
       <c r="U14" s="12" t="n">
         <f aca="false">S14-SUM($E$5:E14)-(1+Premissas!$B$17)*SUM($C$5:C14)</f>
-        <v>-819.925197923333</v>
+        <v>-745.386543566667</v>
       </c>
       <c r="V14" s="12" t="n">
         <f aca="false">(G14+H14)*Premissas!$B$21</f>
-        <v>0.146666666666667</v>
+        <v>0.133333333333333</v>
       </c>
       <c r="W14" s="15" t="n">
         <f aca="false">IF(V14&gt;0,DATE(YEAR(B14),MONTH(B14)+1,Premissas!$B$16)-Premissas!$B$11+1-Premissas!$B$15,0)</f>
@@ -4722,7 +4722,7 @@
       </c>
       <c r="X14" s="12" t="n">
         <f aca="false">X13-Y13+C14*(1+Premissas!$B$17)</f>
-        <v>62.6065</v>
+        <v>56.915</v>
       </c>
       <c r="Y14" s="12" t="n">
         <f aca="false">IF(OR(X14&gt;=Premissas!$B$13,B14=DATE(YEAR(B14),MONTH(B14)+1,0)),X14,0)</f>
@@ -4730,7 +4730,7 @@
       </c>
       <c r="Z14" s="12" t="n">
         <f aca="false">Z13-AA13+C14/Premissas!$B$18*Premissas!$B$20</f>
-        <v>9.9</v>
+        <v>9</v>
       </c>
       <c r="AA14" s="12" t="n">
         <f aca="false">IF(OR(Z14&gt;=Premissas!$B$14,B14=DATE(YEAR(B14),MONTH(B14)+1,0)),Z14,0)</f>
@@ -4751,7 +4751,7 @@
       </c>
       <c r="C15" s="12" t="n">
         <f aca="false">IF(A15&lt;=Premissas!$B$7,Premissas!$B$6/Premissas!$B$7,IF(A15&lt;=Premissas!$B$7+Premissas!$B$8,0,IF(A15&lt;=Premissas!$B$7+Premissas!$B$8+Premissas!$B$10,Premissas!$B$9/Premissas!$B$10,0)))</f>
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="D15" s="15" t="n">
         <f aca="false">IF(Y15&gt;0,IF(DAY(B15)&lt;=Premissas!$B$12,DATE(YEAR(B15),MONTH(B15),Premissas!$B$16),DATE(YEAR(B15),MONTH(B15)+1,Premissas!$B$16))-Premissas!$B$11+1-Premissas!$B$15,0)</f>
@@ -4767,15 +4767,15 @@
       </c>
       <c r="G15" s="29" t="n">
         <f aca="false">C15/Premissas!$B$18*Premissas!$B$19*Premissas!$B$23</f>
-        <v>2.56666666666667</v>
+        <v>2.33333333333333</v>
       </c>
       <c r="H15" s="29" t="n">
         <f aca="false">C15/Premissas!$B$18*Premissas!$B$19*Premissas!$B$24</f>
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="I15" s="12" t="n">
         <f aca="false">-IF($A15-(Premissas!$B$60)&gt;=1,INDEX($G$5:$G$94,$A15-(Premissas!$B$60)),0)*(Premissas!$B$59*Unitário!$B$22+(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25))</f>
-        <v>-170.837359</v>
+        <v>-155.30669</v>
       </c>
       <c r="J15" s="12" t="n">
         <f aca="false">IF($A15-(Premissas!$B$54)&gt;=1,INDEX($G$5:$G$94,$A15-(Premissas!$B$54)),0)*Premissas!$B$26*((Premissas!$B$59*Unitário!$B$22+(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25))-Premissas!$B$39)</f>
@@ -4783,7 +4783,7 @@
       </c>
       <c r="K15" s="12" t="n">
         <f aca="false">IF($A15-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($G$5:$G$94,$A15-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(Premissas!$B$59*Unitário!$B$22+(1-Premissas!$B$62)*(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25)-Premissas!$B$62*((1-Premissas!$B$61)*Unitário!$B$24+(1-Premissas!$B$63)*Unitário!$B$25)-Premissas!$B$41)</f>
-        <v>-5.13333333333333</v>
+        <v>-4.66666666666667</v>
       </c>
       <c r="L15" s="12" t="n">
         <f aca="false">IF($A15-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A15-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*(Premissas!$B$51-(1-Premissas!$B$61)*Unitário!$B$24-(1-Premissas!$B$63)*Unitário!$B$25-(1-Premissas!$B$59)*Unitário!$B$22)</f>
@@ -4791,15 +4791,15 @@
       </c>
       <c r="M15" s="12" t="n">
         <f aca="false">IF($A15-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A15-(Premissas!$B$56)),0)*(Premissas!$B$52-Unitário!$B$27)</f>
-        <v>124.21226015</v>
+        <v>112.9202365</v>
       </c>
       <c r="N15" s="12" t="n">
         <f aca="false">-IF($A15-(Premissas!$B$60)&gt;=1,INDEX($H$5:$H$94,$A15-(Premissas!$B$60)),0)*(Premissas!$B$59*Unitário!$B$22+Premissas!$B$31)</f>
-        <v>-38.5</v>
+        <v>-35</v>
       </c>
       <c r="O15" s="12" t="n">
         <f aca="false">IF($A15-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($H$5:$H$94,$A15-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(-Premissas!$B$52-Premissas!$B$41+(1-Premissas!$B$62)*Premissas!$B$31+Premissas!$B$59*Unitário!$B$22)</f>
-        <v>-15.0601</v>
+        <v>-13.691</v>
       </c>
       <c r="P15" s="12" t="n">
         <f aca="false">-Premissas!$B$42*(IF($A15-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A15-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*Premissas!$B$51+IF($A15-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A15-(Premissas!$B$56)),0)*(1-Premissas!$B$27)*Premissas!$B$52)</f>
@@ -4811,11 +4811,11 @@
       </c>
       <c r="R15" s="12" t="n">
         <f aca="false">E15+F15+SUM(I15:Q15)</f>
-        <v>-105.318532183333</v>
+        <v>-95.7441201666667</v>
       </c>
       <c r="S15" s="12" t="n">
         <f aca="false">S14+R15</f>
-        <v>-424.391730106667</v>
+        <v>-385.810663733333</v>
       </c>
       <c r="T15" s="15" t="n">
         <f aca="false">IF(AND($A15&gt;$B$100,S15&gt;=0),1,0)</f>
@@ -4823,11 +4823,11 @@
       </c>
       <c r="U15" s="12" t="n">
         <f aca="false">S15-SUM($E$5:E15)-(1+Premissas!$B$17)*SUM($C$5:C15)</f>
-        <v>-987.850230106667</v>
+        <v>-898.045663733333</v>
       </c>
       <c r="V15" s="12" t="n">
         <f aca="false">(G15+H15)*Premissas!$B$21</f>
-        <v>0.146666666666667</v>
+        <v>0.133333333333333</v>
       </c>
       <c r="W15" s="15" t="n">
         <f aca="false">IF(V15&gt;0,DATE(YEAR(B15),MONTH(B15)+1,Premissas!$B$16)-Premissas!$B$11+1-Premissas!$B$15,0)</f>
@@ -4835,15 +4835,15 @@
       </c>
       <c r="X15" s="12" t="n">
         <f aca="false">X14-Y14+C15*(1+Premissas!$B$17)</f>
-        <v>125.213</v>
+        <v>113.83</v>
       </c>
       <c r="Y15" s="12" t="n">
         <f aca="false">IF(OR(X15&gt;=Premissas!$B$13,B15=DATE(YEAR(B15),MONTH(B15)+1,0)),X15,0)</f>
-        <v>125.213</v>
+        <v>113.83</v>
       </c>
       <c r="Z15" s="12" t="n">
         <f aca="false">Z14-AA14+C15/Premissas!$B$18*Premissas!$B$20</f>
-        <v>19.8</v>
+        <v>18</v>
       </c>
       <c r="AA15" s="12" t="n">
         <f aca="false">IF(OR(Z15&gt;=Premissas!$B$14,B15=DATE(YEAR(B15),MONTH(B15)+1,0)),Z15,0)</f>
@@ -4864,7 +4864,7 @@
       </c>
       <c r="C16" s="12" t="n">
         <f aca="false">IF(A16&lt;=Premissas!$B$7,Premissas!$B$6/Premissas!$B$7,IF(A16&lt;=Premissas!$B$7+Premissas!$B$8,0,IF(A16&lt;=Premissas!$B$7+Premissas!$B$8+Premissas!$B$10,Premissas!$B$9/Premissas!$B$10,0)))</f>
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="D16" s="15" t="n">
         <f aca="false">IF(Y16&gt;0,IF(DAY(B16)&lt;=Premissas!$B$12,DATE(YEAR(B16),MONTH(B16),Premissas!$B$16),DATE(YEAR(B16),MONTH(B16)+1,Premissas!$B$16))-Premissas!$B$11+1-Premissas!$B$15,0)</f>
@@ -4880,23 +4880,23 @@
       </c>
       <c r="G16" s="29" t="n">
         <f aca="false">C16/Premissas!$B$18*Premissas!$B$19*Premissas!$B$23</f>
-        <v>2.56666666666667</v>
+        <v>2.33333333333333</v>
       </c>
       <c r="H16" s="29" t="n">
         <f aca="false">C16/Premissas!$B$18*Premissas!$B$19*Premissas!$B$24</f>
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="I16" s="12" t="n">
         <f aca="false">-IF($A16-(Premissas!$B$60)&gt;=1,INDEX($G$5:$G$94,$A16-(Premissas!$B$60)),0)*(Premissas!$B$59*Unitário!$B$22+(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25))</f>
-        <v>-170.837359</v>
+        <v>-155.30669</v>
       </c>
       <c r="J16" s="12" t="n">
         <f aca="false">IF($A16-(Premissas!$B$54)&gt;=1,INDEX($G$5:$G$94,$A16-(Premissas!$B$54)),0)*Premissas!$B$26*((Premissas!$B$59*Unitário!$B$22+(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25))-Premissas!$B$39)</f>
-        <v>24.68338103</v>
+        <v>22.4394373</v>
       </c>
       <c r="K16" s="12" t="n">
         <f aca="false">IF($A16-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($G$5:$G$94,$A16-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(Premissas!$B$59*Unitário!$B$22+(1-Premissas!$B$62)*(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25)-Premissas!$B$62*((1-Premissas!$B$61)*Unitário!$B$24+(1-Premissas!$B$63)*Unitário!$B$25)-Premissas!$B$41)</f>
-        <v>-5.13333333333333</v>
+        <v>-4.66666666666667</v>
       </c>
       <c r="L16" s="12" t="n">
         <f aca="false">IF($A16-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A16-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*(Premissas!$B$51-(1-Premissas!$B$61)*Unitário!$B$24-(1-Premissas!$B$63)*Unitário!$B$25-(1-Premissas!$B$59)*Unitário!$B$22)</f>
@@ -4904,15 +4904,15 @@
       </c>
       <c r="M16" s="12" t="n">
         <f aca="false">IF($A16-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A16-(Premissas!$B$56)),0)*(Premissas!$B$52-Unitário!$B$27)</f>
-        <v>124.21226015</v>
+        <v>112.9202365</v>
       </c>
       <c r="N16" s="12" t="n">
         <f aca="false">-IF($A16-(Premissas!$B$60)&gt;=1,INDEX($H$5:$H$94,$A16-(Premissas!$B$60)),0)*(Premissas!$B$59*Unitário!$B$22+Premissas!$B$31)</f>
-        <v>-38.5</v>
+        <v>-35</v>
       </c>
       <c r="O16" s="12" t="n">
         <f aca="false">IF($A16-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($H$5:$H$94,$A16-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(-Premissas!$B$52-Premissas!$B$41+(1-Premissas!$B$62)*Premissas!$B$31+Premissas!$B$59*Unitário!$B$22)</f>
-        <v>-15.0601</v>
+        <v>-13.691</v>
       </c>
       <c r="P16" s="12" t="n">
         <f aca="false">-Premissas!$B$42*(IF($A16-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A16-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*Premissas!$B$51+IF($A16-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A16-(Premissas!$B$56)),0)*(1-Premissas!$B$27)*Premissas!$B$52)</f>
@@ -4924,11 +4924,11 @@
       </c>
       <c r="R16" s="12" t="n">
         <f aca="false">E16+F16+SUM(I16:Q16)</f>
-        <v>-80.6351511533333</v>
+        <v>-73.3046828666667</v>
       </c>
       <c r="S16" s="12" t="n">
         <f aca="false">S15+R16</f>
-        <v>-505.02688126</v>
+        <v>-459.1153466</v>
       </c>
       <c r="T16" s="15" t="n">
         <f aca="false">IF(AND($A16&gt;$B$100,S16&gt;=0),1,0)</f>
@@ -4936,11 +4936,11 @@
       </c>
       <c r="U16" s="12" t="n">
         <f aca="false">S16-SUM($E$5:E16)-(1+Premissas!$B$17)*SUM($C$5:C16)</f>
-        <v>-1131.09188126</v>
+        <v>-1028.2653466</v>
       </c>
       <c r="V16" s="12" t="n">
         <f aca="false">(G16+H16)*Premissas!$B$21</f>
-        <v>0.146666666666667</v>
+        <v>0.133333333333333</v>
       </c>
       <c r="W16" s="15" t="n">
         <f aca="false">IF(V16&gt;0,DATE(YEAR(B16),MONTH(B16)+1,Premissas!$B$16)-Premissas!$B$11+1-Premissas!$B$15,0)</f>
@@ -4948,7 +4948,7 @@
       </c>
       <c r="X16" s="12" t="n">
         <f aca="false">X15-Y15+C16*(1+Premissas!$B$17)</f>
-        <v>62.6065</v>
+        <v>56.915</v>
       </c>
       <c r="Y16" s="12" t="n">
         <f aca="false">IF(OR(X16&gt;=Premissas!$B$13,B16=DATE(YEAR(B16),MONTH(B16)+1,0)),X16,0)</f>
@@ -4956,11 +4956,11 @@
       </c>
       <c r="Z16" s="12" t="n">
         <f aca="false">Z15-AA15+C16/Premissas!$B$18*Premissas!$B$20</f>
-        <v>29.7</v>
+        <v>27</v>
       </c>
       <c r="AA16" s="12" t="n">
         <f aca="false">IF(OR(Z16&gt;=Premissas!$B$14,B16=DATE(YEAR(B16),MONTH(B16)+1,0)),Z16,0)</f>
-        <v>29.7</v>
+        <v>27</v>
       </c>
       <c r="AB16" s="15" t="n">
         <f aca="false">IF(AA16&gt;0,IF(DAY(B16)&lt;=Premissas!$B$12,DATE(YEAR(B16),MONTH(B16),Premissas!$B$16),DATE(YEAR(B16),MONTH(B16)+1,Premissas!$B$16))-Premissas!$B$11+1-Premissas!$B$15,0)</f>
@@ -4977,7 +4977,7 @@
       </c>
       <c r="C17" s="12" t="n">
         <f aca="false">IF(A17&lt;=Premissas!$B$7,Premissas!$B$6/Premissas!$B$7,IF(A17&lt;=Premissas!$B$7+Premissas!$B$8,0,IF(A17&lt;=Premissas!$B$7+Premissas!$B$8+Premissas!$B$10,Premissas!$B$9/Premissas!$B$10,0)))</f>
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="D17" s="15" t="n">
         <f aca="false">IF(Y17&gt;0,IF(DAY(B17)&lt;=Premissas!$B$12,DATE(YEAR(B17),MONTH(B17),Premissas!$B$16),DATE(YEAR(B17),MONTH(B17)+1,Premissas!$B$16))-Premissas!$B$11+1-Premissas!$B$15,0)</f>
@@ -4993,23 +4993,23 @@
       </c>
       <c r="G17" s="29" t="n">
         <f aca="false">C17/Premissas!$B$18*Premissas!$B$19*Premissas!$B$23</f>
-        <v>2.56666666666667</v>
+        <v>2.33333333333333</v>
       </c>
       <c r="H17" s="29" t="n">
         <f aca="false">C17/Premissas!$B$18*Premissas!$B$19*Premissas!$B$24</f>
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="I17" s="12" t="n">
         <f aca="false">-IF($A17-(Premissas!$B$60)&gt;=1,INDEX($G$5:$G$94,$A17-(Premissas!$B$60)),0)*(Premissas!$B$59*Unitário!$B$22+(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25))</f>
-        <v>-170.837359</v>
+        <v>-155.30669</v>
       </c>
       <c r="J17" s="12" t="n">
         <f aca="false">IF($A17-(Premissas!$B$54)&gt;=1,INDEX($G$5:$G$94,$A17-(Premissas!$B$54)),0)*Premissas!$B$26*((Premissas!$B$59*Unitário!$B$22+(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25))-Premissas!$B$39)</f>
-        <v>24.68338103</v>
+        <v>22.4394373</v>
       </c>
       <c r="K17" s="12" t="n">
         <f aca="false">IF($A17-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($G$5:$G$94,$A17-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(Premissas!$B$59*Unitário!$B$22+(1-Premissas!$B$62)*(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25)-Premissas!$B$62*((1-Premissas!$B$61)*Unitário!$B$24+(1-Premissas!$B$63)*Unitário!$B$25)-Premissas!$B$41)</f>
-        <v>-5.13333333333333</v>
+        <v>-4.66666666666667</v>
       </c>
       <c r="L17" s="12" t="n">
         <f aca="false">IF($A17-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A17-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*(Premissas!$B$51-(1-Premissas!$B$61)*Unitário!$B$24-(1-Premissas!$B$63)*Unitário!$B$25-(1-Premissas!$B$59)*Unitário!$B$22)</f>
@@ -5017,15 +5017,15 @@
       </c>
       <c r="M17" s="12" t="n">
         <f aca="false">IF($A17-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A17-(Premissas!$B$56)),0)*(Premissas!$B$52-Unitário!$B$27)</f>
-        <v>124.21226015</v>
+        <v>112.9202365</v>
       </c>
       <c r="N17" s="12" t="n">
         <f aca="false">-IF($A17-(Premissas!$B$60)&gt;=1,INDEX($H$5:$H$94,$A17-(Premissas!$B$60)),0)*(Premissas!$B$59*Unitário!$B$22+Premissas!$B$31)</f>
-        <v>-38.5</v>
+        <v>-35</v>
       </c>
       <c r="O17" s="12" t="n">
         <f aca="false">IF($A17-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($H$5:$H$94,$A17-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(-Premissas!$B$52-Premissas!$B$41+(1-Premissas!$B$62)*Premissas!$B$31+Premissas!$B$59*Unitário!$B$22)</f>
-        <v>-15.0601</v>
+        <v>-13.691</v>
       </c>
       <c r="P17" s="12" t="n">
         <f aca="false">-Premissas!$B$42*(IF($A17-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A17-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*Premissas!$B$51+IF($A17-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A17-(Premissas!$B$56)),0)*(1-Premissas!$B$27)*Premissas!$B$52)</f>
@@ -5037,11 +5037,11 @@
       </c>
       <c r="R17" s="12" t="n">
         <f aca="false">E17+F17+SUM(I17:Q17)</f>
-        <v>-80.6351511533333</v>
+        <v>-73.3046828666667</v>
       </c>
       <c r="S17" s="12" t="n">
         <f aca="false">S16+R17</f>
-        <v>-585.662032413333</v>
+        <v>-532.420029466667</v>
       </c>
       <c r="T17" s="15" t="n">
         <f aca="false">IF(AND($A17&gt;$B$100,S17&gt;=0),1,0)</f>
@@ -5049,11 +5049,11 @@
       </c>
       <c r="U17" s="12" t="n">
         <f aca="false">S17-SUM($E$5:E17)-(1+Premissas!$B$17)*SUM($C$5:C17)</f>
-        <v>-1274.33353241333</v>
+        <v>-1158.48502946667</v>
       </c>
       <c r="V17" s="12" t="n">
         <f aca="false">(G17+H17)*Premissas!$B$21</f>
-        <v>0.146666666666667</v>
+        <v>0.133333333333333</v>
       </c>
       <c r="W17" s="15" t="n">
         <f aca="false">IF(V17&gt;0,DATE(YEAR(B17),MONTH(B17)+1,Premissas!$B$16)-Premissas!$B$11+1-Premissas!$B$15,0)</f>
@@ -5061,15 +5061,15 @@
       </c>
       <c r="X17" s="12" t="n">
         <f aca="false">X16-Y16+C17*(1+Premissas!$B$17)</f>
-        <v>125.213</v>
+        <v>113.83</v>
       </c>
       <c r="Y17" s="12" t="n">
         <f aca="false">IF(OR(X17&gt;=Premissas!$B$13,B17=DATE(YEAR(B17),MONTH(B17)+1,0)),X17,0)</f>
-        <v>125.213</v>
+        <v>113.83</v>
       </c>
       <c r="Z17" s="12" t="n">
         <f aca="false">Z16-AA16+C17/Premissas!$B$18*Premissas!$B$20</f>
-        <v>9.9</v>
+        <v>9</v>
       </c>
       <c r="AA17" s="12" t="n">
         <f aca="false">IF(OR(Z17&gt;=Premissas!$B$14,B17=DATE(YEAR(B17),MONTH(B17)+1,0)),Z17,0)</f>
@@ -5090,7 +5090,7 @@
       </c>
       <c r="C18" s="12" t="n">
         <f aca="false">IF(A18&lt;=Premissas!$B$7,Premissas!$B$6/Premissas!$B$7,IF(A18&lt;=Premissas!$B$7+Premissas!$B$8,0,IF(A18&lt;=Premissas!$B$7+Premissas!$B$8+Premissas!$B$10,Premissas!$B$9/Premissas!$B$10,0)))</f>
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="D18" s="15" t="n">
         <f aca="false">IF(Y18&gt;0,IF(DAY(B18)&lt;=Premissas!$B$12,DATE(YEAR(B18),MONTH(B18),Premissas!$B$16),DATE(YEAR(B18),MONTH(B18)+1,Premissas!$B$16))-Premissas!$B$11+1-Premissas!$B$15,0)</f>
@@ -5106,23 +5106,23 @@
       </c>
       <c r="G18" s="29" t="n">
         <f aca="false">C18/Premissas!$B$18*Premissas!$B$19*Premissas!$B$23</f>
-        <v>2.56666666666667</v>
+        <v>2.33333333333333</v>
       </c>
       <c r="H18" s="29" t="n">
         <f aca="false">C18/Premissas!$B$18*Premissas!$B$19*Premissas!$B$24</f>
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="I18" s="12" t="n">
         <f aca="false">-IF($A18-(Premissas!$B$60)&gt;=1,INDEX($G$5:$G$94,$A18-(Premissas!$B$60)),0)*(Premissas!$B$59*Unitário!$B$22+(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25))</f>
-        <v>-170.837359</v>
+        <v>-155.30669</v>
       </c>
       <c r="J18" s="12" t="n">
         <f aca="false">IF($A18-(Premissas!$B$54)&gt;=1,INDEX($G$5:$G$94,$A18-(Premissas!$B$54)),0)*Premissas!$B$26*((Premissas!$B$59*Unitário!$B$22+(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25))-Premissas!$B$39)</f>
-        <v>24.68338103</v>
+        <v>22.4394373</v>
       </c>
       <c r="K18" s="12" t="n">
         <f aca="false">IF($A18-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($G$5:$G$94,$A18-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(Premissas!$B$59*Unitário!$B$22+(1-Premissas!$B$62)*(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25)-Premissas!$B$62*((1-Premissas!$B$61)*Unitário!$B$24+(1-Premissas!$B$63)*Unitário!$B$25)-Premissas!$B$41)</f>
-        <v>-5.13333333333333</v>
+        <v>-4.66666666666667</v>
       </c>
       <c r="L18" s="12" t="n">
         <f aca="false">IF($A18-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A18-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*(Premissas!$B$51-(1-Premissas!$B$61)*Unitário!$B$24-(1-Premissas!$B$63)*Unitário!$B$25-(1-Premissas!$B$59)*Unitário!$B$22)</f>
@@ -5130,15 +5130,15 @@
       </c>
       <c r="M18" s="12" t="n">
         <f aca="false">IF($A18-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A18-(Premissas!$B$56)),0)*(Premissas!$B$52-Unitário!$B$27)</f>
-        <v>124.21226015</v>
+        <v>112.9202365</v>
       </c>
       <c r="N18" s="12" t="n">
         <f aca="false">-IF($A18-(Premissas!$B$60)&gt;=1,INDEX($H$5:$H$94,$A18-(Premissas!$B$60)),0)*(Premissas!$B$59*Unitário!$B$22+Premissas!$B$31)</f>
-        <v>-38.5</v>
+        <v>-35</v>
       </c>
       <c r="O18" s="12" t="n">
         <f aca="false">IF($A18-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($H$5:$H$94,$A18-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(-Premissas!$B$52-Premissas!$B$41+(1-Premissas!$B$62)*Premissas!$B$31+Premissas!$B$59*Unitário!$B$22)</f>
-        <v>-15.0601</v>
+        <v>-13.691</v>
       </c>
       <c r="P18" s="12" t="n">
         <f aca="false">-Premissas!$B$42*(IF($A18-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A18-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*Premissas!$B$51+IF($A18-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A18-(Premissas!$B$56)),0)*(1-Premissas!$B$27)*Premissas!$B$52)</f>
@@ -5150,11 +5150,11 @@
       </c>
       <c r="R18" s="12" t="n">
         <f aca="false">E18+F18+SUM(I18:Q18)</f>
-        <v>-80.6351511533333</v>
+        <v>-73.3046828666667</v>
       </c>
       <c r="S18" s="12" t="n">
         <f aca="false">S17+R18</f>
-        <v>-666.297183566667</v>
+        <v>-605.724712333333</v>
       </c>
       <c r="T18" s="15" t="n">
         <f aca="false">IF(AND($A18&gt;$B$100,S18&gt;=0),1,0)</f>
@@ -5162,11 +5162,11 @@
       </c>
       <c r="U18" s="12" t="n">
         <f aca="false">S18-SUM($E$5:E18)-(1+Premissas!$B$17)*SUM($C$5:C18)</f>
-        <v>-1417.57518356667</v>
+        <v>-1288.70471233333</v>
       </c>
       <c r="V18" s="12" t="n">
         <f aca="false">(G18+H18)*Premissas!$B$21</f>
-        <v>0.146666666666667</v>
+        <v>0.133333333333333</v>
       </c>
       <c r="W18" s="15" t="n">
         <f aca="false">IF(V18&gt;0,DATE(YEAR(B18),MONTH(B18)+1,Premissas!$B$16)-Premissas!$B$11+1-Premissas!$B$15,0)</f>
@@ -5174,7 +5174,7 @@
       </c>
       <c r="X18" s="12" t="n">
         <f aca="false">X17-Y17+C18*(1+Premissas!$B$17)</f>
-        <v>62.6065</v>
+        <v>56.915</v>
       </c>
       <c r="Y18" s="12" t="n">
         <f aca="false">IF(OR(X18&gt;=Premissas!$B$13,B18=DATE(YEAR(B18),MONTH(B18)+1,0)),X18,0)</f>
@@ -5182,7 +5182,7 @@
       </c>
       <c r="Z18" s="12" t="n">
         <f aca="false">Z17-AA17+C18/Premissas!$B$18*Premissas!$B$20</f>
-        <v>19.8</v>
+        <v>18</v>
       </c>
       <c r="AA18" s="12" t="n">
         <f aca="false">IF(OR(Z18&gt;=Premissas!$B$14,B18=DATE(YEAR(B18),MONTH(B18)+1,0)),Z18,0)</f>
@@ -5203,7 +5203,7 @@
       </c>
       <c r="C19" s="12" t="n">
         <f aca="false">IF(A19&lt;=Premissas!$B$7,Premissas!$B$6/Premissas!$B$7,IF(A19&lt;=Premissas!$B$7+Premissas!$B$8,0,IF(A19&lt;=Premissas!$B$7+Premissas!$B$8+Premissas!$B$10,Premissas!$B$9/Premissas!$B$10,0)))</f>
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="D19" s="15" t="n">
         <f aca="false">IF(Y19&gt;0,IF(DAY(B19)&lt;=Premissas!$B$12,DATE(YEAR(B19),MONTH(B19),Premissas!$B$16),DATE(YEAR(B19),MONTH(B19)+1,Premissas!$B$16))-Premissas!$B$11+1-Premissas!$B$15,0)</f>
@@ -5219,23 +5219,23 @@
       </c>
       <c r="G19" s="29" t="n">
         <f aca="false">C19/Premissas!$B$18*Premissas!$B$19*Premissas!$B$23</f>
-        <v>2.56666666666667</v>
+        <v>2.33333333333333</v>
       </c>
       <c r="H19" s="29" t="n">
         <f aca="false">C19/Premissas!$B$18*Premissas!$B$19*Premissas!$B$24</f>
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="I19" s="12" t="n">
         <f aca="false">-IF($A19-(Premissas!$B$60)&gt;=1,INDEX($G$5:$G$94,$A19-(Premissas!$B$60)),0)*(Premissas!$B$59*Unitário!$B$22+(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25))</f>
-        <v>-170.837359</v>
+        <v>-155.30669</v>
       </c>
       <c r="J19" s="12" t="n">
         <f aca="false">IF($A19-(Premissas!$B$54)&gt;=1,INDEX($G$5:$G$94,$A19-(Premissas!$B$54)),0)*Premissas!$B$26*((Premissas!$B$59*Unitário!$B$22+(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25))-Premissas!$B$39)</f>
-        <v>24.68338103</v>
+        <v>22.4394373</v>
       </c>
       <c r="K19" s="12" t="n">
         <f aca="false">IF($A19-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($G$5:$G$94,$A19-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(Premissas!$B$59*Unitário!$B$22+(1-Premissas!$B$62)*(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25)-Premissas!$B$62*((1-Premissas!$B$61)*Unitário!$B$24+(1-Premissas!$B$63)*Unitário!$B$25)-Premissas!$B$41)</f>
-        <v>-5.13333333333333</v>
+        <v>-4.66666666666667</v>
       </c>
       <c r="L19" s="12" t="n">
         <f aca="false">IF($A19-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A19-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*(Premissas!$B$51-(1-Premissas!$B$61)*Unitário!$B$24-(1-Premissas!$B$63)*Unitário!$B$25-(1-Premissas!$B$59)*Unitário!$B$22)</f>
@@ -5243,15 +5243,15 @@
       </c>
       <c r="M19" s="12" t="n">
         <f aca="false">IF($A19-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A19-(Premissas!$B$56)),0)*(Premissas!$B$52-Unitário!$B$27)</f>
-        <v>124.21226015</v>
+        <v>112.9202365</v>
       </c>
       <c r="N19" s="12" t="n">
         <f aca="false">-IF($A19-(Premissas!$B$60)&gt;=1,INDEX($H$5:$H$94,$A19-(Premissas!$B$60)),0)*(Premissas!$B$59*Unitário!$B$22+Premissas!$B$31)</f>
-        <v>-38.5</v>
+        <v>-35</v>
       </c>
       <c r="O19" s="12" t="n">
         <f aca="false">IF($A19-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($H$5:$H$94,$A19-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(-Premissas!$B$52-Premissas!$B$41+(1-Premissas!$B$62)*Premissas!$B$31+Premissas!$B$59*Unitário!$B$22)</f>
-        <v>-15.0601</v>
+        <v>-13.691</v>
       </c>
       <c r="P19" s="12" t="n">
         <f aca="false">-Premissas!$B$42*(IF($A19-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A19-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*Premissas!$B$51+IF($A19-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A19-(Premissas!$B$56)),0)*(1-Premissas!$B$27)*Premissas!$B$52)</f>
@@ -5263,11 +5263,11 @@
       </c>
       <c r="R19" s="12" t="n">
         <f aca="false">E19+F19+SUM(I19:Q19)</f>
-        <v>-80.6351511533333</v>
+        <v>-73.3046828666667</v>
       </c>
       <c r="S19" s="12" t="n">
         <f aca="false">S18+R19</f>
-        <v>-746.93233472</v>
+        <v>-679.0293952</v>
       </c>
       <c r="T19" s="15" t="n">
         <f aca="false">IF(AND($A19&gt;$B$100,S19&gt;=0),1,0)</f>
@@ -5275,11 +5275,11 @@
       </c>
       <c r="U19" s="12" t="n">
         <f aca="false">S19-SUM($E$5:E19)-(1+Premissas!$B$17)*SUM($C$5:C19)</f>
-        <v>-1560.81683472</v>
+        <v>-1418.9243952</v>
       </c>
       <c r="V19" s="12" t="n">
         <f aca="false">(G19+H19)*Premissas!$B$21</f>
-        <v>0.146666666666667</v>
+        <v>0.133333333333333</v>
       </c>
       <c r="W19" s="15" t="n">
         <f aca="false">IF(V19&gt;0,DATE(YEAR(B19),MONTH(B19)+1,Premissas!$B$16)-Premissas!$B$11+1-Premissas!$B$15,0)</f>
@@ -5287,19 +5287,19 @@
       </c>
       <c r="X19" s="12" t="n">
         <f aca="false">X18-Y18+C19*(1+Premissas!$B$17)</f>
-        <v>125.213</v>
+        <v>113.83</v>
       </c>
       <c r="Y19" s="12" t="n">
         <f aca="false">IF(OR(X19&gt;=Premissas!$B$13,B19=DATE(YEAR(B19),MONTH(B19)+1,0)),X19,0)</f>
-        <v>125.213</v>
+        <v>113.83</v>
       </c>
       <c r="Z19" s="12" t="n">
         <f aca="false">Z18-AA18+C19/Premissas!$B$18*Premissas!$B$20</f>
-        <v>29.7</v>
+        <v>27</v>
       </c>
       <c r="AA19" s="12" t="n">
         <f aca="false">IF(OR(Z19&gt;=Premissas!$B$14,B19=DATE(YEAR(B19),MONTH(B19)+1,0)),Z19,0)</f>
-        <v>29.7</v>
+        <v>27</v>
       </c>
       <c r="AB19" s="15" t="n">
         <f aca="false">IF(AA19&gt;0,IF(DAY(B19)&lt;=Premissas!$B$12,DATE(YEAR(B19),MONTH(B19),Premissas!$B$16),DATE(YEAR(B19),MONTH(B19)+1,Premissas!$B$16))-Premissas!$B$11+1-Premissas!$B$15,0)</f>
@@ -5316,7 +5316,7 @@
       </c>
       <c r="C20" s="12" t="n">
         <f aca="false">IF(A20&lt;=Premissas!$B$7,Premissas!$B$6/Premissas!$B$7,IF(A20&lt;=Premissas!$B$7+Premissas!$B$8,0,IF(A20&lt;=Premissas!$B$7+Premissas!$B$8+Premissas!$B$10,Premissas!$B$9/Premissas!$B$10,0)))</f>
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="D20" s="15" t="n">
         <f aca="false">IF(Y20&gt;0,IF(DAY(B20)&lt;=Premissas!$B$12,DATE(YEAR(B20),MONTH(B20),Premissas!$B$16),DATE(YEAR(B20),MONTH(B20)+1,Premissas!$B$16))-Premissas!$B$11+1-Premissas!$B$15,0)</f>
@@ -5332,23 +5332,23 @@
       </c>
       <c r="G20" s="29" t="n">
         <f aca="false">C20/Premissas!$B$18*Premissas!$B$19*Premissas!$B$23</f>
-        <v>2.56666666666667</v>
+        <v>2.33333333333333</v>
       </c>
       <c r="H20" s="29" t="n">
         <f aca="false">C20/Premissas!$B$18*Premissas!$B$19*Premissas!$B$24</f>
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="I20" s="12" t="n">
         <f aca="false">-IF($A20-(Premissas!$B$60)&gt;=1,INDEX($G$5:$G$94,$A20-(Premissas!$B$60)),0)*(Premissas!$B$59*Unitário!$B$22+(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25))</f>
-        <v>-170.837359</v>
+        <v>-155.30669</v>
       </c>
       <c r="J20" s="12" t="n">
         <f aca="false">IF($A20-(Premissas!$B$54)&gt;=1,INDEX($G$5:$G$94,$A20-(Premissas!$B$54)),0)*Premissas!$B$26*((Premissas!$B$59*Unitário!$B$22+(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25))-Premissas!$B$39)</f>
-        <v>24.68338103</v>
+        <v>22.4394373</v>
       </c>
       <c r="K20" s="12" t="n">
         <f aca="false">IF($A20-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($G$5:$G$94,$A20-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(Premissas!$B$59*Unitário!$B$22+(1-Premissas!$B$62)*(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25)-Premissas!$B$62*((1-Premissas!$B$61)*Unitário!$B$24+(1-Premissas!$B$63)*Unitário!$B$25)-Premissas!$B$41)</f>
-        <v>-5.13333333333333</v>
+        <v>-4.66666666666667</v>
       </c>
       <c r="L20" s="12" t="n">
         <f aca="false">IF($A20-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A20-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*(Premissas!$B$51-(1-Premissas!$B$61)*Unitário!$B$24-(1-Premissas!$B$63)*Unitário!$B$25-(1-Premissas!$B$59)*Unitário!$B$22)</f>
@@ -5356,15 +5356,15 @@
       </c>
       <c r="M20" s="12" t="n">
         <f aca="false">IF($A20-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A20-(Premissas!$B$56)),0)*(Premissas!$B$52-Unitário!$B$27)</f>
-        <v>124.21226015</v>
+        <v>112.9202365</v>
       </c>
       <c r="N20" s="12" t="n">
         <f aca="false">-IF($A20-(Premissas!$B$60)&gt;=1,INDEX($H$5:$H$94,$A20-(Premissas!$B$60)),0)*(Premissas!$B$59*Unitário!$B$22+Premissas!$B$31)</f>
-        <v>-38.5</v>
+        <v>-35</v>
       </c>
       <c r="O20" s="12" t="n">
         <f aca="false">IF($A20-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($H$5:$H$94,$A20-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(-Premissas!$B$52-Premissas!$B$41+(1-Premissas!$B$62)*Premissas!$B$31+Premissas!$B$59*Unitário!$B$22)</f>
-        <v>-15.0601</v>
+        <v>-13.691</v>
       </c>
       <c r="P20" s="12" t="n">
         <f aca="false">-Premissas!$B$42*(IF($A20-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A20-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*Premissas!$B$51+IF($A20-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A20-(Premissas!$B$56)),0)*(1-Premissas!$B$27)*Premissas!$B$52)</f>
@@ -5376,11 +5376,11 @@
       </c>
       <c r="R20" s="12" t="n">
         <f aca="false">E20+F20+SUM(I20:Q20)</f>
-        <v>-80.6351511533333</v>
+        <v>-73.3046828666667</v>
       </c>
       <c r="S20" s="12" t="n">
         <f aca="false">S19+R20</f>
-        <v>-827.567485873333</v>
+        <v>-752.334078066667</v>
       </c>
       <c r="T20" s="15" t="n">
         <f aca="false">IF(AND($A20&gt;$B$100,S20&gt;=0),1,0)</f>
@@ -5388,11 +5388,11 @@
       </c>
       <c r="U20" s="12" t="n">
         <f aca="false">S20-SUM($E$5:E20)-(1+Premissas!$B$17)*SUM($C$5:C20)</f>
-        <v>-1704.05848587333</v>
+        <v>-1549.14407806667</v>
       </c>
       <c r="V20" s="12" t="n">
         <f aca="false">(G20+H20)*Premissas!$B$21</f>
-        <v>0.146666666666667</v>
+        <v>0.133333333333333</v>
       </c>
       <c r="W20" s="15" t="n">
         <f aca="false">IF(V20&gt;0,DATE(YEAR(B20),MONTH(B20)+1,Premissas!$B$16)-Premissas!$B$11+1-Premissas!$B$15,0)</f>
@@ -5400,7 +5400,7 @@
       </c>
       <c r="X20" s="12" t="n">
         <f aca="false">X19-Y19+C20*(1+Premissas!$B$17)</f>
-        <v>62.6065</v>
+        <v>56.915</v>
       </c>
       <c r="Y20" s="12" t="n">
         <f aca="false">IF(OR(X20&gt;=Premissas!$B$13,B20=DATE(YEAR(B20),MONTH(B20)+1,0)),X20,0)</f>
@@ -5408,7 +5408,7 @@
       </c>
       <c r="Z20" s="12" t="n">
         <f aca="false">Z19-AA19+C20/Premissas!$B$18*Premissas!$B$20</f>
-        <v>9.9</v>
+        <v>9</v>
       </c>
       <c r="AA20" s="12" t="n">
         <f aca="false">IF(OR(Z20&gt;=Premissas!$B$14,B20=DATE(YEAR(B20),MONTH(B20)+1,0)),Z20,0)</f>
@@ -5453,11 +5453,11 @@
       </c>
       <c r="I21" s="12" t="n">
         <f aca="false">-IF($A21-(Premissas!$B$60)&gt;=1,INDEX($G$5:$G$94,$A21-(Premissas!$B$60)),0)*(Premissas!$B$59*Unitário!$B$22+(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25))</f>
-        <v>-170.837359</v>
+        <v>-155.30669</v>
       </c>
       <c r="J21" s="12" t="n">
         <f aca="false">IF($A21-(Premissas!$B$54)&gt;=1,INDEX($G$5:$G$94,$A21-(Premissas!$B$54)),0)*Premissas!$B$26*((Premissas!$B$59*Unitário!$B$22+(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25))-Premissas!$B$39)</f>
-        <v>24.68338103</v>
+        <v>22.4394373</v>
       </c>
       <c r="K21" s="12" t="n">
         <f aca="false">IF($A21-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($G$5:$G$94,$A21-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(Premissas!$B$59*Unitário!$B$22+(1-Premissas!$B$62)*(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25)-Premissas!$B$62*((1-Premissas!$B$61)*Unitário!$B$24+(1-Premissas!$B$63)*Unitário!$B$25)-Premissas!$B$41)</f>
@@ -5465,7 +5465,7 @@
       </c>
       <c r="L21" s="12" t="n">
         <f aca="false">IF($A21-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A21-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*(Premissas!$B$51-(1-Premissas!$B$61)*Unitário!$B$24-(1-Premissas!$B$63)*Unitário!$B$25-(1-Premissas!$B$59)*Unitário!$B$22)</f>
-        <v>243.3893</v>
+        <v>221.263</v>
       </c>
       <c r="M21" s="12" t="n">
         <f aca="false">IF($A21-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A21-(Premissas!$B$56)),0)*(Premissas!$B$52-Unitário!$B$27)</f>
@@ -5473,7 +5473,7 @@
       </c>
       <c r="N21" s="12" t="n">
         <f aca="false">-IF($A21-(Premissas!$B$60)&gt;=1,INDEX($H$5:$H$94,$A21-(Premissas!$B$60)),0)*(Premissas!$B$59*Unitário!$B$22+Premissas!$B$31)</f>
-        <v>-38.5</v>
+        <v>-35</v>
       </c>
       <c r="O21" s="12" t="n">
         <f aca="false">IF($A21-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($H$5:$H$94,$A21-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(-Premissas!$B$52-Premissas!$B$41+(1-Premissas!$B$62)*Premissas!$B$31+Premissas!$B$59*Unitário!$B$22)</f>
@@ -5489,11 +5489,11 @@
       </c>
       <c r="R21" s="12" t="n">
         <f aca="false">E21+F21+SUM(I21:Q21)</f>
-        <v>58.73532203</v>
+        <v>53.3957473</v>
       </c>
       <c r="S21" s="12" t="n">
         <f aca="false">S20+R21</f>
-        <v>-768.832163843333</v>
+        <v>-698.938330766667</v>
       </c>
       <c r="T21" s="15" t="n">
         <f aca="false">IF(AND($A21&gt;$B$100,S21&gt;=0),1,0)</f>
@@ -5501,7 +5501,7 @@
       </c>
       <c r="U21" s="12" t="n">
         <f aca="false">S21-SUM($E$5:E21)-(1+Premissas!$B$17)*SUM($C$5:C21)</f>
-        <v>-1645.32316384333</v>
+        <v>-1495.74833076667</v>
       </c>
       <c r="V21" s="12" t="n">
         <f aca="false">(G21+H21)*Premissas!$B$21</f>
@@ -5513,7 +5513,7 @@
       </c>
       <c r="X21" s="12" t="n">
         <f aca="false">X20-Y20+C21*(1+Premissas!$B$17)</f>
-        <v>62.6065</v>
+        <v>56.915</v>
       </c>
       <c r="Y21" s="12" t="n">
         <f aca="false">IF(OR(X21&gt;=Premissas!$B$13,B21=DATE(YEAR(B21),MONTH(B21)+1,0)),X21,0)</f>
@@ -5521,7 +5521,7 @@
       </c>
       <c r="Z21" s="12" t="n">
         <f aca="false">Z20-AA20+C21/Premissas!$B$18*Premissas!$B$20</f>
-        <v>9.9</v>
+        <v>9</v>
       </c>
       <c r="AA21" s="12" t="n">
         <f aca="false">IF(OR(Z21&gt;=Premissas!$B$14,B21=DATE(YEAR(B21),MONTH(B21)+1,0)),Z21,0)</f>
@@ -5570,7 +5570,7 @@
       </c>
       <c r="J22" s="12" t="n">
         <f aca="false">IF($A22-(Premissas!$B$54)&gt;=1,INDEX($G$5:$G$94,$A22-(Premissas!$B$54)),0)*Premissas!$B$26*((Premissas!$B$59*Unitário!$B$22+(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25))-Premissas!$B$39)</f>
-        <v>24.68338103</v>
+        <v>22.4394373</v>
       </c>
       <c r="K22" s="12" t="n">
         <f aca="false">IF($A22-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($G$5:$G$94,$A22-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(Premissas!$B$59*Unitário!$B$22+(1-Premissas!$B$62)*(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25)-Premissas!$B$62*((1-Premissas!$B$61)*Unitário!$B$24+(1-Premissas!$B$63)*Unitário!$B$25)-Premissas!$B$41)</f>
@@ -5578,7 +5578,7 @@
       </c>
       <c r="L22" s="12" t="n">
         <f aca="false">IF($A22-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A22-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*(Premissas!$B$51-(1-Premissas!$B$61)*Unitário!$B$24-(1-Premissas!$B$63)*Unitário!$B$25-(1-Premissas!$B$59)*Unitário!$B$22)</f>
-        <v>243.3893</v>
+        <v>221.263</v>
       </c>
       <c r="M22" s="12" t="n">
         <f aca="false">IF($A22-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A22-(Premissas!$B$56)),0)*(Premissas!$B$52-Unitário!$B$27)</f>
@@ -5602,11 +5602,11 @@
       </c>
       <c r="R22" s="12" t="n">
         <f aca="false">E22+F22+SUM(I22:Q22)</f>
-        <v>268.07268103</v>
+        <v>243.7024373</v>
       </c>
       <c r="S22" s="12" t="n">
         <f aca="false">S21+R22</f>
-        <v>-500.759482813333</v>
+        <v>-455.235893466667</v>
       </c>
       <c r="T22" s="15" t="n">
         <f aca="false">IF(AND($A22&gt;$B$100,S22&gt;=0),1,0)</f>
@@ -5614,7 +5614,7 @@
       </c>
       <c r="U22" s="12" t="n">
         <f aca="false">S22-SUM($E$5:E22)-(1+Premissas!$B$17)*SUM($C$5:C22)</f>
-        <v>-1377.25048281333</v>
+        <v>-1252.04589346667</v>
       </c>
       <c r="V22" s="12" t="n">
         <f aca="false">(G22+H22)*Premissas!$B$21</f>
@@ -5626,7 +5626,7 @@
       </c>
       <c r="X22" s="12" t="n">
         <f aca="false">X21-Y21+C22*(1+Premissas!$B$17)</f>
-        <v>62.6065</v>
+        <v>56.915</v>
       </c>
       <c r="Y22" s="12" t="n">
         <f aca="false">IF(OR(X22&gt;=Premissas!$B$13,B22=DATE(YEAR(B22),MONTH(B22)+1,0)),X22,0)</f>
@@ -5634,7 +5634,7 @@
       </c>
       <c r="Z22" s="12" t="n">
         <f aca="false">Z21-AA21+C22/Premissas!$B$18*Premissas!$B$20</f>
-        <v>9.9</v>
+        <v>9</v>
       </c>
       <c r="AA22" s="12" t="n">
         <f aca="false">IF(OR(Z22&gt;=Premissas!$B$14,B22=DATE(YEAR(B22),MONTH(B22)+1,0)),Z22,0)</f>
@@ -5687,11 +5687,11 @@
       </c>
       <c r="K23" s="12" t="n">
         <f aca="false">IF($A23-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($G$5:$G$94,$A23-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(Premissas!$B$59*Unitário!$B$22+(1-Premissas!$B$62)*(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25)-Premissas!$B$62*((1-Premissas!$B$61)*Unitário!$B$24+(1-Premissas!$B$63)*Unitário!$B$25)-Premissas!$B$41)</f>
-        <v>-5.13333333333333</v>
+        <v>-4.66666666666667</v>
       </c>
       <c r="L23" s="12" t="n">
         <f aca="false">IF($A23-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A23-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*(Premissas!$B$51-(1-Premissas!$B$61)*Unitário!$B$24-(1-Premissas!$B$63)*Unitário!$B$25-(1-Premissas!$B$59)*Unitário!$B$22)</f>
-        <v>243.3893</v>
+        <v>221.263</v>
       </c>
       <c r="M23" s="12" t="n">
         <f aca="false">IF($A23-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A23-(Premissas!$B$56)),0)*(Premissas!$B$52-Unitário!$B$27)</f>
@@ -5703,7 +5703,7 @@
       </c>
       <c r="O23" s="12" t="n">
         <f aca="false">IF($A23-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($H$5:$H$94,$A23-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(-Premissas!$B$52-Premissas!$B$41+(1-Premissas!$B$62)*Premissas!$B$31+Premissas!$B$59*Unitário!$B$22)</f>
-        <v>-15.0601</v>
+        <v>-13.691</v>
       </c>
       <c r="P23" s="12" t="n">
         <f aca="false">-Premissas!$B$42*(IF($A23-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A23-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*Premissas!$B$51+IF($A23-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A23-(Premissas!$B$56)),0)*(1-Premissas!$B$27)*Premissas!$B$52)</f>
@@ -5715,11 +5715,11 @@
       </c>
       <c r="R23" s="12" t="n">
         <f aca="false">E23+F23+SUM(I23:Q23)</f>
-        <v>223.195866666667</v>
+        <v>202.905333333333</v>
       </c>
       <c r="S23" s="12" t="n">
         <f aca="false">S22+R23</f>
-        <v>-277.563616146667</v>
+        <v>-252.330560133333</v>
       </c>
       <c r="T23" s="15" t="n">
         <f aca="false">IF(AND($A23&gt;$B$100,S23&gt;=0),1,0)</f>
@@ -5727,7 +5727,7 @@
       </c>
       <c r="U23" s="12" t="n">
         <f aca="false">S23-SUM($E$5:E23)-(1+Premissas!$B$17)*SUM($C$5:C23)</f>
-        <v>-1154.05461614667</v>
+        <v>-1049.14056013333</v>
       </c>
       <c r="V23" s="12" t="n">
         <f aca="false">(G23+H23)*Premissas!$B$21</f>
@@ -5739,7 +5739,7 @@
       </c>
       <c r="X23" s="12" t="n">
         <f aca="false">X22-Y22+C23*(1+Premissas!$B$17)</f>
-        <v>62.6065</v>
+        <v>56.915</v>
       </c>
       <c r="Y23" s="12" t="n">
         <f aca="false">IF(OR(X23&gt;=Premissas!$B$13,B23=DATE(YEAR(B23),MONTH(B23)+1,0)),X23,0)</f>
@@ -5747,7 +5747,7 @@
       </c>
       <c r="Z23" s="12" t="n">
         <f aca="false">Z22-AA22+C23/Premissas!$B$18*Premissas!$B$20</f>
-        <v>9.9</v>
+        <v>9</v>
       </c>
       <c r="AA23" s="12" t="n">
         <f aca="false">IF(OR(Z23&gt;=Premissas!$B$14,B23=DATE(YEAR(B23),MONTH(B23)+1,0)),Z23,0)</f>
@@ -5800,11 +5800,11 @@
       </c>
       <c r="K24" s="12" t="n">
         <f aca="false">IF($A24-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($G$5:$G$94,$A24-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(Premissas!$B$59*Unitário!$B$22+(1-Premissas!$B$62)*(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25)-Premissas!$B$62*((1-Premissas!$B$61)*Unitário!$B$24+(1-Premissas!$B$63)*Unitário!$B$25)-Premissas!$B$41)</f>
-        <v>-5.13333333333333</v>
+        <v>-4.66666666666667</v>
       </c>
       <c r="L24" s="12" t="n">
         <f aca="false">IF($A24-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A24-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*(Premissas!$B$51-(1-Premissas!$B$61)*Unitário!$B$24-(1-Premissas!$B$63)*Unitário!$B$25-(1-Premissas!$B$59)*Unitário!$B$22)</f>
-        <v>243.3893</v>
+        <v>221.263</v>
       </c>
       <c r="M24" s="12" t="n">
         <f aca="false">IF($A24-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A24-(Premissas!$B$56)),0)*(Premissas!$B$52-Unitário!$B$27)</f>
@@ -5816,7 +5816,7 @@
       </c>
       <c r="O24" s="12" t="n">
         <f aca="false">IF($A24-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($H$5:$H$94,$A24-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(-Premissas!$B$52-Premissas!$B$41+(1-Premissas!$B$62)*Premissas!$B$31+Premissas!$B$59*Unitário!$B$22)</f>
-        <v>-15.0601</v>
+        <v>-13.691</v>
       </c>
       <c r="P24" s="12" t="n">
         <f aca="false">-Premissas!$B$42*(IF($A24-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A24-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*Premissas!$B$51+IF($A24-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A24-(Premissas!$B$56)),0)*(1-Premissas!$B$27)*Premissas!$B$52)</f>
@@ -5828,11 +5828,11 @@
       </c>
       <c r="R24" s="12" t="n">
         <f aca="false">E24+F24+SUM(I24:Q24)</f>
-        <v>223.195866666667</v>
+        <v>202.905333333333</v>
       </c>
       <c r="S24" s="12" t="n">
         <f aca="false">S23+R24</f>
-        <v>-54.3677494800001</v>
+        <v>-49.4252268000001</v>
       </c>
       <c r="T24" s="15" t="n">
         <f aca="false">IF(AND($A24&gt;$B$100,S24&gt;=0),1,0)</f>
@@ -5840,7 +5840,7 @@
       </c>
       <c r="U24" s="12" t="n">
         <f aca="false">S24-SUM($E$5:E24)-(1+Premissas!$B$17)*SUM($C$5:C24)</f>
-        <v>-930.85874948</v>
+        <v>-846.2352268</v>
       </c>
       <c r="V24" s="12" t="n">
         <f aca="false">(G24+H24)*Premissas!$B$21</f>
@@ -5852,7 +5852,7 @@
       </c>
       <c r="X24" s="12" t="n">
         <f aca="false">X23-Y23+C24*(1+Premissas!$B$17)</f>
-        <v>62.6065</v>
+        <v>56.915</v>
       </c>
       <c r="Y24" s="12" t="n">
         <f aca="false">IF(OR(X24&gt;=Premissas!$B$13,B24=DATE(YEAR(B24),MONTH(B24)+1,0)),X24,0)</f>
@@ -5860,7 +5860,7 @@
       </c>
       <c r="Z24" s="12" t="n">
         <f aca="false">Z23-AA23+C24/Premissas!$B$18*Premissas!$B$20</f>
-        <v>9.9</v>
+        <v>9</v>
       </c>
       <c r="AA24" s="12" t="n">
         <f aca="false">IF(OR(Z24&gt;=Premissas!$B$14,B24=DATE(YEAR(B24),MONTH(B24)+1,0)),Z24,0)</f>
@@ -5913,11 +5913,11 @@
       </c>
       <c r="K25" s="12" t="n">
         <f aca="false">IF($A25-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($G$5:$G$94,$A25-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(Premissas!$B$59*Unitário!$B$22+(1-Premissas!$B$62)*(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25)-Premissas!$B$62*((1-Premissas!$B$61)*Unitário!$B$24+(1-Premissas!$B$63)*Unitário!$B$25)-Premissas!$B$41)</f>
-        <v>-5.13333333333333</v>
+        <v>-4.66666666666667</v>
       </c>
       <c r="L25" s="12" t="n">
         <f aca="false">IF($A25-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A25-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*(Premissas!$B$51-(1-Premissas!$B$61)*Unitário!$B$24-(1-Premissas!$B$63)*Unitário!$B$25-(1-Premissas!$B$59)*Unitário!$B$22)</f>
-        <v>243.3893</v>
+        <v>221.263</v>
       </c>
       <c r="M25" s="12" t="n">
         <f aca="false">IF($A25-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A25-(Premissas!$B$56)),0)*(Premissas!$B$52-Unitário!$B$27)</f>
@@ -5929,7 +5929,7 @@
       </c>
       <c r="O25" s="12" t="n">
         <f aca="false">IF($A25-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($H$5:$H$94,$A25-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(-Premissas!$B$52-Premissas!$B$41+(1-Premissas!$B$62)*Premissas!$B$31+Premissas!$B$59*Unitário!$B$22)</f>
-        <v>-15.0601</v>
+        <v>-13.691</v>
       </c>
       <c r="P25" s="12" t="n">
         <f aca="false">-Premissas!$B$42*(IF($A25-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A25-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*Premissas!$B$51+IF($A25-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A25-(Premissas!$B$56)),0)*(1-Premissas!$B$27)*Premissas!$B$52)</f>
@@ -5941,11 +5941,11 @@
       </c>
       <c r="R25" s="12" t="n">
         <f aca="false">E25+F25+SUM(I25:Q25)</f>
-        <v>223.195866666667</v>
+        <v>202.905333333333</v>
       </c>
       <c r="S25" s="12" t="n">
         <f aca="false">S24+R25</f>
-        <v>168.828117186667</v>
+        <v>153.480106533333</v>
       </c>
       <c r="T25" s="15" t="n">
         <f aca="false">IF(AND($A25&gt;$B$100,S25&gt;=0),1,0)</f>
@@ -5953,7 +5953,7 @@
       </c>
       <c r="U25" s="12" t="n">
         <f aca="false">S25-SUM($E$5:E25)-(1+Premissas!$B$17)*SUM($C$5:C25)</f>
-        <v>-707.662882813334</v>
+        <v>-643.329893466667</v>
       </c>
       <c r="V25" s="12" t="n">
         <f aca="false">(G25+H25)*Premissas!$B$21</f>
@@ -5965,7 +5965,7 @@
       </c>
       <c r="X25" s="12" t="n">
         <f aca="false">X24-Y24+C25*(1+Premissas!$B$17)</f>
-        <v>62.6065</v>
+        <v>56.915</v>
       </c>
       <c r="Y25" s="12" t="n">
         <f aca="false">IF(OR(X25&gt;=Premissas!$B$13,B25=DATE(YEAR(B25),MONTH(B25)+1,0)),X25,0)</f>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="Z25" s="12" t="n">
         <f aca="false">Z24-AA24+C25/Premissas!$B$18*Premissas!$B$20</f>
-        <v>9.9</v>
+        <v>9</v>
       </c>
       <c r="AA25" s="12" t="n">
         <f aca="false">IF(OR(Z25&gt;=Premissas!$B$14,B25=DATE(YEAR(B25),MONTH(B25)+1,0)),Z25,0)</f>
@@ -6026,11 +6026,11 @@
       </c>
       <c r="K26" s="12" t="n">
         <f aca="false">IF($A26-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($G$5:$G$94,$A26-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(Premissas!$B$59*Unitário!$B$22+(1-Premissas!$B$62)*(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25)-Premissas!$B$62*((1-Premissas!$B$61)*Unitário!$B$24+(1-Premissas!$B$63)*Unitário!$B$25)-Premissas!$B$41)</f>
-        <v>-5.13333333333333</v>
+        <v>-4.66666666666667</v>
       </c>
       <c r="L26" s="12" t="n">
         <f aca="false">IF($A26-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A26-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*(Premissas!$B$51-(1-Premissas!$B$61)*Unitário!$B$24-(1-Premissas!$B$63)*Unitário!$B$25-(1-Premissas!$B$59)*Unitário!$B$22)</f>
-        <v>243.3893</v>
+        <v>221.263</v>
       </c>
       <c r="M26" s="12" t="n">
         <f aca="false">IF($A26-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A26-(Premissas!$B$56)),0)*(Premissas!$B$52-Unitário!$B$27)</f>
@@ -6042,7 +6042,7 @@
       </c>
       <c r="O26" s="12" t="n">
         <f aca="false">IF($A26-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($H$5:$H$94,$A26-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(-Premissas!$B$52-Premissas!$B$41+(1-Premissas!$B$62)*Premissas!$B$31+Premissas!$B$59*Unitário!$B$22)</f>
-        <v>-15.0601</v>
+        <v>-13.691</v>
       </c>
       <c r="P26" s="12" t="n">
         <f aca="false">-Premissas!$B$42*(IF($A26-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A26-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*Premissas!$B$51+IF($A26-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A26-(Premissas!$B$56)),0)*(1-Premissas!$B$27)*Premissas!$B$52)</f>
@@ -6054,11 +6054,11 @@
       </c>
       <c r="R26" s="12" t="n">
         <f aca="false">E26+F26+SUM(I26:Q26)</f>
-        <v>223.195866666667</v>
+        <v>202.905333333333</v>
       </c>
       <c r="S26" s="12" t="n">
         <f aca="false">S25+R26</f>
-        <v>392.023983853333</v>
+        <v>356.385439866667</v>
       </c>
       <c r="T26" s="15" t="n">
         <f aca="false">IF(AND($A26&gt;$B$100,S26&gt;=0),1,0)</f>
@@ -6066,7 +6066,7 @@
       </c>
       <c r="U26" s="12" t="n">
         <f aca="false">S26-SUM($E$5:E26)-(1+Premissas!$B$17)*SUM($C$5:C26)</f>
-        <v>-484.467016146667</v>
+        <v>-440.424560133333</v>
       </c>
       <c r="V26" s="12" t="n">
         <f aca="false">(G26+H26)*Premissas!$B$21</f>
@@ -6078,7 +6078,7 @@
       </c>
       <c r="X26" s="12" t="n">
         <f aca="false">X25-Y25+C26*(1+Premissas!$B$17)</f>
-        <v>62.6065</v>
+        <v>56.915</v>
       </c>
       <c r="Y26" s="12" t="n">
         <f aca="false">IF(OR(X26&gt;=Premissas!$B$13,B26=DATE(YEAR(B26),MONTH(B26)+1,0)),X26,0)</f>
@@ -6086,7 +6086,7 @@
       </c>
       <c r="Z26" s="12" t="n">
         <f aca="false">Z25-AA25+C26/Premissas!$B$18*Premissas!$B$20</f>
-        <v>9.9</v>
+        <v>9</v>
       </c>
       <c r="AA26" s="12" t="n">
         <f aca="false">IF(OR(Z26&gt;=Premissas!$B$14,B26=DATE(YEAR(B26),MONTH(B26)+1,0)),Z26,0)</f>
@@ -6139,11 +6139,11 @@
       </c>
       <c r="K27" s="12" t="n">
         <f aca="false">IF($A27-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($G$5:$G$94,$A27-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(Premissas!$B$59*Unitário!$B$22+(1-Premissas!$B$62)*(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25)-Premissas!$B$62*((1-Premissas!$B$61)*Unitário!$B$24+(1-Premissas!$B$63)*Unitário!$B$25)-Premissas!$B$41)</f>
-        <v>-5.13333333333333</v>
+        <v>-4.66666666666667</v>
       </c>
       <c r="L27" s="12" t="n">
         <f aca="false">IF($A27-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A27-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*(Premissas!$B$51-(1-Premissas!$B$61)*Unitário!$B$24-(1-Premissas!$B$63)*Unitário!$B$25-(1-Premissas!$B$59)*Unitário!$B$22)</f>
-        <v>243.3893</v>
+        <v>221.263</v>
       </c>
       <c r="M27" s="12" t="n">
         <f aca="false">IF($A27-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A27-(Premissas!$B$56)),0)*(Premissas!$B$52-Unitário!$B$27)</f>
@@ -6155,7 +6155,7 @@
       </c>
       <c r="O27" s="12" t="n">
         <f aca="false">IF($A27-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($H$5:$H$94,$A27-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(-Premissas!$B$52-Premissas!$B$41+(1-Premissas!$B$62)*Premissas!$B$31+Premissas!$B$59*Unitário!$B$22)</f>
-        <v>-15.0601</v>
+        <v>-13.691</v>
       </c>
       <c r="P27" s="12" t="n">
         <f aca="false">-Premissas!$B$42*(IF($A27-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A27-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*Premissas!$B$51+IF($A27-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A27-(Premissas!$B$56)),0)*(1-Premissas!$B$27)*Premissas!$B$52)</f>
@@ -6167,11 +6167,11 @@
       </c>
       <c r="R27" s="12" t="n">
         <f aca="false">E27+F27+SUM(I27:Q27)</f>
-        <v>223.195866666667</v>
+        <v>202.905333333333</v>
       </c>
       <c r="S27" s="12" t="n">
         <f aca="false">S26+R27</f>
-        <v>615.21985052</v>
+        <v>559.2907732</v>
       </c>
       <c r="T27" s="15" t="n">
         <f aca="false">IF(AND($A27&gt;$B$100,S27&gt;=0),1,0)</f>
@@ -6179,7 +6179,7 @@
       </c>
       <c r="U27" s="12" t="n">
         <f aca="false">S27-SUM($E$5:E27)-(1+Premissas!$B$17)*SUM($C$5:C27)</f>
-        <v>-261.27114948</v>
+        <v>-237.5192268</v>
       </c>
       <c r="V27" s="12" t="n">
         <f aca="false">(G27+H27)*Premissas!$B$21</f>
@@ -6191,7 +6191,7 @@
       </c>
       <c r="X27" s="12" t="n">
         <f aca="false">X26-Y26+C27*(1+Premissas!$B$17)</f>
-        <v>62.6065</v>
+        <v>56.915</v>
       </c>
       <c r="Y27" s="12" t="n">
         <f aca="false">IF(OR(X27&gt;=Premissas!$B$13,B27=DATE(YEAR(B27),MONTH(B27)+1,0)),X27,0)</f>
@@ -6199,7 +6199,7 @@
       </c>
       <c r="Z27" s="12" t="n">
         <f aca="false">Z26-AA26+C27/Premissas!$B$18*Premissas!$B$20</f>
-        <v>9.9</v>
+        <v>9</v>
       </c>
       <c r="AA27" s="12" t="n">
         <f aca="false">IF(OR(Z27&gt;=Premissas!$B$14,B27=DATE(YEAR(B27),MONTH(B27)+1,0)),Z27,0)</f>
@@ -6252,7 +6252,7 @@
       </c>
       <c r="K28" s="12" t="n">
         <f aca="false">IF($A28-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($G$5:$G$94,$A28-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(Premissas!$B$59*Unitário!$B$22+(1-Premissas!$B$62)*(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25)-Premissas!$B$62*((1-Premissas!$B$61)*Unitário!$B$24+(1-Premissas!$B$63)*Unitário!$B$25)-Premissas!$B$41)</f>
-        <v>-5.13333333333333</v>
+        <v>-4.66666666666667</v>
       </c>
       <c r="L28" s="12" t="n">
         <f aca="false">IF($A28-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A28-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*(Premissas!$B$51-(1-Premissas!$B$61)*Unitário!$B$24-(1-Premissas!$B$63)*Unitário!$B$25-(1-Premissas!$B$59)*Unitário!$B$22)</f>
@@ -6268,7 +6268,7 @@
       </c>
       <c r="O28" s="12" t="n">
         <f aca="false">IF($A28-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($H$5:$H$94,$A28-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(-Premissas!$B$52-Premissas!$B$41+(1-Premissas!$B$62)*Premissas!$B$31+Premissas!$B$59*Unitário!$B$22)</f>
-        <v>-15.0601</v>
+        <v>-13.691</v>
       </c>
       <c r="P28" s="12" t="n">
         <f aca="false">-Premissas!$B$42*(IF($A28-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A28-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*Premissas!$B$51+IF($A28-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A28-(Premissas!$B$56)),0)*(1-Premissas!$B$27)*Premissas!$B$52)</f>
@@ -6280,11 +6280,11 @@
       </c>
       <c r="R28" s="12" t="n">
         <f aca="false">E28+F28+SUM(I28:Q28)</f>
-        <v>-20.1934333333333</v>
+        <v>-18.3576666666667</v>
       </c>
       <c r="S28" s="12" t="n">
         <f aca="false">S27+R28</f>
-        <v>595.026417186666</v>
+        <v>540.933106533333</v>
       </c>
       <c r="T28" s="15" t="n">
         <f aca="false">IF(AND($A28&gt;$B$100,S28&gt;=0),1,0)</f>
@@ -6292,7 +6292,7 @@
       </c>
       <c r="U28" s="12" t="n">
         <f aca="false">S28-SUM($E$5:E28)-(1+Premissas!$B$17)*SUM($C$5:C28)</f>
-        <v>-281.464582813334</v>
+        <v>-255.876893466667</v>
       </c>
       <c r="V28" s="12" t="n">
         <f aca="false">(G28+H28)*Premissas!$B$21</f>
@@ -6304,7 +6304,7 @@
       </c>
       <c r="X28" s="12" t="n">
         <f aca="false">X27-Y27+C28*(1+Premissas!$B$17)</f>
-        <v>62.6065</v>
+        <v>56.915</v>
       </c>
       <c r="Y28" s="12" t="n">
         <f aca="false">IF(OR(X28&gt;=Premissas!$B$13,B28=DATE(YEAR(B28),MONTH(B28)+1,0)),X28,0)</f>
@@ -6312,7 +6312,7 @@
       </c>
       <c r="Z28" s="12" t="n">
         <f aca="false">Z27-AA27+C28/Premissas!$B$18*Premissas!$B$20</f>
-        <v>9.9</v>
+        <v>9</v>
       </c>
       <c r="AA28" s="12" t="n">
         <f aca="false">IF(OR(Z28&gt;=Premissas!$B$14,B28=DATE(YEAR(B28),MONTH(B28)+1,0)),Z28,0)</f>
@@ -6365,7 +6365,7 @@
       </c>
       <c r="K29" s="12" t="n">
         <f aca="false">IF($A29-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($G$5:$G$94,$A29-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(Premissas!$B$59*Unitário!$B$22+(1-Premissas!$B$62)*(Premissas!$B$61*Unitário!$B$24+Premissas!$B$63*Unitário!$B$25)-Premissas!$B$62*((1-Premissas!$B$61)*Unitário!$B$24+(1-Premissas!$B$63)*Unitário!$B$25)-Premissas!$B$41)</f>
-        <v>-5.13333333333333</v>
+        <v>-4.66666666666667</v>
       </c>
       <c r="L29" s="12" t="n">
         <f aca="false">IF($A29-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A29-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*(Premissas!$B$51-(1-Premissas!$B$61)*Unitário!$B$24-(1-Premissas!$B$63)*Unitário!$B$25-(1-Premissas!$B$59)*Unitário!$B$22)</f>
@@ -6381,7 +6381,7 @@
       </c>
       <c r="O29" s="12" t="n">
         <f aca="false">IF($A29-(Premissas!$B$54+Premissas!$B$57)&gt;=1,INDEX($H$5:$H$94,$A29-(Premissas!$B$54+Premissas!$B$57)),0)*Premissas!$B$27*(-Premissas!$B$52-Premissas!$B$41+(1-Premissas!$B$62)*Premissas!$B$31+Premissas!$B$59*Unitário!$B$22)</f>
-        <v>-15.0601</v>
+        <v>-13.691</v>
       </c>
       <c r="P29" s="12" t="n">
         <f aca="false">-Premissas!$B$42*(IF($A29-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A29-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*Premissas!$B$51+IF($A29-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A29-(Premissas!$B$56)),0)*(1-Premissas!$B$27)*Premissas!$B$52)</f>
@@ -6393,11 +6393,11 @@
       </c>
       <c r="R29" s="12" t="n">
         <f aca="false">E29+F29+SUM(I29:Q29)</f>
-        <v>-20.1934333333333</v>
+        <v>-18.3576666666667</v>
       </c>
       <c r="S29" s="12" t="n">
         <f aca="false">S28+R29</f>
-        <v>574.832983853333</v>
+        <v>522.575439866667</v>
       </c>
       <c r="T29" s="15" t="n">
         <f aca="false">IF(AND($A29&gt;$B$100,S29&gt;=0),1,0)</f>
@@ -6405,7 +6405,7 @@
       </c>
       <c r="U29" s="12" t="n">
         <f aca="false">S29-SUM($E$5:E29)-(1+Premissas!$B$17)*SUM($C$5:C29)</f>
-        <v>-301.658016146667</v>
+        <v>-274.234560133333</v>
       </c>
       <c r="V29" s="12" t="n">
         <f aca="false">(G29+H29)*Premissas!$B$21</f>
@@ -6417,7 +6417,7 @@
       </c>
       <c r="X29" s="12" t="n">
         <f aca="false">X28-Y28+C29*(1+Premissas!$B$17)</f>
-        <v>62.6065</v>
+        <v>56.915</v>
       </c>
       <c r="Y29" s="12" t="n">
         <f aca="false">IF(OR(X29&gt;=Premissas!$B$13,B29=DATE(YEAR(B29),MONTH(B29)+1,0)),X29,0)</f>
@@ -6425,7 +6425,7 @@
       </c>
       <c r="Z29" s="12" t="n">
         <f aca="false">Z28-AA28+C29/Premissas!$B$18*Premissas!$B$20</f>
-        <v>9.9</v>
+        <v>9</v>
       </c>
       <c r="AA29" s="12" t="n">
         <f aca="false">IF(OR(Z29&gt;=Premissas!$B$14,B29=DATE(YEAR(B29),MONTH(B29)+1,0)),Z29,0)</f>
@@ -6482,7 +6482,7 @@
       </c>
       <c r="L30" s="12" t="n">
         <f aca="false">IF($A30-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A30-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*(Premissas!$B$51-(1-Premissas!$B$61)*Unitário!$B$24-(1-Premissas!$B$63)*Unitário!$B$25-(1-Premissas!$B$59)*Unitário!$B$22)</f>
-        <v>243.3893</v>
+        <v>221.263</v>
       </c>
       <c r="M30" s="12" t="n">
         <f aca="false">IF($A30-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A30-(Premissas!$B$56)),0)*(Premissas!$B$52-Unitário!$B$27)</f>
@@ -6506,11 +6506,11 @@
       </c>
       <c r="R30" s="12" t="n">
         <f aca="false">E30+F30+SUM(I30:Q30)</f>
-        <v>243.3893</v>
+        <v>221.263</v>
       </c>
       <c r="S30" s="12" t="n">
         <f aca="false">S29+R30</f>
-        <v>818.222283853333</v>
+        <v>743.838439866667</v>
       </c>
       <c r="T30" s="15" t="n">
         <f aca="false">IF(AND($A30&gt;$B$100,S30&gt;=0),1,0)</f>
@@ -6518,7 +6518,7 @@
       </c>
       <c r="U30" s="12" t="n">
         <f aca="false">S30-SUM($E$5:E30)-(1+Premissas!$B$17)*SUM($C$5:C30)</f>
-        <v>-58.2687161466671</v>
+        <v>-52.9715601333334</v>
       </c>
       <c r="V30" s="12" t="n">
         <f aca="false">(G30+H30)*Premissas!$B$21</f>
@@ -6530,7 +6530,7 @@
       </c>
       <c r="X30" s="12" t="n">
         <f aca="false">X29-Y29+C30*(1+Premissas!$B$17)</f>
-        <v>62.6065</v>
+        <v>56.915</v>
       </c>
       <c r="Y30" s="12" t="n">
         <f aca="false">IF(OR(X30&gt;=Premissas!$B$13,B30=DATE(YEAR(B30),MONTH(B30)+1,0)),X30,0)</f>
@@ -6538,7 +6538,7 @@
       </c>
       <c r="Z30" s="12" t="n">
         <f aca="false">Z29-AA29+C30/Premissas!$B$18*Premissas!$B$20</f>
-        <v>9.9</v>
+        <v>9</v>
       </c>
       <c r="AA30" s="12" t="n">
         <f aca="false">IF(OR(Z30&gt;=Premissas!$B$14,B30=DATE(YEAR(B30),MONTH(B30)+1,0)),Z30,0)</f>
@@ -6595,7 +6595,7 @@
       </c>
       <c r="L31" s="12" t="n">
         <f aca="false">IF($A31-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A31-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*(Premissas!$B$51-(1-Premissas!$B$61)*Unitário!$B$24-(1-Premissas!$B$63)*Unitário!$B$25-(1-Premissas!$B$59)*Unitário!$B$22)</f>
-        <v>243.3893</v>
+        <v>221.263</v>
       </c>
       <c r="M31" s="12" t="n">
         <f aca="false">IF($A31-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A31-(Premissas!$B$56)),0)*(Premissas!$B$52-Unitário!$B$27)</f>
@@ -6619,11 +6619,11 @@
       </c>
       <c r="R31" s="12" t="n">
         <f aca="false">E31+F31+SUM(I31:Q31)</f>
-        <v>243.3893</v>
+        <v>221.263</v>
       </c>
       <c r="S31" s="12" t="n">
         <f aca="false">S30+R31</f>
-        <v>1061.61158385333</v>
+        <v>965.101439866667</v>
       </c>
       <c r="T31" s="15" t="n">
         <f aca="false">IF(AND($A31&gt;$B$100,S31&gt;=0),1,0)</f>
@@ -6631,7 +6631,7 @@
       </c>
       <c r="U31" s="12" t="n">
         <f aca="false">S31-SUM($E$5:E31)-(1+Premissas!$B$17)*SUM($C$5:C31)</f>
-        <v>185.120583853333</v>
+        <v>168.291439866667</v>
       </c>
       <c r="V31" s="12" t="n">
         <f aca="false">(G31+H31)*Premissas!$B$21</f>
@@ -6643,7 +6643,7 @@
       </c>
       <c r="X31" s="12" t="n">
         <f aca="false">X30-Y30+C31*(1+Premissas!$B$17)</f>
-        <v>62.6065</v>
+        <v>56.915</v>
       </c>
       <c r="Y31" s="12" t="n">
         <f aca="false">IF(OR(X31&gt;=Premissas!$B$13,B31=DATE(YEAR(B31),MONTH(B31)+1,0)),X31,0)</f>
@@ -6651,7 +6651,7 @@
       </c>
       <c r="Z31" s="12" t="n">
         <f aca="false">Z30-AA30+C31/Premissas!$B$18*Premissas!$B$20</f>
-        <v>9.9</v>
+        <v>9</v>
       </c>
       <c r="AA31" s="12" t="n">
         <f aca="false">IF(OR(Z31&gt;=Premissas!$B$14,B31=DATE(YEAR(B31),MONTH(B31)+1,0)),Z31,0)</f>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="L32" s="12" t="n">
         <f aca="false">IF($A32-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A32-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*(Premissas!$B$51-(1-Premissas!$B$61)*Unitário!$B$24-(1-Premissas!$B$63)*Unitário!$B$25-(1-Premissas!$B$59)*Unitário!$B$22)</f>
-        <v>243.3893</v>
+        <v>221.263</v>
       </c>
       <c r="M32" s="12" t="n">
         <f aca="false">IF($A32-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A32-(Premissas!$B$56)),0)*(Premissas!$B$52-Unitário!$B$27)</f>
@@ -6732,11 +6732,11 @@
       </c>
       <c r="R32" s="12" t="n">
         <f aca="false">E32+F32+SUM(I32:Q32)</f>
-        <v>243.3893</v>
+        <v>221.263</v>
       </c>
       <c r="S32" s="12" t="n">
         <f aca="false">S31+R32</f>
-        <v>1305.00088385333</v>
+        <v>1186.36443986667</v>
       </c>
       <c r="T32" s="15" t="n">
         <f aca="false">IF(AND($A32&gt;$B$100,S32&gt;=0),1,0)</f>
@@ -6744,7 +6744,7 @@
       </c>
       <c r="U32" s="12" t="n">
         <f aca="false">S32-SUM($E$5:E32)-(1+Premissas!$B$17)*SUM($C$5:C32)</f>
-        <v>428.509883853333</v>
+        <v>389.554439866667</v>
       </c>
       <c r="V32" s="12" t="n">
         <f aca="false">(G32+H32)*Premissas!$B$21</f>
@@ -6756,7 +6756,7 @@
       </c>
       <c r="X32" s="12" t="n">
         <f aca="false">X31-Y31+C32*(1+Premissas!$B$17)</f>
-        <v>62.6065</v>
+        <v>56.915</v>
       </c>
       <c r="Y32" s="12" t="n">
         <f aca="false">IF(OR(X32&gt;=Premissas!$B$13,B32=DATE(YEAR(B32),MONTH(B32)+1,0)),X32,0)</f>
@@ -6764,7 +6764,7 @@
       </c>
       <c r="Z32" s="12" t="n">
         <f aca="false">Z31-AA31+C32/Premissas!$B$18*Premissas!$B$20</f>
-        <v>9.9</v>
+        <v>9</v>
       </c>
       <c r="AA32" s="12" t="n">
         <f aca="false">IF(OR(Z32&gt;=Premissas!$B$14,B32=DATE(YEAR(B32),MONTH(B32)+1,0)),Z32,0)</f>
@@ -6821,7 +6821,7 @@
       </c>
       <c r="L33" s="12" t="n">
         <f aca="false">IF($A33-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A33-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*(Premissas!$B$51-(1-Premissas!$B$61)*Unitário!$B$24-(1-Premissas!$B$63)*Unitário!$B$25-(1-Premissas!$B$59)*Unitário!$B$22)</f>
-        <v>243.3893</v>
+        <v>221.263</v>
       </c>
       <c r="M33" s="12" t="n">
         <f aca="false">IF($A33-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A33-(Premissas!$B$56)),0)*(Premissas!$B$52-Unitário!$B$27)</f>
@@ -6845,11 +6845,11 @@
       </c>
       <c r="R33" s="12" t="n">
         <f aca="false">E33+F33+SUM(I33:Q33)</f>
-        <v>243.3893</v>
+        <v>221.263</v>
       </c>
       <c r="S33" s="12" t="n">
         <f aca="false">S32+R33</f>
-        <v>1548.39018385333</v>
+        <v>1407.62743986667</v>
       </c>
       <c r="T33" s="15" t="n">
         <f aca="false">IF(AND($A33&gt;$B$100,S33&gt;=0),1,0)</f>
@@ -6857,7 +6857,7 @@
       </c>
       <c r="U33" s="12" t="n">
         <f aca="false">S33-SUM($E$5:E33)-(1+Premissas!$B$17)*SUM($C$5:C33)</f>
-        <v>671.899183853333</v>
+        <v>610.817439866667</v>
       </c>
       <c r="V33" s="12" t="n">
         <f aca="false">(G33+H33)*Premissas!$B$21</f>
@@ -6869,7 +6869,7 @@
       </c>
       <c r="X33" s="12" t="n">
         <f aca="false">X32-Y32+C33*(1+Premissas!$B$17)</f>
-        <v>62.6065</v>
+        <v>56.915</v>
       </c>
       <c r="Y33" s="12" t="n">
         <f aca="false">IF(OR(X33&gt;=Premissas!$B$13,B33=DATE(YEAR(B33),MONTH(B33)+1,0)),X33,0)</f>
@@ -6877,7 +6877,7 @@
       </c>
       <c r="Z33" s="12" t="n">
         <f aca="false">Z32-AA32+C33/Premissas!$B$18*Premissas!$B$20</f>
-        <v>9.9</v>
+        <v>9</v>
       </c>
       <c r="AA33" s="12" t="n">
         <f aca="false">IF(OR(Z33&gt;=Premissas!$B$14,B33=DATE(YEAR(B33),MONTH(B33)+1,0)),Z33,0)</f>
@@ -6934,7 +6934,7 @@
       </c>
       <c r="L34" s="12" t="n">
         <f aca="false">IF($A34-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A34-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*(Premissas!$B$51-(1-Premissas!$B$61)*Unitário!$B$24-(1-Premissas!$B$63)*Unitário!$B$25-(1-Premissas!$B$59)*Unitário!$B$22)</f>
-        <v>243.3893</v>
+        <v>221.263</v>
       </c>
       <c r="M34" s="12" t="n">
         <f aca="false">IF($A34-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A34-(Premissas!$B$56)),0)*(Premissas!$B$52-Unitário!$B$27)</f>
@@ -6958,11 +6958,11 @@
       </c>
       <c r="R34" s="12" t="n">
         <f aca="false">E34+F34+SUM(I34:Q34)</f>
-        <v>243.3893</v>
+        <v>221.263</v>
       </c>
       <c r="S34" s="12" t="n">
         <f aca="false">S33+R34</f>
-        <v>1791.77948385333</v>
+        <v>1628.89043986667</v>
       </c>
       <c r="T34" s="15" t="n">
         <f aca="false">IF(AND($A34&gt;$B$100,S34&gt;=0),1,0)</f>
@@ -6970,7 +6970,7 @@
       </c>
       <c r="U34" s="12" t="n">
         <f aca="false">S34-SUM($E$5:E34)-(1+Premissas!$B$17)*SUM($C$5:C34)</f>
-        <v>915.288483853333</v>
+        <v>832.080439866667</v>
       </c>
       <c r="V34" s="12" t="n">
         <f aca="false">(G34+H34)*Premissas!$B$21</f>
@@ -6982,7 +6982,7 @@
       </c>
       <c r="X34" s="12" t="n">
         <f aca="false">X33-Y33+C34*(1+Premissas!$B$17)</f>
-        <v>62.6065</v>
+        <v>56.915</v>
       </c>
       <c r="Y34" s="12" t="n">
         <f aca="false">IF(OR(X34&gt;=Premissas!$B$13,B34=DATE(YEAR(B34),MONTH(B34)+1,0)),X34,0)</f>
@@ -6990,7 +6990,7 @@
       </c>
       <c r="Z34" s="12" t="n">
         <f aca="false">Z33-AA33+C34/Premissas!$B$18*Premissas!$B$20</f>
-        <v>9.9</v>
+        <v>9</v>
       </c>
       <c r="AA34" s="12" t="n">
         <f aca="false">IF(OR(Z34&gt;=Premissas!$B$14,B34=DATE(YEAR(B34),MONTH(B34)+1,0)),Z34,0)</f>
@@ -7047,7 +7047,7 @@
       </c>
       <c r="L35" s="12" t="n">
         <f aca="false">IF($A35-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A35-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*(Premissas!$B$51-(1-Premissas!$B$61)*Unitário!$B$24-(1-Premissas!$B$63)*Unitário!$B$25-(1-Premissas!$B$59)*Unitário!$B$22)</f>
-        <v>243.3893</v>
+        <v>221.263</v>
       </c>
       <c r="M35" s="12" t="n">
         <f aca="false">IF($A35-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A35-(Premissas!$B$56)),0)*(Premissas!$B$52-Unitário!$B$27)</f>
@@ -7071,11 +7071,11 @@
       </c>
       <c r="R35" s="12" t="n">
         <f aca="false">E35+F35+SUM(I35:Q35)</f>
-        <v>243.3893</v>
+        <v>221.263</v>
       </c>
       <c r="S35" s="12" t="n">
         <f aca="false">S34+R35</f>
-        <v>2035.16878385333</v>
+        <v>1850.15343986667</v>
       </c>
       <c r="T35" s="15" t="n">
         <f aca="false">IF(AND($A35&gt;$B$100,S35&gt;=0),1,0)</f>
@@ -7083,7 +7083,7 @@
       </c>
       <c r="U35" s="12" t="n">
         <f aca="false">S35-SUM($E$5:E35)-(1+Premissas!$B$17)*SUM($C$5:C35)</f>
-        <v>1158.67778385333</v>
+        <v>1053.34343986667</v>
       </c>
       <c r="V35" s="12" t="n">
         <f aca="false">(G35+H35)*Premissas!$B$21</f>
@@ -7095,7 +7095,7 @@
       </c>
       <c r="X35" s="12" t="n">
         <f aca="false">X34-Y34+C35*(1+Premissas!$B$17)</f>
-        <v>62.6065</v>
+        <v>56.915</v>
       </c>
       <c r="Y35" s="12" t="n">
         <f aca="false">IF(OR(X35&gt;=Premissas!$B$13,B35=DATE(YEAR(B35),MONTH(B35)+1,0)),X35,0)</f>
@@ -7103,7 +7103,7 @@
       </c>
       <c r="Z35" s="12" t="n">
         <f aca="false">Z34-AA34+C35/Premissas!$B$18*Premissas!$B$20</f>
-        <v>9.9</v>
+        <v>9</v>
       </c>
       <c r="AA35" s="12" t="n">
         <f aca="false">IF(OR(Z35&gt;=Premissas!$B$14,B35=DATE(YEAR(B35),MONTH(B35)+1,0)),Z35,0)</f>
@@ -7160,7 +7160,7 @@
       </c>
       <c r="L36" s="12" t="n">
         <f aca="false">IF($A36-(Premissas!$B$54+Premissas!$B$55)&gt;=1,INDEX($G$5:$G$94,$A36-(Premissas!$B$54+Premissas!$B$55)),0)*Unitário!$B$21*(Premissas!$B$51-(1-Premissas!$B$61)*Unitário!$B$24-(1-Premissas!$B$63)*Unitário!$B$25-(1-Premissas!$B$59)*Unitário!$B$22)</f>
-        <v>243.3893</v>
+        <v>221.263</v>
       </c>
       <c r="M36" s="12" t="n">
         <f aca="false">IF($A36-(Premissas!$B$56)&gt;=1,INDEX($H$5:$H$94,$A36-(Premissas!$B$56)),0)*(Premissas!$B$52-Unitário!$B$27)</f>
@@ -7184,11 +7184,11 @@
       </c>
       <c r="R36" s="12" t="n">
         <f aca="false">E36+F36+SUM(I36:Q36)</f>
-        <v>243.3893</v>
+        <v>221.263</v>
       </c>
       <c r="S36" s="12" t="n">
         <f aca="false">S35+R36</f>
-        <v>2278.55808385333</v>
+        <v>2071.41643986667</v>
       </c>
       <c r="T36" s="15" t="n">
         <f aca="false">IF(AND($A36&gt;$B$100,S36&gt;=0),1,0)</f>
@@ -7196,7 +7196,7 @@
       </c>
       <c r="U36" s="12" t="n">
         <f aca="false">S36-SUM($E$5:E36)-(1+Premissas!$B$17)*SUM($C$5:C36)</f>
-        <v>1402.06708385333</v>
+        <v>1274.60643986667</v>
       </c>
       <c r="V36" s="12" t="n">
         <f aca="false">(G36+H36)*Premissas!$B$21</f>
@@ -7208,7 +7208,7 @@
       </c>
       <c r="X36" s="12" t="n">
         <f aca="false">X35-Y35+C36*(1+Premissas!$B$17)</f>
-        <v>62.6065</v>
+        <v>56.915</v>
       </c>
       <c r="Y36" s="12" t="n">
         <f aca="false">IF(OR(X36&gt;=Premissas!$B$13,B36=DATE(YEAR(B36),MONTH(B36)+1,0)),X36,0)</f>
@@ -7216,7 +7216,7 @@
       </c>
       <c r="Z36" s="12" t="n">
         <f aca="false">Z35-AA35+C36/Premissas!$B$18*Premissas!$B$20</f>
-        <v>9.9</v>
+        <v>9</v>
       </c>
       <c r="AA36" s="12" t="n">
         <f aca="false">IF(OR(Z36&gt;=Premissas!$B$14,B36=DATE(YEAR(B36),MONTH(B36)+1,0)),Z36,0)</f>
@@ -7301,7 +7301,7 @@
       </c>
       <c r="S37" s="12" t="n">
         <f aca="false">S36+R37</f>
-        <v>2278.55808385333</v>
+        <v>2071.41643986667</v>
       </c>
       <c r="T37" s="15" t="n">
         <f aca="false">IF(AND($A37&gt;$B$100,S37&gt;=0),1,0)</f>
@@ -7309,7 +7309,7 @@
       </c>
       <c r="U37" s="12" t="n">
         <f aca="false">S37-SUM($E$5:E37)-(1+Premissas!$B$17)*SUM($C$5:C37)</f>
-        <v>1402.06708385333</v>
+        <v>1274.60643986667</v>
       </c>
       <c r="V37" s="12" t="n">
         <f aca="false">(G37+H37)*Premissas!$B$21</f>
@@ -7321,7 +7321,7 @@
       </c>
       <c r="X37" s="12" t="n">
         <f aca="false">X36-Y36+C37*(1+Premissas!$B$17)</f>
-        <v>62.6065</v>
+        <v>56.915</v>
       </c>
       <c r="Y37" s="12" t="n">
         <f aca="false">IF(OR(X37&gt;=Premissas!$B$13,B37=DATE(YEAR(B37),MONTH(B37)+1,0)),X37,0)</f>
@@ -7329,7 +7329,7 @@
       </c>
       <c r="Z37" s="12" t="n">
         <f aca="false">Z36-AA36+C37/Premissas!$B$18*Premissas!$B$20</f>
-        <v>9.9</v>
+        <v>9</v>
       </c>
       <c r="AA37" s="12" t="n">
         <f aca="false">IF(OR(Z37&gt;=Premissas!$B$14,B37=DATE(YEAR(B37),MONTH(B37)+1,0)),Z37,0)</f>
@@ -7414,7 +7414,7 @@
       </c>
       <c r="S38" s="12" t="n">
         <f aca="false">S37+R38</f>
-        <v>2278.55808385333</v>
+        <v>2071.41643986667</v>
       </c>
       <c r="T38" s="15" t="n">
         <f aca="false">IF(AND($A38&gt;$B$100,S38&gt;=0),1,0)</f>
@@ -7422,7 +7422,7 @@
       </c>
       <c r="U38" s="12" t="n">
         <f aca="false">S38-SUM($E$5:E38)-(1+Premissas!$B$17)*SUM($C$5:C38)</f>
-        <v>1402.06708385333</v>
+        <v>1274.60643986667</v>
       </c>
       <c r="V38" s="12" t="n">
         <f aca="false">(G38+H38)*Premissas!$B$21</f>
@@ -7434,7 +7434,7 @@
       </c>
       <c r="X38" s="12" t="n">
         <f aca="false">X37-Y37+C38*(1+Premissas!$B$17)</f>
-        <v>62.6065</v>
+        <v>56.915</v>
       </c>
       <c r="Y38" s="12" t="n">
         <f aca="false">IF(OR(X38&gt;=Premissas!$B$13,B38=DATE(YEAR(B38),MONTH(B38)+1,0)),X38,0)</f>
@@ -7442,7 +7442,7 @@
       </c>
       <c r="Z38" s="12" t="n">
         <f aca="false">Z37-AA37+C38/Premissas!$B$18*Premissas!$B$20</f>
-        <v>9.9</v>
+        <v>9</v>
       </c>
       <c r="AA38" s="12" t="n">
         <f aca="false">IF(OR(Z38&gt;=Premissas!$B$14,B38=DATE(YEAR(B38),MONTH(B38)+1,0)),Z38,0)</f>
@@ -7527,7 +7527,7 @@
       </c>
       <c r="S39" s="12" t="n">
         <f aca="false">S38+R39</f>
-        <v>2278.55808385333</v>
+        <v>2071.41643986667</v>
       </c>
       <c r="T39" s="15" t="n">
         <f aca="false">IF(AND($A39&gt;$B$100,S39&gt;=0),1,0)</f>
@@ -7535,7 +7535,7 @@
       </c>
       <c r="U39" s="12" t="n">
         <f aca="false">S39-SUM($E$5:E39)-(1+Premissas!$B$17)*SUM($C$5:C39)</f>
-        <v>1402.06708385333</v>
+        <v>1274.60643986667</v>
       </c>
       <c r="V39" s="12" t="n">
         <f aca="false">(G39+H39)*Premissas!$B$21</f>
@@ -7547,7 +7547,7 @@
       </c>
       <c r="X39" s="12" t="n">
         <f aca="false">X38-Y38+C39*(1+Premissas!$B$17)</f>
-        <v>62.6065</v>
+        <v>56.915</v>
       </c>
       <c r="Y39" s="12" t="n">
         <f aca="false">IF(OR(X39&gt;=Premissas!$B$13,B39=DATE(YEAR(B39),MONTH(B39)+1,0)),X39,0)</f>
@@ -7555,7 +7555,7 @@
       </c>
       <c r="Z39" s="12" t="n">
         <f aca="false">Z38-AA38+C39/Premissas!$B$18*Premissas!$B$20</f>
-        <v>9.9</v>
+        <v>9</v>
       </c>
       <c r="AA39" s="12" t="n">
         <f aca="false">IF(OR(Z39&gt;=Premissas!$B$14,B39=DATE(YEAR(B39),MONTH(B39)+1,0)),Z39,0)</f>
@@ -7584,11 +7584,11 @@
       </c>
       <c r="E40" s="12" t="n">
         <f aca="false">-SUMIF($D$5:$D$94,A40,$Y$5:$Y$94)</f>
-        <v>-813.8845</v>
+        <v>-739.895</v>
       </c>
       <c r="F40" s="12" t="n">
         <f aca="false">-SUMIF($W$5:$W$94,A40,$V$5:$V$94)-SUMIF($AB$5:$AB$94,A40,$AA$5:$AA$94)</f>
-        <v>-129.726666666667</v>
+        <v>-117.933333333333</v>
       </c>
       <c r="G40" s="29" t="n">
         <f aca="false">C40/Premissas!$B$18*Premissas!$B$19*Premissas!$B$23</f>
@@ -7636,11 +7636,11 @@
       </c>
       <c r="R40" s="12" t="n">
         <f aca="false">E40+F40+SUM(I40:Q40)</f>
-        <v>-1001.10116666667</v>
+        <v>-915.318333333334</v>
       </c>
       <c r="S40" s="12" t="n">
         <f aca="false">S39+R40</f>
-        <v>1277.45691718667</v>
+        <v>1156.09810653333</v>
       </c>
       <c r="T40" s="15" t="n">
         <f aca="false">IF(AND($A40&gt;$B$100,S40&gt;=0),1,0)</f>
@@ -7648,7 +7648,7 @@
       </c>
       <c r="U40" s="12" t="n">
         <f aca="false">S40-SUM($E$5:E40)-(1+Premissas!$B$17)*SUM($C$5:C40)</f>
-        <v>1214.85041718667</v>
+        <v>1099.18310653333</v>
       </c>
       <c r="V40" s="12" t="n">
         <f aca="false">(G40+H40)*Premissas!$B$21</f>
@@ -7660,7 +7660,7 @@
       </c>
       <c r="X40" s="12" t="n">
         <f aca="false">X39-Y39+C40*(1+Premissas!$B$17)</f>
-        <v>62.6065</v>
+        <v>56.915</v>
       </c>
       <c r="Y40" s="12" t="n">
         <f aca="false">IF(OR(X40&gt;=Premissas!$B$13,B40=DATE(YEAR(B40),MONTH(B40)+1,0)),X40,0)</f>
@@ -7668,7 +7668,7 @@
       </c>
       <c r="Z40" s="12" t="n">
         <f aca="false">Z39-AA39+C40/Premissas!$B$18*Premissas!$B$20</f>
-        <v>9.9</v>
+        <v>9</v>
       </c>
       <c r="AA40" s="12" t="n">
         <f aca="false">IF(OR(Z40&gt;=Premissas!$B$14,B40=DATE(YEAR(B40),MONTH(B40)+1,0)),Z40,0)</f>
@@ -7753,7 +7753,7 @@
       </c>
       <c r="S41" s="12" t="n">
         <f aca="false">S40+R41</f>
-        <v>1277.45691718667</v>
+        <v>1156.09810653333</v>
       </c>
       <c r="T41" s="15" t="n">
         <f aca="false">IF(AND($A41&gt;$B$100,S41&gt;=0),1,0)</f>
@@ -7761,7 +7761,7 @@
       </c>
       <c r="U41" s="12" t="n">
         <f aca="false">S41-SUM($E$5:E41)-(1+Premissas!$B$17)*SUM($C$5:C41)</f>
-        <v>1214.85041718667</v>
+        <v>1099.18310653333</v>
       </c>
       <c r="V41" s="12" t="n">
         <f aca="false">(G41+H41)*Premissas!$B$21</f>
@@ -7773,7 +7773,7 @@
       </c>
       <c r="X41" s="12" t="n">
         <f aca="false">X40-Y40+C41*(1+Premissas!$B$17)</f>
-        <v>62.6065</v>
+        <v>56.915</v>
       </c>
       <c r="Y41" s="12" t="n">
         <f aca="false">IF(OR(X41&gt;=Premissas!$B$13,B41=DATE(YEAR(B41),MONTH(B41)+1,0)),X41,0)</f>
@@ -7781,7 +7781,7 @@
       </c>
       <c r="Z41" s="12" t="n">
         <f aca="false">Z40-AA40+C41/Premissas!$B$18*Premissas!$B$20</f>
-        <v>9.9</v>
+        <v>9</v>
       </c>
       <c r="AA41" s="12" t="n">
         <f aca="false">IF(OR(Z41&gt;=Premissas!$B$14,B41=DATE(YEAR(B41),MONTH(B41)+1,0)),Z41,0)</f>
@@ -7866,7 +7866,7 @@
       </c>
       <c r="S42" s="12" t="n">
         <f aca="false">S41+R42</f>
-        <v>1277.45691718667</v>
+        <v>1156.09810653333</v>
       </c>
       <c r="T42" s="15" t="n">
         <f aca="false">IF(AND($A42&gt;$B$100,S42&gt;=0),1,0)</f>
@@ -7874,7 +7874,7 @@
       </c>
       <c r="U42" s="12" t="n">
         <f aca="false">S42-SUM($E$5:E42)-(1+Premissas!$B$17)*SUM($C$5:C42)</f>
-        <v>1214.85041718667</v>
+        <v>1099.18310653333</v>
       </c>
       <c r="V42" s="12" t="n">
         <f aca="false">(G42+H42)*Premissas!$B$21</f>
@@ -7886,7 +7886,7 @@
       </c>
       <c r="X42" s="12" t="n">
         <f aca="false">X41-Y41+C42*(1+Premissas!$B$17)</f>
-        <v>62.6065</v>
+        <v>56.915</v>
       </c>
       <c r="Y42" s="12" t="n">
         <f aca="false">IF(OR(X42&gt;=Premissas!$B$13,B42=DATE(YEAR(B42),MONTH(B42)+1,0)),X42,0)</f>
@@ -7894,7 +7894,7 @@
       </c>
       <c r="Z42" s="12" t="n">
         <f aca="false">Z41-AA41+C42/Premissas!$B$18*Premissas!$B$20</f>
-        <v>9.9</v>
+        <v>9</v>
       </c>
       <c r="AA42" s="12" t="n">
         <f aca="false">IF(OR(Z42&gt;=Premissas!$B$14,B42=DATE(YEAR(B42),MONTH(B42)+1,0)),Z42,0)</f>
@@ -7979,7 +7979,7 @@
       </c>
       <c r="S43" s="12" t="n">
         <f aca="false">S42+R43</f>
-        <v>1277.45691718667</v>
+        <v>1156.09810653333</v>
       </c>
       <c r="T43" s="15" t="n">
         <f aca="false">IF(AND($A43&gt;$B$100,S43&gt;=0),1,0)</f>
@@ -7987,7 +7987,7 @@
       </c>
       <c r="U43" s="12" t="n">
         <f aca="false">S43-SUM($E$5:E43)-(1+Premissas!$B$17)*SUM($C$5:C43)</f>
-        <v>1214.85041718667</v>
+        <v>1099.18310653333</v>
       </c>
       <c r="V43" s="12" t="n">
         <f aca="false">(G43+H43)*Premissas!$B$21</f>
@@ -7999,19 +7999,19 @@
       </c>
       <c r="X43" s="12" t="n">
         <f aca="false">X42-Y42+C43*(1+Premissas!$B$17)</f>
-        <v>62.6065</v>
+        <v>56.915</v>
       </c>
       <c r="Y43" s="12" t="n">
         <f aca="false">IF(OR(X43&gt;=Premissas!$B$13,B43=DATE(YEAR(B43),MONTH(B43)+1,0)),X43,0)</f>
-        <v>62.6065</v>
+        <v>56.915</v>
       </c>
       <c r="Z43" s="12" t="n">
         <f aca="false">Z42-AA42+C43/Premissas!$B$18*Premissas!$B$20</f>
-        <v>9.9</v>
+        <v>9</v>
       </c>
       <c r="AA43" s="12" t="n">
         <f aca="false">IF(OR(Z43&gt;=Premissas!$B$14,B43=DATE(YEAR(B43),MONTH(B43)+1,0)),Z43,0)</f>
-        <v>9.9</v>
+        <v>9</v>
       </c>
       <c r="AB43" s="15" t="n">
         <f aca="false">IF(AA43&gt;0,IF(DAY(B43)&lt;=Premissas!$B$12,DATE(YEAR(B43),MONTH(B43),Premissas!$B$16),DATE(YEAR(B43),MONTH(B43)+1,Premissas!$B$16))-Premissas!$B$11+1-Premissas!$B$15,0)</f>
@@ -8092,7 +8092,7 @@
       </c>
       <c r="S44" s="12" t="n">
         <f aca="false">S43+R44</f>
-        <v>1277.45691718667</v>
+        <v>1156.09810653333</v>
       </c>
       <c r="T44" s="15" t="n">
         <f aca="false">IF(AND($A44&gt;$B$100,S44&gt;=0),1,0)</f>
@@ -8100,7 +8100,7 @@
       </c>
       <c r="U44" s="12" t="n">
         <f aca="false">S44-SUM($E$5:E44)-(1+Premissas!$B$17)*SUM($C$5:C44)</f>
-        <v>1214.85041718667</v>
+        <v>1099.18310653333</v>
       </c>
       <c r="V44" s="12" t="n">
         <f aca="false">(G44+H44)*Premissas!$B$21</f>
@@ -8205,7 +8205,7 @@
       </c>
       <c r="S45" s="12" t="n">
         <f aca="false">S44+R45</f>
-        <v>1277.45691718667</v>
+        <v>1156.09810653333</v>
       </c>
       <c r="T45" s="15" t="n">
         <f aca="false">IF(AND($A45&gt;$B$100,S45&gt;=0),1,0)</f>
@@ -8213,7 +8213,7 @@
       </c>
       <c r="U45" s="12" t="n">
         <f aca="false">S45-SUM($E$5:E45)-(1+Premissas!$B$17)*SUM($C$5:C45)</f>
-        <v>1214.85041718667</v>
+        <v>1099.18310653333</v>
       </c>
       <c r="V45" s="12" t="n">
         <f aca="false">(G45+H45)*Premissas!$B$21</f>
@@ -8318,7 +8318,7 @@
       </c>
       <c r="S46" s="12" t="n">
         <f aca="false">S45+R46</f>
-        <v>1277.45691718667</v>
+        <v>1156.09810653333</v>
       </c>
       <c r="T46" s="15" t="n">
         <f aca="false">IF(AND($A46&gt;$B$100,S46&gt;=0),1,0)</f>
@@ -8326,7 +8326,7 @@
       </c>
       <c r="U46" s="12" t="n">
         <f aca="false">S46-SUM($E$5:E46)-(1+Premissas!$B$17)*SUM($C$5:C46)</f>
-        <v>1214.85041718667</v>
+        <v>1099.18310653333</v>
       </c>
       <c r="V46" s="12" t="n">
         <f aca="false">(G46+H46)*Premissas!$B$21</f>
@@ -8431,7 +8431,7 @@
       </c>
       <c r="S47" s="12" t="n">
         <f aca="false">S46+R47</f>
-        <v>1277.45691718667</v>
+        <v>1156.09810653333</v>
       </c>
       <c r="T47" s="15" t="n">
         <f aca="false">IF(AND($A47&gt;$B$100,S47&gt;=0),1,0)</f>
@@ -8439,7 +8439,7 @@
       </c>
       <c r="U47" s="12" t="n">
         <f aca="false">S47-SUM($E$5:E47)-(1+Premissas!$B$17)*SUM($C$5:C47)</f>
-        <v>1214.85041718667</v>
+        <v>1099.18310653333</v>
       </c>
       <c r="V47" s="12" t="n">
         <f aca="false">(G47+H47)*Premissas!$B$21</f>
@@ -8544,7 +8544,7 @@
       </c>
       <c r="S48" s="12" t="n">
         <f aca="false">S47+R48</f>
-        <v>1277.45691718667</v>
+        <v>1156.09810653333</v>
       </c>
       <c r="T48" s="15" t="n">
         <f aca="false">IF(AND($A48&gt;$B$100,S48&gt;=0),1,0)</f>
@@ -8552,7 +8552,7 @@
       </c>
       <c r="U48" s="12" t="n">
         <f aca="false">S48-SUM($E$5:E48)-(1+Premissas!$B$17)*SUM($C$5:C48)</f>
-        <v>1214.85041718667</v>
+        <v>1099.18310653333</v>
       </c>
       <c r="V48" s="12" t="n">
         <f aca="false">(G48+H48)*Premissas!$B$21</f>
@@ -8657,7 +8657,7 @@
       </c>
       <c r="S49" s="12" t="n">
         <f aca="false">S48+R49</f>
-        <v>1277.45691718667</v>
+        <v>1156.09810653333</v>
       </c>
       <c r="T49" s="15" t="n">
         <f aca="false">IF(AND($A49&gt;$B$100,S49&gt;=0),1,0)</f>
@@ -8665,7 +8665,7 @@
       </c>
       <c r="U49" s="12" t="n">
         <f aca="false">S49-SUM($E$5:E49)-(1+Premissas!$B$17)*SUM($C$5:C49)</f>
-        <v>1214.85041718667</v>
+        <v>1099.18310653333</v>
       </c>
       <c r="V49" s="12" t="n">
         <f aca="false">(G49+H49)*Premissas!$B$21</f>
@@ -8770,7 +8770,7 @@
       </c>
       <c r="S50" s="12" t="n">
         <f aca="false">S49+R50</f>
-        <v>1277.45691718667</v>
+        <v>1156.09810653333</v>
       </c>
       <c r="T50" s="15" t="n">
         <f aca="false">IF(AND($A50&gt;$B$100,S50&gt;=0),1,0)</f>
@@ -8778,7 +8778,7 @@
       </c>
       <c r="U50" s="12" t="n">
         <f aca="false">S50-SUM($E$5:E50)-(1+Premissas!$B$17)*SUM($C$5:C50)</f>
-        <v>1214.85041718667</v>
+        <v>1099.18310653333</v>
       </c>
       <c r="V50" s="12" t="n">
         <f aca="false">(G50+H50)*Premissas!$B$21</f>
@@ -8883,7 +8883,7 @@
       </c>
       <c r="S51" s="12" t="n">
         <f aca="false">S50+R51</f>
-        <v>1277.45691718667</v>
+        <v>1156.09810653333</v>
       </c>
       <c r="T51" s="15" t="n">
         <f aca="false">IF(AND($A51&gt;$B$100,S51&gt;=0),1,0)</f>
@@ -8891,7 +8891,7 @@
       </c>
       <c r="U51" s="12" t="n">
         <f aca="false">S51-SUM($E$5:E51)-(1+Premissas!$B$17)*SUM($C$5:C51)</f>
-        <v>1214.85041718667</v>
+        <v>1099.18310653333</v>
       </c>
       <c r="V51" s="12" t="n">
         <f aca="false">(G51+H51)*Premissas!$B$21</f>
@@ -8996,7 +8996,7 @@
       </c>
       <c r="S52" s="12" t="n">
         <f aca="false">S51+R52</f>
-        <v>1277.45691718667</v>
+        <v>1156.09810653333</v>
       </c>
       <c r="T52" s="15" t="n">
         <f aca="false">IF(AND($A52&gt;$B$100,S52&gt;=0),1,0)</f>
@@ -9004,7 +9004,7 @@
       </c>
       <c r="U52" s="12" t="n">
         <f aca="false">S52-SUM($E$5:E52)-(1+Premissas!$B$17)*SUM($C$5:C52)</f>
-        <v>1214.85041718667</v>
+        <v>1099.18310653333</v>
       </c>
       <c r="V52" s="12" t="n">
         <f aca="false">(G52+H52)*Premissas!$B$21</f>
@@ -9109,7 +9109,7 @@
       </c>
       <c r="S53" s="12" t="n">
         <f aca="false">S52+R53</f>
-        <v>1277.45691718667</v>
+        <v>1156.09810653333</v>
       </c>
       <c r="T53" s="15" t="n">
         <f aca="false">IF(AND($A53&gt;$B$100,S53&gt;=0),1,0)</f>
@@ -9117,7 +9117,7 @@
       </c>
       <c r="U53" s="12" t="n">
         <f aca="false">S53-SUM($E$5:E53)-(1+Premissas!$B$17)*SUM($C$5:C53)</f>
-        <v>1214.85041718667</v>
+        <v>1099.18310653333</v>
       </c>
       <c r="V53" s="12" t="n">
         <f aca="false">(G53+H53)*Premissas!$B$21</f>
@@ -9222,7 +9222,7 @@
       </c>
       <c r="S54" s="12" t="n">
         <f aca="false">S53+R54</f>
-        <v>1277.45691718667</v>
+        <v>1156.09810653333</v>
       </c>
       <c r="T54" s="15" t="n">
         <f aca="false">IF(AND($A54&gt;$B$100,S54&gt;=0),1,0)</f>
@@ -9230,7 +9230,7 @@
       </c>
       <c r="U54" s="12" t="n">
         <f aca="false">S54-SUM($E$5:E54)-(1+Premissas!$B$17)*SUM($C$5:C54)</f>
-        <v>1214.85041718667</v>
+        <v>1099.18310653333</v>
       </c>
       <c r="V54" s="12" t="n">
         <f aca="false">(G54+H54)*Premissas!$B$21</f>
@@ -9335,7 +9335,7 @@
       </c>
       <c r="S55" s="12" t="n">
         <f aca="false">S54+R55</f>
-        <v>1277.45691718667</v>
+        <v>1156.09810653333</v>
       </c>
       <c r="T55" s="15" t="n">
         <f aca="false">IF(AND($A55&gt;$B$100,S55&gt;=0),1,0)</f>
@@ -9343,7 +9343,7 @@
       </c>
       <c r="U55" s="12" t="n">
         <f aca="false">S55-SUM($E$5:E55)-(1+Premissas!$B$17)*SUM($C$5:C55)</f>
-        <v>1214.85041718667</v>
+        <v>1099.18310653333</v>
       </c>
       <c r="V55" s="12" t="n">
         <f aca="false">(G55+H55)*Premissas!$B$21</f>
@@ -9448,7 +9448,7 @@
       </c>
       <c r="S56" s="12" t="n">
         <f aca="false">S55+R56</f>
-        <v>1277.45691718667</v>
+        <v>1156.09810653333</v>
       </c>
       <c r="T56" s="15" t="n">
         <f aca="false">IF(AND($A56&gt;$B$100,S56&gt;=0),1,0)</f>
@@ -9456,7 +9456,7 @@
       </c>
       <c r="U56" s="12" t="n">
         <f aca="false">S56-SUM($E$5:E56)-(1+Premissas!$B$17)*SUM($C$5:C56)</f>
-        <v>1214.85041718667</v>
+        <v>1099.18310653333</v>
       </c>
       <c r="V56" s="12" t="n">
         <f aca="false">(G56+H56)*Premissas!$B$21</f>
@@ -9561,7 +9561,7 @@
       </c>
       <c r="S57" s="12" t="n">
         <f aca="false">S56+R57</f>
-        <v>1277.45691718667</v>
+        <v>1156.09810653333</v>
       </c>
       <c r="T57" s="15" t="n">
         <f aca="false">IF(AND($A57&gt;$B$100,S57&gt;=0),1,0)</f>
@@ -9569,7 +9569,7 @@
       </c>
       <c r="U57" s="12" t="n">
         <f aca="false">S57-SUM($E$5:E57)-(1+Premissas!$B$17)*SUM($C$5:C57)</f>
-        <v>1214.85041718667</v>
+        <v>1099.18310653333</v>
       </c>
       <c r="V57" s="12" t="n">
         <f aca="false">(G57+H57)*Premissas!$B$21</f>
@@ -9674,7 +9674,7 @@
       </c>
       <c r="S58" s="12" t="n">
         <f aca="false">S57+R58</f>
-        <v>1277.45691718667</v>
+        <v>1156.09810653333</v>
       </c>
       <c r="T58" s="15" t="n">
         <f aca="false">IF(AND($A58&gt;$B$100,S58&gt;=0),1,0)</f>
@@ -9682,7 +9682,7 @@
       </c>
       <c r="U58" s="12" t="n">
         <f aca="false">S58-SUM($E$5:E58)-(1+Premissas!$B$17)*SUM($C$5:C58)</f>
-        <v>1214.85041718667</v>
+        <v>1099.18310653333</v>
       </c>
       <c r="V58" s="12" t="n">
         <f aca="false">(G58+H58)*Premissas!$B$21</f>
@@ -9787,7 +9787,7 @@
       </c>
       <c r="S59" s="12" t="n">
         <f aca="false">S58+R59</f>
-        <v>1277.45691718667</v>
+        <v>1156.09810653333</v>
       </c>
       <c r="T59" s="15" t="n">
         <f aca="false">IF(AND($A59&gt;$B$100,S59&gt;=0),1,0)</f>
@@ -9795,7 +9795,7 @@
       </c>
       <c r="U59" s="12" t="n">
         <f aca="false">S59-SUM($E$5:E59)-(1+Premissas!$B$17)*SUM($C$5:C59)</f>
-        <v>1214.85041718667</v>
+        <v>1099.18310653333</v>
       </c>
       <c r="V59" s="12" t="n">
         <f aca="false">(G59+H59)*Premissas!$B$21</f>
@@ -9900,7 +9900,7 @@
       </c>
       <c r="S60" s="12" t="n">
         <f aca="false">S59+R60</f>
-        <v>1277.45691718667</v>
+        <v>1156.09810653333</v>
       </c>
       <c r="T60" s="15" t="n">
         <f aca="false">IF(AND($A60&gt;$B$100,S60&gt;=0),1,0)</f>
@@ -9908,7 +9908,7 @@
       </c>
       <c r="U60" s="12" t="n">
         <f aca="false">S60-SUM($E$5:E60)-(1+Premissas!$B$17)*SUM($C$5:C60)</f>
-        <v>1214.85041718667</v>
+        <v>1099.18310653333</v>
       </c>
       <c r="V60" s="12" t="n">
         <f aca="false">(G60+H60)*Premissas!$B$21</f>
@@ -10013,7 +10013,7 @@
       </c>
       <c r="S61" s="12" t="n">
         <f aca="false">S60+R61</f>
-        <v>1277.45691718667</v>
+        <v>1156.09810653333</v>
       </c>
       <c r="T61" s="15" t="n">
         <f aca="false">IF(AND($A61&gt;$B$100,S61&gt;=0),1,0)</f>
@@ -10021,7 +10021,7 @@
       </c>
       <c r="U61" s="12" t="n">
         <f aca="false">S61-SUM($E$5:E61)-(1+Premissas!$B$17)*SUM($C$5:C61)</f>
-        <v>1214.85041718667</v>
+        <v>1099.18310653333</v>
       </c>
       <c r="V61" s="12" t="n">
         <f aca="false">(G61+H61)*Premissas!$B$21</f>
@@ -10126,7 +10126,7 @@
       </c>
       <c r="S62" s="12" t="n">
         <f aca="false">S61+R62</f>
-        <v>1277.45691718667</v>
+        <v>1156.09810653333</v>
       </c>
       <c r="T62" s="15" t="n">
         <f aca="false">IF(AND($A62&gt;$B$100,S62&gt;=0),1,0)</f>
@@ -10134,7 +10134,7 @@
       </c>
       <c r="U62" s="12" t="n">
         <f aca="false">S62-SUM($E$5:E62)-(1+Premissas!$B$17)*SUM($C$5:C62)</f>
-        <v>1214.85041718667</v>
+        <v>1099.18310653333</v>
       </c>
       <c r="V62" s="12" t="n">
         <f aca="false">(G62+H62)*Premissas!$B$21</f>
@@ -10239,7 +10239,7 @@
       </c>
       <c r="S63" s="12" t="n">
         <f aca="false">S62+R63</f>
-        <v>1277.45691718667</v>
+        <v>1156.09810653333</v>
       </c>
       <c r="T63" s="15" t="n">
         <f aca="false">IF(AND($A63&gt;$B$100,S63&gt;=0),1,0)</f>
@@ -10247,7 +10247,7 @@
       </c>
       <c r="U63" s="12" t="n">
         <f aca="false">S63-SUM($E$5:E63)-(1+Premissas!$B$17)*SUM($C$5:C63)</f>
-        <v>1214.85041718667</v>
+        <v>1099.18310653333</v>
       </c>
       <c r="V63" s="12" t="n">
         <f aca="false">(G63+H63)*Premissas!$B$21</f>
@@ -10352,7 +10352,7 @@
       </c>
       <c r="S64" s="12" t="n">
         <f aca="false">S63+R64</f>
-        <v>1277.45691718667</v>
+        <v>1156.09810653333</v>
       </c>
       <c r="T64" s="15" t="n">
         <f aca="false">IF(AND($A64&gt;$B$100,S64&gt;=0),1,0)</f>
@@ -10360,7 +10360,7 @@
       </c>
       <c r="U64" s="12" t="n">
         <f aca="false">S64-SUM($E$5:E64)-(1+Premissas!$B$17)*SUM($C$5:C64)</f>
-        <v>1214.85041718667</v>
+        <v>1099.18310653333</v>
       </c>
       <c r="V64" s="12" t="n">
         <f aca="false">(G64+H64)*Premissas!$B$21</f>
@@ -10465,7 +10465,7 @@
       </c>
       <c r="S65" s="12" t="n">
         <f aca="false">S64+R65</f>
-        <v>1277.45691718667</v>
+        <v>1156.09810653333</v>
       </c>
       <c r="T65" s="15" t="n">
         <f aca="false">IF(AND($A65&gt;$B$100,S65&gt;=0),1,0)</f>
@@ -10473,7 +10473,7 @@
       </c>
       <c r="U65" s="12" t="n">
         <f aca="false">S65-SUM($E$5:E65)-(1+Premissas!$B$17)*SUM($C$5:C65)</f>
-        <v>1214.85041718667</v>
+        <v>1099.18310653333</v>
       </c>
       <c r="V65" s="12" t="n">
         <f aca="false">(G65+H65)*Premissas!$B$21</f>
@@ -10578,7 +10578,7 @@
       </c>
       <c r="S66" s="12" t="n">
         <f aca="false">S65+R66</f>
-        <v>1277.45691718667</v>
+        <v>1156.09810653333</v>
       </c>
       <c r="T66" s="15" t="n">
         <f aca="false">IF(AND($A66&gt;$B$100,S66&gt;=0),1,0)</f>
@@ -10586,7 +10586,7 @@
       </c>
       <c r="U66" s="12" t="n">
         <f aca="false">S66-SUM($E$5:E66)-(1+Premissas!$B$17)*SUM($C$5:C66)</f>
-        <v>1214.85041718667</v>
+        <v>1099.18310653333</v>
       </c>
       <c r="V66" s="12" t="n">
         <f aca="false">(G66+H66)*Premissas!$B$21</f>
@@ -10691,7 +10691,7 @@
       </c>
       <c r="S67" s="12" t="n">
         <f aca="false">S66+R67</f>
-        <v>1277.45691718667</v>
+        <v>1156.09810653333</v>
       </c>
       <c r="T67" s="15" t="n">
         <f aca="false">IF(AND($A67&gt;$B$100,S67&gt;=0),1,0)</f>
@@ -10699,7 +10699,7 @@
       </c>
       <c r="U67" s="12" t="n">
         <f aca="false">S67-SUM($E$5:E67)-(1+Premissas!$B$17)*SUM($C$5:C67)</f>
-        <v>1214.85041718667</v>
+        <v>1099.18310653333</v>
       </c>
       <c r="V67" s="12" t="n">
         <f aca="false">(G67+H67)*Premissas!$B$21</f>
@@ -10804,7 +10804,7 @@
       </c>
       <c r="S68" s="12" t="n">
         <f aca="false">S67+R68</f>
-        <v>1277.45691718667</v>
+        <v>1156.09810653333</v>
       </c>
       <c r="T68" s="15" t="n">
         <f aca="false">IF(AND($A68&gt;$B$100,S68&gt;=0),1,0)</f>
@@ -10812,7 +10812,7 @@
       </c>
       <c r="U68" s="12" t="n">
         <f aca="false">S68-SUM($E$5:E68)-(1+Premissas!$B$17)*SUM($C$5:C68)</f>
-        <v>1214.85041718667</v>
+        <v>1099.18310653333</v>
       </c>
       <c r="V68" s="12" t="n">
         <f aca="false">(G68+H68)*Premissas!$B$21</f>
@@ -10917,7 +10917,7 @@
       </c>
       <c r="S69" s="12" t="n">
         <f aca="false">S68+R69</f>
-        <v>1277.45691718667</v>
+        <v>1156.09810653333</v>
       </c>
       <c r="T69" s="15" t="n">
         <f aca="false">IF(AND($A69&gt;$B$100,S69&gt;=0),1,0)</f>
@@ -10925,7 +10925,7 @@
       </c>
       <c r="U69" s="12" t="n">
         <f aca="false">S69-SUM($E$5:E69)-(1+Premissas!$B$17)*SUM($C$5:C69)</f>
-        <v>1214.85041718667</v>
+        <v>1099.18310653333</v>
       </c>
       <c r="V69" s="12" t="n">
         <f aca="false">(G69+H69)*Premissas!$B$21</f>
@@ -10974,11 +10974,11 @@
       </c>
       <c r="E70" s="12" t="n">
         <f aca="false">-SUMIF($D$5:$D$94,A70,$Y$5:$Y$94)</f>
-        <v>-62.6065</v>
+        <v>-56.915</v>
       </c>
       <c r="F70" s="12" t="n">
         <f aca="false">-SUMIF($W$5:$W$94,A70,$V$5:$V$94)-SUMIF($AB$5:$AB$94,A70,$AA$5:$AA$94)</f>
-        <v>-10.9266666666667</v>
+        <v>-9.93333333333334</v>
       </c>
       <c r="G70" s="29" t="n">
         <f aca="false">C70/Premissas!$B$18*Premissas!$B$19*Premissas!$B$23</f>
@@ -11026,11 +11026,11 @@
       </c>
       <c r="R70" s="12" t="n">
         <f aca="false">E70+F70+SUM(I70:Q70)</f>
-        <v>-131.023166666667</v>
+        <v>-124.338333333333</v>
       </c>
       <c r="S70" s="12" t="n">
         <f aca="false">S69+R70</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="T70" s="15" t="n">
         <f aca="false">IF(AND($A70&gt;$B$100,S70&gt;=0),1,0)</f>
@@ -11038,7 +11038,7 @@
       </c>
       <c r="U70" s="12" t="n">
         <f aca="false">S70-SUM($E$5:E70)-(1+Premissas!$B$17)*SUM($C$5:C70)</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="V70" s="12" t="n">
         <f aca="false">(G70+H70)*Premissas!$B$21</f>
@@ -11143,7 +11143,7 @@
       </c>
       <c r="S71" s="12" t="n">
         <f aca="false">S70+R71</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="T71" s="15" t="n">
         <f aca="false">IF(AND($A71&gt;$B$100,S71&gt;=0),1,0)</f>
@@ -11151,7 +11151,7 @@
       </c>
       <c r="U71" s="12" t="n">
         <f aca="false">S71-SUM($E$5:E71)-(1+Premissas!$B$17)*SUM($C$5:C71)</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="V71" s="12" t="n">
         <f aca="false">(G71+H71)*Premissas!$B$21</f>
@@ -11256,7 +11256,7 @@
       </c>
       <c r="S72" s="12" t="n">
         <f aca="false">S71+R72</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="T72" s="15" t="n">
         <f aca="false">IF(AND($A72&gt;$B$100,S72&gt;=0),1,0)</f>
@@ -11264,7 +11264,7 @@
       </c>
       <c r="U72" s="12" t="n">
         <f aca="false">S72-SUM($E$5:E72)-(1+Premissas!$B$17)*SUM($C$5:C72)</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="V72" s="12" t="n">
         <f aca="false">(G72+H72)*Premissas!$B$21</f>
@@ -11369,7 +11369,7 @@
       </c>
       <c r="S73" s="12" t="n">
         <f aca="false">S72+R73</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="T73" s="15" t="n">
         <f aca="false">IF(AND($A73&gt;$B$100,S73&gt;=0),1,0)</f>
@@ -11377,7 +11377,7 @@
       </c>
       <c r="U73" s="12" t="n">
         <f aca="false">S73-SUM($E$5:E73)-(1+Premissas!$B$17)*SUM($C$5:C73)</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="V73" s="12" t="n">
         <f aca="false">(G73+H73)*Premissas!$B$21</f>
@@ -11482,7 +11482,7 @@
       </c>
       <c r="S74" s="12" t="n">
         <f aca="false">S73+R74</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="T74" s="15" t="n">
         <f aca="false">IF(AND($A74&gt;$B$100,S74&gt;=0),1,0)</f>
@@ -11490,7 +11490,7 @@
       </c>
       <c r="U74" s="12" t="n">
         <f aca="false">S74-SUM($E$5:E74)-(1+Premissas!$B$17)*SUM($C$5:C74)</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="V74" s="12" t="n">
         <f aca="false">(G74+H74)*Premissas!$B$21</f>
@@ -11595,7 +11595,7 @@
       </c>
       <c r="S75" s="12" t="n">
         <f aca="false">S74+R75</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="T75" s="15" t="n">
         <f aca="false">IF(AND($A75&gt;$B$100,S75&gt;=0),1,0)</f>
@@ -11603,7 +11603,7 @@
       </c>
       <c r="U75" s="12" t="n">
         <f aca="false">S75-SUM($E$5:E75)-(1+Premissas!$B$17)*SUM($C$5:C75)</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="V75" s="12" t="n">
         <f aca="false">(G75+H75)*Premissas!$B$21</f>
@@ -11708,7 +11708,7 @@
       </c>
       <c r="S76" s="12" t="n">
         <f aca="false">S75+R76</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="T76" s="15" t="n">
         <f aca="false">IF(AND($A76&gt;$B$100,S76&gt;=0),1,0)</f>
@@ -11716,7 +11716,7 @@
       </c>
       <c r="U76" s="12" t="n">
         <f aca="false">S76-SUM($E$5:E76)-(1+Premissas!$B$17)*SUM($C$5:C76)</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="V76" s="12" t="n">
         <f aca="false">(G76+H76)*Premissas!$B$21</f>
@@ -11821,7 +11821,7 @@
       </c>
       <c r="S77" s="12" t="n">
         <f aca="false">S76+R77</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="T77" s="15" t="n">
         <f aca="false">IF(AND($A77&gt;$B$100,S77&gt;=0),1,0)</f>
@@ -11829,7 +11829,7 @@
       </c>
       <c r="U77" s="12" t="n">
         <f aca="false">S77-SUM($E$5:E77)-(1+Premissas!$B$17)*SUM($C$5:C77)</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="V77" s="12" t="n">
         <f aca="false">(G77+H77)*Premissas!$B$21</f>
@@ -11934,7 +11934,7 @@
       </c>
       <c r="S78" s="12" t="n">
         <f aca="false">S77+R78</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="T78" s="15" t="n">
         <f aca="false">IF(AND($A78&gt;$B$100,S78&gt;=0),1,0)</f>
@@ -11942,7 +11942,7 @@
       </c>
       <c r="U78" s="12" t="n">
         <f aca="false">S78-SUM($E$5:E78)-(1+Premissas!$B$17)*SUM($C$5:C78)</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="V78" s="12" t="n">
         <f aca="false">(G78+H78)*Premissas!$B$21</f>
@@ -12047,7 +12047,7 @@
       </c>
       <c r="S79" s="12" t="n">
         <f aca="false">S78+R79</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="T79" s="15" t="n">
         <f aca="false">IF(AND($A79&gt;$B$100,S79&gt;=0),1,0)</f>
@@ -12055,7 +12055,7 @@
       </c>
       <c r="U79" s="12" t="n">
         <f aca="false">S79-SUM($E$5:E79)-(1+Premissas!$B$17)*SUM($C$5:C79)</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="V79" s="12" t="n">
         <f aca="false">(G79+H79)*Premissas!$B$21</f>
@@ -12160,7 +12160,7 @@
       </c>
       <c r="S80" s="12" t="n">
         <f aca="false">S79+R80</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="T80" s="15" t="n">
         <f aca="false">IF(AND($A80&gt;$B$100,S80&gt;=0),1,0)</f>
@@ -12168,7 +12168,7 @@
       </c>
       <c r="U80" s="12" t="n">
         <f aca="false">S80-SUM($E$5:E80)-(1+Premissas!$B$17)*SUM($C$5:C80)</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="V80" s="12" t="n">
         <f aca="false">(G80+H80)*Premissas!$B$21</f>
@@ -12273,7 +12273,7 @@
       </c>
       <c r="S81" s="12" t="n">
         <f aca="false">S80+R81</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="T81" s="15" t="n">
         <f aca="false">IF(AND($A81&gt;$B$100,S81&gt;=0),1,0)</f>
@@ -12281,7 +12281,7 @@
       </c>
       <c r="U81" s="12" t="n">
         <f aca="false">S81-SUM($E$5:E81)-(1+Premissas!$B$17)*SUM($C$5:C81)</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="V81" s="12" t="n">
         <f aca="false">(G81+H81)*Premissas!$B$21</f>
@@ -12386,7 +12386,7 @@
       </c>
       <c r="S82" s="12" t="n">
         <f aca="false">S81+R82</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="T82" s="15" t="n">
         <f aca="false">IF(AND($A82&gt;$B$100,S82&gt;=0),1,0)</f>
@@ -12394,7 +12394,7 @@
       </c>
       <c r="U82" s="12" t="n">
         <f aca="false">S82-SUM($E$5:E82)-(1+Premissas!$B$17)*SUM($C$5:C82)</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="V82" s="12" t="n">
         <f aca="false">(G82+H82)*Premissas!$B$21</f>
@@ -12499,7 +12499,7 @@
       </c>
       <c r="S83" s="12" t="n">
         <f aca="false">S82+R83</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="T83" s="15" t="n">
         <f aca="false">IF(AND($A83&gt;$B$100,S83&gt;=0),1,0)</f>
@@ -12507,7 +12507,7 @@
       </c>
       <c r="U83" s="12" t="n">
         <f aca="false">S83-SUM($E$5:E83)-(1+Premissas!$B$17)*SUM($C$5:C83)</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="V83" s="12" t="n">
         <f aca="false">(G83+H83)*Premissas!$B$21</f>
@@ -12612,7 +12612,7 @@
       </c>
       <c r="S84" s="12" t="n">
         <f aca="false">S83+R84</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="T84" s="15" t="n">
         <f aca="false">IF(AND($A84&gt;$B$100,S84&gt;=0),1,0)</f>
@@ -12620,7 +12620,7 @@
       </c>
       <c r="U84" s="12" t="n">
         <f aca="false">S84-SUM($E$5:E84)-(1+Premissas!$B$17)*SUM($C$5:C84)</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="V84" s="12" t="n">
         <f aca="false">(G84+H84)*Premissas!$B$21</f>
@@ -12725,7 +12725,7 @@
       </c>
       <c r="S85" s="12" t="n">
         <f aca="false">S84+R85</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="T85" s="15" t="n">
         <f aca="false">IF(AND($A85&gt;$B$100,S85&gt;=0),1,0)</f>
@@ -12733,7 +12733,7 @@
       </c>
       <c r="U85" s="12" t="n">
         <f aca="false">S85-SUM($E$5:E85)-(1+Premissas!$B$17)*SUM($C$5:C85)</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="V85" s="12" t="n">
         <f aca="false">(G85+H85)*Premissas!$B$21</f>
@@ -12838,7 +12838,7 @@
       </c>
       <c r="S86" s="12" t="n">
         <f aca="false">S85+R86</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="T86" s="15" t="n">
         <f aca="false">IF(AND($A86&gt;$B$100,S86&gt;=0),1,0)</f>
@@ -12846,7 +12846,7 @@
       </c>
       <c r="U86" s="12" t="n">
         <f aca="false">S86-SUM($E$5:E86)-(1+Premissas!$B$17)*SUM($C$5:C86)</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="V86" s="12" t="n">
         <f aca="false">(G86+H86)*Premissas!$B$21</f>
@@ -12951,7 +12951,7 @@
       </c>
       <c r="S87" s="12" t="n">
         <f aca="false">S86+R87</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="T87" s="15" t="n">
         <f aca="false">IF(AND($A87&gt;$B$100,S87&gt;=0),1,0)</f>
@@ -12959,7 +12959,7 @@
       </c>
       <c r="U87" s="12" t="n">
         <f aca="false">S87-SUM($E$5:E87)-(1+Premissas!$B$17)*SUM($C$5:C87)</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="V87" s="12" t="n">
         <f aca="false">(G87+H87)*Premissas!$B$21</f>
@@ -13064,7 +13064,7 @@
       </c>
       <c r="S88" s="12" t="n">
         <f aca="false">S87+R88</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="T88" s="15" t="n">
         <f aca="false">IF(AND($A88&gt;$B$100,S88&gt;=0),1,0)</f>
@@ -13072,7 +13072,7 @@
       </c>
       <c r="U88" s="12" t="n">
         <f aca="false">S88-SUM($E$5:E88)-(1+Premissas!$B$17)*SUM($C$5:C88)</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="V88" s="12" t="n">
         <f aca="false">(G88+H88)*Premissas!$B$21</f>
@@ -13177,7 +13177,7 @@
       </c>
       <c r="S89" s="12" t="n">
         <f aca="false">S88+R89</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="T89" s="15" t="n">
         <f aca="false">IF(AND($A89&gt;$B$100,S89&gt;=0),1,0)</f>
@@ -13185,7 +13185,7 @@
       </c>
       <c r="U89" s="12" t="n">
         <f aca="false">S89-SUM($E$5:E89)-(1+Premissas!$B$17)*SUM($C$5:C89)</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="V89" s="12" t="n">
         <f aca="false">(G89+H89)*Premissas!$B$21</f>
@@ -13290,7 +13290,7 @@
       </c>
       <c r="S90" s="12" t="n">
         <f aca="false">S89+R90</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="T90" s="15" t="n">
         <f aca="false">IF(AND($A90&gt;$B$100,S90&gt;=0),1,0)</f>
@@ -13298,7 +13298,7 @@
       </c>
       <c r="U90" s="12" t="n">
         <f aca="false">S90-SUM($E$5:E90)-(1+Premissas!$B$17)*SUM($C$5:C90)</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="V90" s="12" t="n">
         <f aca="false">(G90+H90)*Premissas!$B$21</f>
@@ -13403,7 +13403,7 @@
       </c>
       <c r="S91" s="12" t="n">
         <f aca="false">S90+R91</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="T91" s="15" t="n">
         <f aca="false">IF(AND($A91&gt;$B$100,S91&gt;=0),1,0)</f>
@@ -13411,7 +13411,7 @@
       </c>
       <c r="U91" s="12" t="n">
         <f aca="false">S91-SUM($E$5:E91)-(1+Premissas!$B$17)*SUM($C$5:C91)</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="V91" s="12" t="n">
         <f aca="false">(G91+H91)*Premissas!$B$21</f>
@@ -13516,7 +13516,7 @@
       </c>
       <c r="S92" s="12" t="n">
         <f aca="false">S91+R92</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="T92" s="15" t="n">
         <f aca="false">IF(AND($A92&gt;$B$100,S92&gt;=0),1,0)</f>
@@ -13524,7 +13524,7 @@
       </c>
       <c r="U92" s="12" t="n">
         <f aca="false">S92-SUM($E$5:E92)-(1+Premissas!$B$17)*SUM($C$5:C92)</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="V92" s="12" t="n">
         <f aca="false">(G92+H92)*Premissas!$B$21</f>
@@ -13629,7 +13629,7 @@
       </c>
       <c r="S93" s="12" t="n">
         <f aca="false">S92+R93</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="T93" s="15" t="n">
         <f aca="false">IF(AND($A93&gt;$B$100,S93&gt;=0),1,0)</f>
@@ -13637,7 +13637,7 @@
       </c>
       <c r="U93" s="12" t="n">
         <f aca="false">S93-SUM($E$5:E93)-(1+Premissas!$B$17)*SUM($C$5:C93)</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="V93" s="12" t="n">
         <f aca="false">(G93+H93)*Premissas!$B$21</f>
@@ -13742,7 +13742,7 @@
       </c>
       <c r="S94" s="12" t="n">
         <f aca="false">S93+R94</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="T94" s="15" t="n">
         <f aca="false">IF(AND($A94&gt;$B$100,S94&gt;=0),1,0)</f>
@@ -13750,7 +13750,7 @@
       </c>
       <c r="U94" s="12" t="n">
         <f aca="false">S94-SUM($E$5:E94)-(1+Premissas!$B$17)*SUM($C$5:C94)</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
       <c r="V94" s="12" t="n">
         <f aca="false">(G94+H94)*Premissas!$B$21</f>
@@ -13787,51 +13787,51 @@
       </c>
       <c r="C95" s="14" t="n">
         <f aca="false">SUM(C5:C94)</f>
-        <v>770</v>
+        <v>700</v>
       </c>
       <c r="E95" s="14" t="n">
         <f aca="false">SUM(E5:E94)</f>
-        <v>-876.491</v>
+        <v>-796.81</v>
       </c>
       <c r="F95" s="14" t="n">
         <f aca="false">SUM(F5:F94)</f>
-        <v>-140.653333333333</v>
+        <v>-127.866666666667</v>
       </c>
       <c r="G95" s="31" t="n">
         <f aca="false">SUM(G5:G94)</f>
-        <v>35.9333333333333</v>
+        <v>32.6666666666667</v>
       </c>
       <c r="H95" s="31" t="n">
         <f aca="false">SUM(H5:H94)</f>
-        <v>15.4</v>
+        <v>14</v>
       </c>
       <c r="I95" s="14" t="n">
         <f aca="false">SUM(I5:I94)</f>
-        <v>-2391.723026</v>
+        <v>-2174.29366</v>
       </c>
       <c r="J95" s="14" t="n">
         <f aca="false">SUM(J5:J94)</f>
-        <v>345.56733442</v>
+        <v>314.1521222</v>
       </c>
       <c r="K95" s="14" t="n">
         <f aca="false">SUM(K5:K94)</f>
-        <v>-71.8666666666667</v>
+        <v>-65.3333333333333</v>
       </c>
       <c r="L95" s="14" t="n">
         <f aca="false">SUM(L5:L94)</f>
-        <v>3407.4502</v>
+        <v>3097.682</v>
       </c>
       <c r="M95" s="14" t="n">
         <f aca="false">SUM(M5:M94)</f>
-        <v>1738.9716421</v>
+        <v>1580.883311</v>
       </c>
       <c r="N95" s="14" t="n">
         <f aca="false">SUM(N5:N94)</f>
-        <v>-539</v>
+        <v>-490</v>
       </c>
       <c r="O95" s="14" t="n">
         <f aca="false">SUM(O5:O94)</f>
-        <v>-210.8414</v>
+        <v>-191.674</v>
       </c>
       <c r="P95" s="14" t="n">
         <f aca="false">SUM(P5:P94)</f>
@@ -13843,7 +13843,7 @@
       </c>
       <c r="R95" s="14" t="n">
         <f aca="false">SUM(R5:R94)</f>
-        <v>1146.43375052</v>
+        <v>1031.7597732</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13852,7 +13852,7 @@
       </c>
       <c r="B99" s="14" t="n">
         <f aca="false">MIN(S5:S94)</f>
-        <v>-827.567485873333</v>
+        <v>-752.334078066667</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13879,7 +13879,7 @@
       </c>
       <c r="B102" s="14" t="n">
         <f aca="false">MIN(U5:U94)</f>
-        <v>-1704.05848587333</v>
+        <v>-1549.14407806667</v>
       </c>
     </row>
   </sheetData>

</xml_diff>